<commit_message>
Publish fixed round dashboard data
</commit_message>
<xml_diff>
--- a/github_vercel_app/public/files/Scorito_scores_met_kansen_latest.xlsx
+++ b/github_vercel_app/public/files/Scorito_scores_met_kansen_latest.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="WK 2026 Voorspellingen" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WK 2026 Voorspellingen" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -867,47 +867,47 @@
       </c>
       <c r="J4" s="7" t="inlineStr">
         <is>
-          <t>1.41</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K4" s="7" t="inlineStr">
         <is>
-          <t>4.47</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L4" s="7" t="inlineStr">
         <is>
-          <t>8.25</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M4" s="7" t="inlineStr">
         <is>
-          <t>67.3%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N4" s="7" t="inlineStr">
         <is>
-          <t>21.2%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O4" s="7" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P4" s="7" t="inlineStr">
         <is>
-          <t>83.5%</t>
+          <t>88.1%</t>
         </is>
       </c>
       <c r="Q4" s="7" t="inlineStr">
         <is>
-          <t>9.0%</t>
+          <t>6.6%</t>
         </is>
       </c>
       <c r="R4" s="7" t="inlineStr">
         <is>
-          <t>7.4%</t>
+          <t>5.3%</t>
         </is>
       </c>
     </row>
@@ -952,52 +952,52 @@
       </c>
       <c r="I5" s="10" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>2.67</t>
+          <t>2.55</t>
         </is>
       </c>
       <c r="K5" s="7" t="inlineStr">
         <is>
-          <t>3.12</t>
+          <t>3.07</t>
         </is>
       </c>
       <c r="L5" s="7" t="inlineStr">
         <is>
-          <t>2.78</t>
+          <t>3.06</t>
         </is>
       </c>
       <c r="M5" s="7" t="inlineStr">
         <is>
-          <t>35.5%</t>
+          <t>37.5%</t>
         </is>
       </c>
       <c r="N5" s="7" t="inlineStr">
         <is>
-          <t>30.4%</t>
+          <t>31.2%</t>
         </is>
       </c>
       <c r="O5" s="7" t="inlineStr">
         <is>
-          <t>34.1%</t>
+          <t>31.3%</t>
         </is>
       </c>
       <c r="P5" s="7" t="inlineStr">
         <is>
-          <t>58.6%</t>
+          <t>62.5%</t>
         </is>
       </c>
       <c r="Q5" s="7" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>15.7%</t>
         </is>
       </c>
       <c r="R5" s="7" t="inlineStr">
         <is>
-          <t>24.5%</t>
+          <t>21.8%</t>
         </is>
       </c>
     </row>
@@ -1047,47 +1047,47 @@
       </c>
       <c r="J6" s="7" t="inlineStr">
         <is>
-          <t>1.81</t>
+          <t>1.83</t>
         </is>
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>3.57</t>
+          <t>3.48</t>
         </is>
       </c>
       <c r="L6" s="7" t="inlineStr">
         <is>
-          <t>4.57</t>
+          <t>4.78</t>
         </is>
       </c>
       <c r="M6" s="7" t="inlineStr">
         <is>
-          <t>52.5%</t>
+          <t>52.4%</t>
         </is>
       </c>
       <c r="N6" s="7" t="inlineStr">
         <is>
-          <t>26.6%</t>
+          <t>27.6%</t>
         </is>
       </c>
       <c r="O6" s="7" t="inlineStr">
         <is>
-          <t>20.8%</t>
+          <t>20.1%</t>
         </is>
       </c>
       <c r="P6" s="7" t="inlineStr">
         <is>
-          <t>74.7%</t>
+          <t>76.1%</t>
         </is>
       </c>
       <c r="Q6" s="7" t="inlineStr">
         <is>
-          <t>13.1%</t>
+          <t>12.8%</t>
         </is>
       </c>
       <c r="R6" s="7" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>11.0%</t>
         </is>
       </c>
     </row>
@@ -1137,47 +1137,47 @@
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>1.93</t>
+          <t>2.10</t>
         </is>
       </c>
       <c r="K7" s="7" t="inlineStr">
         <is>
-          <t>3.42</t>
+          <t>3.22</t>
         </is>
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
-          <t>4.13</t>
+          <t>3.87</t>
         </is>
       </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
-          <t>49.2%</t>
+          <t>45.6%</t>
         </is>
       </c>
       <c r="N7" s="7" t="inlineStr">
         <is>
-          <t>27.8%</t>
+          <t>29.7%</t>
         </is>
       </c>
       <c r="O7" s="7" t="inlineStr">
         <is>
-          <t>23.0%</t>
+          <t>24.7%</t>
         </is>
       </c>
       <c r="P7" s="7" t="inlineStr">
         <is>
-          <t>45.2%</t>
+          <t>44.5%</t>
         </is>
       </c>
       <c r="Q7" s="7" t="inlineStr">
         <is>
-          <t>18.6%</t>
+          <t>18.2%</t>
         </is>
       </c>
       <c r="R7" s="7" t="inlineStr">
         <is>
-          <t>36.2%</t>
+          <t>37.3%</t>
         </is>
       </c>
     </row>
@@ -1217,22 +1217,22 @@
       </c>
       <c r="H8" s="10" t="inlineStr">
         <is>
-          <t>0-2</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="I8" s="10" t="inlineStr">
         <is>
-          <t>0-2</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
-          <t>12.67</t>
+          <t>13.53</t>
         </is>
       </c>
       <c r="K8" s="7" t="inlineStr">
         <is>
-          <t>6.67</t>
+          <t>6.33</t>
         </is>
       </c>
       <c r="L8" s="7" t="inlineStr">
@@ -1242,32 +1242,32 @@
       </c>
       <c r="M8" s="7" t="inlineStr">
         <is>
-          <t>7.5%</t>
+          <t>7.0%</t>
         </is>
       </c>
       <c r="N8" s="7" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>15.0%</t>
         </is>
       </c>
       <c r="O8" s="7" t="inlineStr">
         <is>
-          <t>78.2%</t>
+          <t>77.9%</t>
         </is>
       </c>
       <c r="P8" s="7" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>10.6%</t>
         </is>
       </c>
       <c r="Q8" s="7" t="inlineStr">
         <is>
-          <t>12.4%</t>
+          <t>12.2%</t>
         </is>
       </c>
       <c r="R8" s="7" t="inlineStr">
         <is>
-          <t>76.5%</t>
+          <t>77.2%</t>
         </is>
       </c>
     </row>
@@ -1317,47 +1317,47 @@
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
-          <t>1.65</t>
+          <t>1.63</t>
         </is>
       </c>
       <c r="K9" s="7" t="inlineStr">
         <is>
-          <t>3.80</t>
+          <t>3.82</t>
         </is>
       </c>
       <c r="L9" s="7" t="inlineStr">
         <is>
-          <t>5.42</t>
+          <t>5.71</t>
         </is>
       </c>
       <c r="M9" s="7" t="inlineStr">
         <is>
-          <t>57.5%</t>
+          <t>58.4%</t>
         </is>
       </c>
       <c r="N9" s="7" t="inlineStr">
         <is>
-          <t>25.0%</t>
+          <t>24.9%</t>
         </is>
       </c>
       <c r="O9" s="7" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>16.7%</t>
         </is>
       </c>
       <c r="P9" s="7" t="inlineStr">
         <is>
-          <t>55.3%</t>
+          <t>52.0%</t>
         </is>
       </c>
       <c r="Q9" s="7" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>18.0%</t>
         </is>
       </c>
       <c r="R9" s="7" t="inlineStr">
         <is>
-          <t>28.3%</t>
+          <t>30.0%</t>
         </is>
       </c>
     </row>
@@ -1412,42 +1412,42 @@
       </c>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>4.28</t>
+          <t>4.17</t>
         </is>
       </c>
       <c r="L10" s="7" t="inlineStr">
         <is>
-          <t>1.54</t>
+          <t>1.57</t>
         </is>
       </c>
       <c r="M10" s="7" t="inlineStr">
         <is>
-          <t>16.5%</t>
+          <t>16.6%</t>
         </is>
       </c>
       <c r="N10" s="7" t="inlineStr">
         <is>
-          <t>22.1%</t>
+          <t>22.8%</t>
         </is>
       </c>
       <c r="O10" s="7" t="inlineStr">
         <is>
-          <t>61.4%</t>
+          <t>60.6%</t>
         </is>
       </c>
       <c r="P10" s="7" t="inlineStr">
         <is>
-          <t>20.9%</t>
+          <t>20.2%</t>
         </is>
       </c>
       <c r="Q10" s="7" t="inlineStr">
         <is>
-          <t>16.1%</t>
+          <t>19.7%</t>
         </is>
       </c>
       <c r="R10" s="7" t="inlineStr">
         <is>
-          <t>63.0%</t>
+          <t>60.1%</t>
         </is>
       </c>
     </row>
@@ -1502,12 +1502,12 @@
       </c>
       <c r="K11" s="7" t="inlineStr">
         <is>
-          <t>3.73</t>
+          <t>3.72</t>
         </is>
       </c>
       <c r="L11" s="7" t="inlineStr">
         <is>
-          <t>1.70</t>
+          <t>1.71</t>
         </is>
       </c>
       <c r="M11" s="7" t="inlineStr">
@@ -1517,27 +1517,27 @@
       </c>
       <c r="N11" s="7" t="inlineStr">
         <is>
-          <t>25.4%</t>
+          <t>25.5%</t>
         </is>
       </c>
       <c r="O11" s="7" t="inlineStr">
         <is>
-          <t>55.7%</t>
+          <t>55.5%</t>
         </is>
       </c>
       <c r="P11" s="7" t="inlineStr">
         <is>
-          <t>27.1%</t>
+          <t>26.5%</t>
         </is>
       </c>
       <c r="Q11" s="7" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>16.5%</t>
         </is>
       </c>
       <c r="R11" s="7" t="inlineStr">
         <is>
-          <t>55.4%</t>
+          <t>57.0%</t>
         </is>
       </c>
     </row>
@@ -1587,47 +1587,47 @@
       </c>
       <c r="J12" s="7" t="inlineStr">
         <is>
-          <t>1.03</t>
+          <t>1.04</t>
         </is>
       </c>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>17.17</t>
+          <t>16.49</t>
         </is>
       </c>
       <c r="L12" s="7" t="inlineStr">
         <is>
-          <t>36.33</t>
+          <t>45.65</t>
         </is>
       </c>
       <c r="M12" s="7" t="inlineStr">
         <is>
-          <t>91.9%</t>
+          <t>92.1%</t>
         </is>
       </c>
       <c r="N12" s="7" t="inlineStr">
         <is>
-          <t>5.5%</t>
+          <t>5.8%</t>
         </is>
       </c>
       <c r="O12" s="7" t="inlineStr">
         <is>
-          <t>2.6%</t>
+          <t>2.1%</t>
         </is>
       </c>
       <c r="P12" s="7" t="inlineStr">
         <is>
-          <t>85.1%</t>
+          <t>83.5%</t>
         </is>
       </c>
       <c r="Q12" s="7" t="inlineStr">
         <is>
-          <t>7.5%</t>
+          <t>9.3%</t>
         </is>
       </c>
       <c r="R12" s="7" t="inlineStr">
         <is>
-          <t>7.4%</t>
+          <t>7.2%</t>
         </is>
       </c>
     </row>
@@ -1677,22 +1677,22 @@
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>2.00</t>
+          <t>1.98</t>
         </is>
       </c>
       <c r="K13" s="7" t="inlineStr">
         <is>
-          <t>3.52</t>
+          <t>3.57</t>
         </is>
       </c>
       <c r="L13" s="7" t="inlineStr">
         <is>
-          <t>3.57</t>
+          <t>3.78</t>
         </is>
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
-          <t>47.0%</t>
+          <t>48.1%</t>
         </is>
       </c>
       <c r="N13" s="7" t="inlineStr">
@@ -1702,22 +1702,22 @@
       </c>
       <c r="O13" s="7" t="inlineStr">
         <is>
-          <t>26.3%</t>
+          <t>25.2%</t>
         </is>
       </c>
       <c r="P13" s="7" t="inlineStr">
         <is>
-          <t>45.8%</t>
+          <t>48.6%</t>
         </is>
       </c>
       <c r="Q13" s="7" t="inlineStr">
         <is>
-          <t>12.9%</t>
+          <t>13.2%</t>
         </is>
       </c>
       <c r="R13" s="7" t="inlineStr">
         <is>
-          <t>41.3%</t>
+          <t>38.2%</t>
         </is>
       </c>
     </row>
@@ -1767,47 +1767,47 @@
       </c>
       <c r="J14" s="7" t="inlineStr">
         <is>
-          <t>3.53</t>
+          <t>3.58</t>
         </is>
       </c>
       <c r="K14" s="7" t="inlineStr">
         <is>
-          <t>2.83</t>
+          <t>2.80</t>
         </is>
       </c>
       <c r="L14" s="7" t="inlineStr">
         <is>
-          <t>2.39</t>
+          <t>2.42</t>
         </is>
       </c>
       <c r="M14" s="7" t="inlineStr">
         <is>
-          <t>26.9%</t>
+          <t>26.6%</t>
         </is>
       </c>
       <c r="N14" s="7" t="inlineStr">
         <is>
-          <t>33.5%</t>
+          <t>34.0%</t>
         </is>
       </c>
       <c r="O14" s="7" t="inlineStr">
         <is>
-          <t>39.7%</t>
+          <t>39.4%</t>
         </is>
       </c>
       <c r="P14" s="7" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>14.3%</t>
         </is>
       </c>
       <c r="Q14" s="7" t="inlineStr">
         <is>
-          <t>16.3%</t>
+          <t>16.6%</t>
         </is>
       </c>
       <c r="R14" s="7" t="inlineStr">
         <is>
-          <t>70.2%</t>
+          <t>69.1%</t>
         </is>
       </c>
     </row>
@@ -1857,17 +1857,17 @@
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
-          <t>1.88</t>
+          <t>1.89</t>
         </is>
       </c>
       <c r="K15" s="7" t="inlineStr">
         <is>
-          <t>3.40</t>
+          <t>3.47</t>
         </is>
       </c>
       <c r="L15" s="7" t="inlineStr">
         <is>
-          <t>4.37</t>
+          <t>4.29</t>
         </is>
       </c>
       <c r="M15" s="7" t="inlineStr">
@@ -1877,27 +1877,27 @@
       </c>
       <c r="N15" s="7" t="inlineStr">
         <is>
-          <t>27.9%</t>
+          <t>27.4%</t>
         </is>
       </c>
       <c r="O15" s="7" t="inlineStr">
         <is>
-          <t>21.7%</t>
+          <t>22.2%</t>
         </is>
       </c>
       <c r="P15" s="7" t="inlineStr">
         <is>
-          <t>41.2%</t>
+          <t>41.4%</t>
         </is>
       </c>
       <c r="Q15" s="7" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>16.5%</t>
         </is>
       </c>
       <c r="R15" s="7" t="inlineStr">
         <is>
-          <t>43.5%</t>
+          <t>42.1%</t>
         </is>
       </c>
     </row>
@@ -1952,42 +1952,42 @@
       </c>
       <c r="K16" s="7" t="inlineStr">
         <is>
-          <t>10.67</t>
+          <t>11.01</t>
         </is>
       </c>
       <c r="L16" s="7" t="inlineStr">
         <is>
-          <t>24.33</t>
+          <t>26.34</t>
         </is>
       </c>
       <c r="M16" s="7" t="inlineStr">
         <is>
-          <t>87.2%</t>
+          <t>87.7%</t>
         </is>
       </c>
       <c r="N16" s="7" t="inlineStr">
         <is>
-          <t>8.9%</t>
+          <t>8.7%</t>
         </is>
       </c>
       <c r="O16" s="7" t="inlineStr">
         <is>
-          <t>3.9%</t>
+          <t>3.6%</t>
         </is>
       </c>
       <c r="P16" s="7" t="inlineStr">
         <is>
-          <t>89.2%</t>
+          <t>89.0%</t>
         </is>
       </c>
       <c r="Q16" s="7" t="inlineStr">
         <is>
-          <t>6.4%</t>
+          <t>6.2%</t>
         </is>
       </c>
       <c r="R16" s="7" t="inlineStr">
         <is>
-          <t>4.5%</t>
+          <t>4.8%</t>
         </is>
       </c>
     </row>
@@ -2037,47 +2037,47 @@
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
-          <t>1.65</t>
+          <t>1.62</t>
         </is>
       </c>
       <c r="K17" s="7" t="inlineStr">
         <is>
-          <t>3.80</t>
+          <t>3.92</t>
         </is>
       </c>
       <c r="L17" s="7" t="inlineStr">
         <is>
-          <t>5.25</t>
+          <t>5.61</t>
         </is>
       </c>
       <c r="M17" s="7" t="inlineStr">
         <is>
-          <t>57.2%</t>
+          <t>58.8%</t>
         </is>
       </c>
       <c r="N17" s="7" t="inlineStr">
         <is>
-          <t>24.8%</t>
+          <t>24.3%</t>
         </is>
       </c>
       <c r="O17" s="7" t="inlineStr">
         <is>
-          <t>18.0%</t>
+          <t>17.0%</t>
         </is>
       </c>
       <c r="P17" s="7" t="inlineStr">
         <is>
-          <t>55.8%</t>
+          <t>53.8%</t>
         </is>
       </c>
       <c r="Q17" s="7" t="inlineStr">
         <is>
-          <t>12.4%</t>
+          <t>12.1%</t>
         </is>
       </c>
       <c r="R17" s="7" t="inlineStr">
         <is>
-          <t>31.8%</t>
+          <t>34.1%</t>
         </is>
       </c>
     </row>
@@ -2127,47 +2127,47 @@
       </c>
       <c r="J18" s="7" t="inlineStr">
         <is>
-          <t>7.58</t>
+          <t>7.94</t>
         </is>
       </c>
       <c r="K18" s="7" t="inlineStr">
         <is>
-          <t>4.39</t>
+          <t>4.37</t>
         </is>
       </c>
       <c r="L18" s="7" t="inlineStr">
         <is>
-          <t>1.44</t>
+          <t>1.43</t>
         </is>
       </c>
       <c r="M18" s="7" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>11.9%</t>
         </is>
       </c>
       <c r="N18" s="7" t="inlineStr">
         <is>
-          <t>21.6%</t>
+          <t>21.7%</t>
         </is>
       </c>
       <c r="O18" s="7" t="inlineStr">
         <is>
-          <t>65.9%</t>
+          <t>66.3%</t>
         </is>
       </c>
       <c r="P18" s="7" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>13.5%</t>
         </is>
       </c>
       <c r="Q18" s="7" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>15.7%</t>
         </is>
       </c>
       <c r="R18" s="7" t="inlineStr">
         <is>
-          <t>72.3%</t>
+          <t>70.8%</t>
         </is>
       </c>
     </row>
@@ -2207,57 +2207,57 @@
       </c>
       <c r="H19" s="10" t="inlineStr">
         <is>
-          <t>2-0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="I19" s="10" t="inlineStr">
         <is>
-          <t>2-0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J19" s="7" t="inlineStr">
         <is>
-          <t>1.85</t>
+          <t>1.83</t>
         </is>
       </c>
       <c r="K19" s="7" t="inlineStr">
         <is>
-          <t>3.43</t>
+          <t>3.46</t>
         </is>
       </c>
       <c r="L19" s="7" t="inlineStr">
         <is>
-          <t>4.44</t>
+          <t>4.65</t>
         </is>
       </c>
       <c r="M19" s="7" t="inlineStr">
         <is>
-          <t>51.1%</t>
+          <t>52.0%</t>
         </is>
       </c>
       <c r="N19" s="7" t="inlineStr">
         <is>
-          <t>27.6%</t>
+          <t>27.5%</t>
         </is>
       </c>
       <c r="O19" s="7" t="inlineStr">
         <is>
-          <t>21.3%</t>
+          <t>20.5%</t>
         </is>
       </c>
       <c r="P19" s="7" t="inlineStr">
         <is>
-          <t>70.1%</t>
+          <t>69.5%</t>
         </is>
       </c>
       <c r="Q19" s="7" t="inlineStr">
         <is>
-          <t>10.4%</t>
+          <t>11.1%</t>
         </is>
       </c>
       <c r="R19" s="7" t="inlineStr">
         <is>
-          <t>19.5%</t>
+          <t>19.4%</t>
         </is>
       </c>
     </row>
@@ -2312,42 +2312,42 @@
       </c>
       <c r="K20" s="7" t="inlineStr">
         <is>
-          <t>4.41</t>
+          <t>4.33</t>
         </is>
       </c>
       <c r="L20" s="7" t="inlineStr">
         <is>
-          <t>6.83</t>
+          <t>7.15</t>
         </is>
       </c>
       <c r="M20" s="7" t="inlineStr">
         <is>
-          <t>64.6%</t>
+          <t>64.7%</t>
         </is>
       </c>
       <c r="N20" s="7" t="inlineStr">
         <is>
-          <t>21.5%</t>
+          <t>22.0%</t>
         </is>
       </c>
       <c r="O20" s="7" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>13.3%</t>
         </is>
       </c>
       <c r="P20" s="7" t="inlineStr">
         <is>
-          <t>65.1%</t>
+          <t>64.7%</t>
         </is>
       </c>
       <c r="Q20" s="7" t="inlineStr">
         <is>
-          <t>13.6%</t>
+          <t>13.4%</t>
         </is>
       </c>
       <c r="R20" s="7" t="inlineStr">
         <is>
-          <t>21.3%</t>
+          <t>21.9%</t>
         </is>
       </c>
     </row>
@@ -2397,47 +2397,47 @@
       </c>
       <c r="J21" s="7" t="inlineStr">
         <is>
-          <t>13.17</t>
+          <t>14.10</t>
         </is>
       </c>
       <c r="K21" s="7" t="inlineStr">
         <is>
-          <t>7.00</t>
+          <t>6.86</t>
         </is>
       </c>
       <c r="L21" s="7" t="inlineStr">
         <is>
-          <t>1.21</t>
+          <t>1.20</t>
         </is>
       </c>
       <c r="M21" s="7" t="inlineStr">
         <is>
-          <t>7.3%</t>
+          <t>6.8%</t>
         </is>
       </c>
       <c r="N21" s="7" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>13.9%</t>
         </is>
       </c>
       <c r="O21" s="7" t="inlineStr">
         <is>
-          <t>79.1%</t>
+          <t>79.4%</t>
         </is>
       </c>
       <c r="P21" s="7" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>16.1%</t>
         </is>
       </c>
       <c r="Q21" s="7" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>14.8%</t>
         </is>
       </c>
       <c r="R21" s="7" t="inlineStr">
         <is>
-          <t>69.9%</t>
+          <t>69.2%</t>
         </is>
       </c>
     </row>
@@ -2487,47 +2487,47 @@
       </c>
       <c r="J22" s="7" t="inlineStr">
         <is>
-          <t>1.39</t>
+          <t>1.40</t>
         </is>
       </c>
       <c r="K22" s="7" t="inlineStr">
         <is>
-          <t>4.62</t>
+          <t>4.49</t>
         </is>
       </c>
       <c r="L22" s="7" t="inlineStr">
         <is>
-          <t>8.58</t>
+          <t>8.77</t>
         </is>
       </c>
       <c r="M22" s="7" t="inlineStr">
         <is>
-          <t>68.4%</t>
+          <t>68.0%</t>
         </is>
       </c>
       <c r="N22" s="7" t="inlineStr">
         <is>
-          <t>20.6%</t>
+          <t>21.2%</t>
         </is>
       </c>
       <c r="O22" s="7" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>10.8%</t>
         </is>
       </c>
       <c r="P22" s="7" t="inlineStr">
         <is>
-          <t>77.3%</t>
+          <t>77.0%</t>
         </is>
       </c>
       <c r="Q22" s="7" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.9%</t>
         </is>
       </c>
       <c r="R22" s="7" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.1%</t>
         </is>
       </c>
     </row>
@@ -2577,27 +2577,27 @@
       </c>
       <c r="J23" s="7" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.33</t>
         </is>
       </c>
       <c r="K23" s="7" t="inlineStr">
         <is>
-          <t>5.50</t>
+          <t>5.31</t>
         </is>
       </c>
       <c r="L23" s="7" t="inlineStr">
         <is>
-          <t>9.00</t>
+          <t>8.96</t>
         </is>
       </c>
       <c r="M23" s="7" t="inlineStr">
         <is>
-          <t>72.1%</t>
+          <t>71.5%</t>
         </is>
       </c>
       <c r="N23" s="7" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>17.9%</t>
         </is>
       </c>
       <c r="O23" s="7" t="inlineStr">
@@ -2607,17 +2607,17 @@
       </c>
       <c r="P23" s="7" t="inlineStr">
         <is>
-          <t>62.6%</t>
+          <t>61.3%</t>
         </is>
       </c>
       <c r="Q23" s="7" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.6%</t>
         </is>
       </c>
       <c r="R23" s="7" t="inlineStr">
         <is>
-          <t>23.2%</t>
+          <t>24.1%</t>
         </is>
       </c>
     </row>
@@ -2667,47 +2667,47 @@
       </c>
       <c r="J24" s="7" t="inlineStr">
         <is>
-          <t>1.27</t>
+          <t>1.28</t>
         </is>
       </c>
       <c r="K24" s="7" t="inlineStr">
         <is>
-          <t>5.83</t>
+          <t>5.61</t>
         </is>
       </c>
       <c r="L24" s="7" t="inlineStr">
         <is>
-          <t>10.33</t>
+          <t>10.93</t>
         </is>
       </c>
       <c r="M24" s="7" t="inlineStr">
         <is>
-          <t>74.6%</t>
+          <t>74.3%</t>
         </is>
       </c>
       <c r="N24" s="7" t="inlineStr">
         <is>
-          <t>16.2%</t>
+          <t>17.0%</t>
         </is>
       </c>
       <c r="O24" s="7" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>8.7%</t>
         </is>
       </c>
       <c r="P24" s="7" t="inlineStr">
         <is>
-          <t>75.7%</t>
+          <t>75.6%</t>
         </is>
       </c>
       <c r="Q24" s="7" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>14.0%</t>
         </is>
       </c>
       <c r="R24" s="7" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.4%</t>
         </is>
       </c>
     </row>
@@ -2757,17 +2757,17 @@
       </c>
       <c r="J25" s="7" t="inlineStr">
         <is>
-          <t>1.72</t>
+          <t>1.73</t>
         </is>
       </c>
       <c r="K25" s="7" t="inlineStr">
         <is>
-          <t>3.78</t>
+          <t>3.77</t>
         </is>
       </c>
       <c r="L25" s="7" t="inlineStr">
         <is>
-          <t>4.78</t>
+          <t>4.87</t>
         </is>
       </c>
       <c r="M25" s="7" t="inlineStr">
@@ -2777,27 +2777,27 @@
       </c>
       <c r="N25" s="7" t="inlineStr">
         <is>
-          <t>25.1%</t>
+          <t>25.3%</t>
         </is>
       </c>
       <c r="O25" s="7" t="inlineStr">
         <is>
-          <t>19.8%</t>
+          <t>19.6%</t>
         </is>
       </c>
       <c r="P25" s="7" t="inlineStr">
         <is>
-          <t>50.8%</t>
+          <t>52.7%</t>
         </is>
       </c>
       <c r="Q25" s="7" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>17.4%</t>
         </is>
       </c>
       <c r="R25" s="7" t="inlineStr">
         <is>
-          <t>33.5%</t>
+          <t>29.9%</t>
         </is>
       </c>
     </row>
@@ -2820,12 +2820,12 @@
           <t>L</t>
         </is>
       </c>
-      <c r="E26" s="9" t="inlineStr">
+      <c r="E26" s="8" t="inlineStr">
         <is>
           <t>Ghana</t>
         </is>
       </c>
-      <c r="F26" s="8" t="inlineStr">
+      <c r="F26" s="9" t="inlineStr">
         <is>
           <t>Panama</t>
         </is>
@@ -2842,12 +2842,12 @@
       </c>
       <c r="I26" s="10" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J26" s="7" t="inlineStr">
         <is>
-          <t>2.07</t>
+          <t>2.14</t>
         </is>
       </c>
       <c r="K26" s="7" t="inlineStr">
@@ -2857,37 +2857,37 @@
       </c>
       <c r="L26" s="7" t="inlineStr">
         <is>
-          <t>3.58</t>
+          <t>3.45</t>
         </is>
       </c>
       <c r="M26" s="7" t="inlineStr">
         <is>
-          <t>45.8%</t>
+          <t>44.5%</t>
         </is>
       </c>
       <c r="N26" s="7" t="inlineStr">
         <is>
-          <t>27.7%</t>
+          <t>27.9%</t>
         </is>
       </c>
       <c r="O26" s="7" t="inlineStr">
         <is>
-          <t>26.5%</t>
+          <t>27.6%</t>
         </is>
       </c>
       <c r="P26" s="7" t="inlineStr">
         <is>
-          <t>22.9%</t>
+          <t>23.2%</t>
         </is>
       </c>
       <c r="Q26" s="7" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>13.4%</t>
         </is>
       </c>
       <c r="R26" s="7" t="inlineStr">
         <is>
-          <t>64.1%</t>
+          <t>63.4%</t>
         </is>
       </c>
     </row>
@@ -2937,47 +2937,47 @@
       </c>
       <c r="J27" s="7" t="inlineStr">
         <is>
-          <t>8.25</t>
+          <t>8.75</t>
         </is>
       </c>
       <c r="K27" s="7" t="inlineStr">
         <is>
-          <t>4.60</t>
+          <t>4.58</t>
         </is>
       </c>
       <c r="L27" s="7" t="inlineStr">
         <is>
-          <t>1.40</t>
+          <t>1.39</t>
         </is>
       </c>
       <c r="M27" s="7" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>10.9%</t>
         </is>
       </c>
       <c r="N27" s="7" t="inlineStr">
         <is>
-          <t>20.6%</t>
+          <t>20.8%</t>
         </is>
       </c>
       <c r="O27" s="7" t="inlineStr">
         <is>
-          <t>67.8%</t>
+          <t>68.4%</t>
         </is>
       </c>
       <c r="P27" s="7" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>17.5%</t>
         </is>
       </c>
       <c r="Q27" s="7" t="inlineStr">
         <is>
-          <t>13.4%</t>
+          <t>16.2%</t>
         </is>
       </c>
       <c r="R27" s="7" t="inlineStr">
         <is>
-          <t>70.1%</t>
+          <t>66.3%</t>
         </is>
       </c>
     </row>
@@ -3027,47 +3027,47 @@
       </c>
       <c r="J28" s="7" t="inlineStr">
         <is>
-          <t>1.95</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="K28" s="7" t="inlineStr">
         <is>
-          <t>3.32</t>
+          <t>3.75</t>
         </is>
       </c>
       <c r="L28" s="7" t="inlineStr">
         <is>
-          <t>4.10</t>
+          <t>4.69</t>
         </is>
       </c>
       <c r="M28" s="7" t="inlineStr">
         <is>
-          <t>48.5%</t>
+          <t>54.4%</t>
         </is>
       </c>
       <c r="N28" s="7" t="inlineStr">
         <is>
-          <t>28.5%</t>
+          <t>25.4%</t>
         </is>
       </c>
       <c r="O28" s="7" t="inlineStr">
         <is>
-          <t>23.1%</t>
+          <t>20.3%</t>
         </is>
       </c>
       <c r="P28" s="7" t="inlineStr">
         <is>
-          <t>52.4%</t>
+          <t>50.8%</t>
         </is>
       </c>
       <c r="Q28" s="7" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="R28" s="7" t="inlineStr">
         <is>
-          <t>32.5%</t>
+          <t>34.7%</t>
         </is>
       </c>
     </row>
@@ -3117,47 +3117,47 @@
       </c>
       <c r="J29" s="7" t="inlineStr">
         <is>
-          <t>1.58</t>
+          <t>1.60</t>
         </is>
       </c>
       <c r="K29" s="7" t="inlineStr">
         <is>
-          <t>3.90</t>
+          <t>3.96</t>
         </is>
       </c>
       <c r="L29" s="7" t="inlineStr">
         <is>
-          <t>5.33</t>
+          <t>5.63</t>
         </is>
       </c>
       <c r="M29" s="7" t="inlineStr">
         <is>
-          <t>58.8%</t>
+          <t>59.2%</t>
         </is>
       </c>
       <c r="N29" s="7" t="inlineStr">
         <is>
-          <t>23.8%</t>
+          <t>23.9%</t>
         </is>
       </c>
       <c r="O29" s="7" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>16.8%</t>
         </is>
       </c>
       <c r="P29" s="7" t="inlineStr">
         <is>
-          <t>74.8%</t>
+          <t>77.0%</t>
         </is>
       </c>
       <c r="Q29" s="7" t="inlineStr">
         <is>
-          <t>11.3%</t>
+          <t>10.4%</t>
         </is>
       </c>
       <c r="R29" s="7" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>12.6%</t>
         </is>
       </c>
     </row>
@@ -3212,42 +3212,42 @@
       </c>
       <c r="K30" s="7" t="inlineStr">
         <is>
-          <t>5.00</t>
+          <t>5.17</t>
         </is>
       </c>
       <c r="L30" s="7" t="inlineStr">
         <is>
-          <t>9.92</t>
+          <t>10.83</t>
         </is>
       </c>
       <c r="M30" s="7" t="inlineStr">
         <is>
-          <t>71.9%</t>
+          <t>72.9%</t>
         </is>
       </c>
       <c r="N30" s="7" t="inlineStr">
         <is>
-          <t>18.7%</t>
+          <t>18.3%</t>
         </is>
       </c>
       <c r="O30" s="7" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>8.8%</t>
         </is>
       </c>
       <c r="P30" s="7" t="inlineStr">
         <is>
-          <t>82.7%</t>
+          <t>81.9%</t>
         </is>
       </c>
       <c r="Q30" s="7" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.8%</t>
         </is>
       </c>
       <c r="R30" s="7" t="inlineStr">
         <is>
-          <t>7.7%</t>
+          <t>8.4%</t>
         </is>
       </c>
     </row>
@@ -3297,47 +3297,47 @@
       </c>
       <c r="J31" s="7" t="inlineStr">
         <is>
-          <t>1.79</t>
+          <t>1.99</t>
         </is>
       </c>
       <c r="K31" s="7" t="inlineStr">
         <is>
-          <t>3.45</t>
+          <t>3.32</t>
         </is>
       </c>
       <c r="L31" s="7" t="inlineStr">
         <is>
-          <t>4.43</t>
+          <t>4.03</t>
         </is>
       </c>
       <c r="M31" s="7" t="inlineStr">
         <is>
-          <t>52.0%</t>
+          <t>47.8%</t>
         </is>
       </c>
       <c r="N31" s="7" t="inlineStr">
         <is>
-          <t>27.0%</t>
+          <t>28.6%</t>
         </is>
       </c>
       <c r="O31" s="7" t="inlineStr">
         <is>
-          <t>21.0%</t>
+          <t>23.6%</t>
         </is>
       </c>
       <c r="P31" s="7" t="inlineStr">
         <is>
-          <t>64.6%</t>
+          <t>62.8%</t>
         </is>
       </c>
       <c r="Q31" s="7" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>16.3%</t>
         </is>
       </c>
       <c r="R31" s="7" t="inlineStr">
         <is>
-          <t>20.0%</t>
+          <t>20.9%</t>
         </is>
       </c>
     </row>
@@ -3392,42 +3392,42 @@
       </c>
       <c r="K32" s="7" t="inlineStr">
         <is>
-          <t>3.72</t>
+          <t>3.84</t>
         </is>
       </c>
       <c r="L32" s="7" t="inlineStr">
         <is>
-          <t>4.34</t>
+          <t>4.46</t>
         </is>
       </c>
       <c r="M32" s="7" t="inlineStr">
         <is>
-          <t>53.7%</t>
+          <t>54.4%</t>
         </is>
       </c>
       <c r="N32" s="7" t="inlineStr">
         <is>
-          <t>25.0%</t>
+          <t>24.5%</t>
         </is>
       </c>
       <c r="O32" s="7" t="inlineStr">
         <is>
-          <t>21.4%</t>
+          <t>21.1%</t>
         </is>
       </c>
       <c r="P32" s="7" t="inlineStr">
         <is>
-          <t>55.3%</t>
+          <t>54.0%</t>
         </is>
       </c>
       <c r="Q32" s="7" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>17.1%</t>
         </is>
       </c>
       <c r="R32" s="7" t="inlineStr">
         <is>
-          <t>29.4%</t>
+          <t>28.9%</t>
         </is>
       </c>
     </row>
@@ -3477,7 +3477,7 @@
       </c>
       <c r="J33" s="7" t="inlineStr">
         <is>
-          <t>3.93</t>
+          <t>4.02</t>
         </is>
       </c>
       <c r="K33" s="7" t="inlineStr">
@@ -3487,22 +3487,22 @@
       </c>
       <c r="L33" s="7" t="inlineStr">
         <is>
-          <t>1.95</t>
+          <t>1.98</t>
         </is>
       </c>
       <c r="M33" s="7" t="inlineStr">
         <is>
-          <t>23.6%</t>
+          <t>23.4%</t>
         </is>
       </c>
       <c r="N33" s="7" t="inlineStr">
         <is>
-          <t>28.7%</t>
+          <t>29.1%</t>
         </is>
       </c>
       <c r="O33" s="7" t="inlineStr">
         <is>
-          <t>47.6%</t>
+          <t>47.5%</t>
         </is>
       </c>
       <c r="P33" s="7" t="inlineStr">
@@ -3567,47 +3567,47 @@
       </c>
       <c r="J34" s="7" t="inlineStr">
         <is>
-          <t>1.08</t>
+          <t>1.07</t>
         </is>
       </c>
       <c r="K34" s="7" t="inlineStr">
         <is>
-          <t>11.17</t>
+          <t>10.85</t>
         </is>
       </c>
       <c r="L34" s="7" t="inlineStr">
         <is>
-          <t>24.50</t>
+          <t>29.58</t>
         </is>
       </c>
       <c r="M34" s="7" t="inlineStr">
         <is>
-          <t>87.7%</t>
+          <t>88.1%</t>
         </is>
       </c>
       <c r="N34" s="7" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.7%</t>
         </is>
       </c>
       <c r="O34" s="7" t="inlineStr">
         <is>
-          <t>3.9%</t>
+          <t>3.2%</t>
         </is>
       </c>
       <c r="P34" s="7" t="inlineStr">
         <is>
-          <t>86.7%</t>
+          <t>87.6%</t>
         </is>
       </c>
       <c r="Q34" s="7" t="inlineStr">
         <is>
-          <t>6.8%</t>
+          <t>6.4%</t>
         </is>
       </c>
       <c r="R34" s="7" t="inlineStr">
         <is>
-          <t>6.5%</t>
+          <t>6.0%</t>
         </is>
       </c>
     </row>
@@ -3657,17 +3657,17 @@
       </c>
       <c r="J35" s="7" t="inlineStr">
         <is>
-          <t>2.18</t>
+          <t>2.21</t>
         </is>
       </c>
       <c r="K35" s="7" t="inlineStr">
         <is>
-          <t>3.10</t>
+          <t>3.13</t>
         </is>
       </c>
       <c r="L35" s="7" t="inlineStr">
         <is>
-          <t>3.35</t>
+          <t>3.41</t>
         </is>
       </c>
       <c r="M35" s="7" t="inlineStr">
@@ -3677,27 +3677,27 @@
       </c>
       <c r="N35" s="7" t="inlineStr">
         <is>
-          <t>29.9%</t>
+          <t>30.0%</t>
         </is>
       </c>
       <c r="O35" s="7" t="inlineStr">
         <is>
-          <t>27.6%</t>
+          <t>27.5%</t>
         </is>
       </c>
       <c r="P35" s="7" t="inlineStr">
         <is>
-          <t>40.9%</t>
+          <t>39.7%</t>
         </is>
       </c>
       <c r="Q35" s="7" t="inlineStr">
         <is>
-          <t>15.5%</t>
+          <t>16.6%</t>
         </is>
       </c>
       <c r="R35" s="7" t="inlineStr">
         <is>
-          <t>43.6%</t>
+          <t>43.7%</t>
         </is>
       </c>
     </row>
@@ -3737,12 +3737,12 @@
       </c>
       <c r="H36" s="10" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>2-0</t>
         </is>
       </c>
       <c r="I36" s="10" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>2-0</t>
         </is>
       </c>
       <c r="J36" s="7" t="inlineStr">
@@ -3752,17 +3752,17 @@
       </c>
       <c r="K36" s="7" t="inlineStr">
         <is>
-          <t>3.93</t>
+          <t>3.98</t>
         </is>
       </c>
       <c r="L36" s="7" t="inlineStr">
         <is>
-          <t>4.92</t>
+          <t>5.16</t>
         </is>
       </c>
       <c r="M36" s="7" t="inlineStr">
         <is>
-          <t>57.4%</t>
+          <t>58.1%</t>
         </is>
       </c>
       <c r="N36" s="7" t="inlineStr">
@@ -3772,22 +3772,22 @@
       </c>
       <c r="O36" s="7" t="inlineStr">
         <is>
-          <t>18.9%</t>
+          <t>18.2%</t>
         </is>
       </c>
       <c r="P36" s="7" t="inlineStr">
         <is>
-          <t>65.3%</t>
+          <t>67.4%</t>
         </is>
       </c>
       <c r="Q36" s="7" t="inlineStr">
         <is>
-          <t>13.8%</t>
+          <t>12.6%</t>
         </is>
       </c>
       <c r="R36" s="7" t="inlineStr">
         <is>
-          <t>21.0%</t>
+          <t>20.0%</t>
         </is>
       </c>
     </row>
@@ -3837,22 +3837,22 @@
       </c>
       <c r="J37" s="7" t="inlineStr">
         <is>
-          <t>1.53</t>
+          <t>1.55</t>
         </is>
       </c>
       <c r="K37" s="7" t="inlineStr">
         <is>
-          <t>4.17</t>
+          <t>4.23</t>
         </is>
       </c>
       <c r="L37" s="7" t="inlineStr">
         <is>
-          <t>5.42</t>
+          <t>5.52</t>
         </is>
       </c>
       <c r="M37" s="7" t="inlineStr">
         <is>
-          <t>60.6%</t>
+          <t>60.7%</t>
         </is>
       </c>
       <c r="N37" s="7" t="inlineStr">
@@ -3862,22 +3862,22 @@
       </c>
       <c r="O37" s="7" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>17.0%</t>
         </is>
       </c>
       <c r="P37" s="7" t="inlineStr">
         <is>
-          <t>70.9%</t>
+          <t>68.9%</t>
         </is>
       </c>
       <c r="Q37" s="7" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>13.6%</t>
         </is>
       </c>
       <c r="R37" s="7" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>17.6%</t>
         </is>
       </c>
     </row>
@@ -3932,42 +3932,42 @@
       </c>
       <c r="K38" s="7" t="inlineStr">
         <is>
-          <t>6.75</t>
+          <t>6.85</t>
         </is>
       </c>
       <c r="L38" s="7" t="inlineStr">
         <is>
-          <t>12.33</t>
+          <t>13.84</t>
         </is>
       </c>
       <c r="M38" s="7" t="inlineStr">
         <is>
-          <t>78.6%</t>
+          <t>79.4%</t>
         </is>
       </c>
       <c r="N38" s="7" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>13.8%</t>
         </is>
       </c>
       <c r="O38" s="7" t="inlineStr">
         <is>
-          <t>7.6%</t>
+          <t>6.8%</t>
         </is>
       </c>
       <c r="P38" s="7" t="inlineStr">
         <is>
-          <t>87.1%</t>
+          <t>87.4%</t>
         </is>
       </c>
       <c r="Q38" s="7" t="inlineStr">
         <is>
-          <t>6.1%</t>
+          <t>6.3%</t>
         </is>
       </c>
       <c r="R38" s="7" t="inlineStr">
         <is>
-          <t>6.8%</t>
+          <t>6.3%</t>
         </is>
       </c>
     </row>
@@ -4017,47 +4017,47 @@
       </c>
       <c r="J39" s="7" t="inlineStr">
         <is>
-          <t>5.08</t>
+          <t>5.23</t>
         </is>
       </c>
       <c r="K39" s="7" t="inlineStr">
         <is>
-          <t>3.50</t>
+          <t>3.53</t>
         </is>
       </c>
       <c r="L39" s="7" t="inlineStr">
         <is>
-          <t>1.69</t>
+          <t>1.70</t>
         </is>
       </c>
       <c r="M39" s="7" t="inlineStr">
         <is>
-          <t>18.3%</t>
+          <t>18.0%</t>
         </is>
       </c>
       <c r="N39" s="7" t="inlineStr">
         <is>
-          <t>26.6%</t>
+          <t>26.7%</t>
         </is>
       </c>
       <c r="O39" s="7" t="inlineStr">
         <is>
-          <t>55.1%</t>
+          <t>55.4%</t>
         </is>
       </c>
       <c r="P39" s="7" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>17.0%</t>
         </is>
       </c>
       <c r="Q39" s="7" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>17.2%</t>
         </is>
       </c>
       <c r="R39" s="7" t="inlineStr">
         <is>
-          <t>67.4%</t>
+          <t>65.8%</t>
         </is>
       </c>
     </row>
@@ -4112,42 +4112,42 @@
       </c>
       <c r="K40" s="7" t="inlineStr">
         <is>
-          <t>9.42</t>
+          <t>9.46</t>
         </is>
       </c>
       <c r="L40" s="7" t="inlineStr">
         <is>
-          <t>19.17</t>
+          <t>24.87</t>
         </is>
       </c>
       <c r="M40" s="7" t="inlineStr">
         <is>
-          <t>85.2%</t>
+          <t>86.2%</t>
         </is>
       </c>
       <c r="N40" s="7" t="inlineStr">
         <is>
-          <t>9.9%</t>
+          <t>10.0%</t>
         </is>
       </c>
       <c r="O40" s="7" t="inlineStr">
         <is>
-          <t>4.9%</t>
+          <t>3.8%</t>
         </is>
       </c>
       <c r="P40" s="7" t="inlineStr">
         <is>
-          <t>89.0%</t>
+          <t>89.2%</t>
         </is>
       </c>
       <c r="Q40" s="7" t="inlineStr">
         <is>
-          <t>7.1%</t>
+          <t>6.9%</t>
         </is>
       </c>
       <c r="R40" s="7" t="inlineStr">
         <is>
-          <t>4.0%</t>
+          <t>3.9%</t>
         </is>
       </c>
     </row>
@@ -4197,47 +4197,47 @@
       </c>
       <c r="J41" s="7" t="inlineStr">
         <is>
-          <t>1.39</t>
+          <t>1.40</t>
         </is>
       </c>
       <c r="K41" s="7" t="inlineStr">
         <is>
-          <t>4.55</t>
+          <t>4.60</t>
         </is>
       </c>
       <c r="L41" s="7" t="inlineStr">
         <is>
-          <t>7.25</t>
+          <t>7.65</t>
         </is>
       </c>
       <c r="M41" s="7" t="inlineStr">
         <is>
-          <t>66.8%</t>
+          <t>67.2%</t>
         </is>
       </c>
       <c r="N41" s="7" t="inlineStr">
         <is>
-          <t>20.4%</t>
+          <t>20.5%</t>
         </is>
       </c>
       <c r="O41" s="7" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>12.3%</t>
         </is>
       </c>
       <c r="P41" s="7" t="inlineStr">
         <is>
-          <t>49.3%</t>
+          <t>49.0%</t>
         </is>
       </c>
       <c r="Q41" s="7" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>13.0%</t>
         </is>
       </c>
       <c r="R41" s="7" t="inlineStr">
         <is>
-          <t>37.8%</t>
+          <t>38.0%</t>
         </is>
       </c>
     </row>
@@ -4287,47 +4287,47 @@
       </c>
       <c r="J42" s="7" t="inlineStr">
         <is>
-          <t>1.43</t>
+          <t>1.42</t>
         </is>
       </c>
       <c r="K42" s="7" t="inlineStr">
         <is>
-          <t>4.34</t>
+          <t>4.43</t>
         </is>
       </c>
       <c r="L42" s="7" t="inlineStr">
         <is>
-          <t>6.92</t>
+          <t>7.51</t>
         </is>
       </c>
       <c r="M42" s="7" t="inlineStr">
         <is>
-          <t>65.1%</t>
+          <t>66.2%</t>
         </is>
       </c>
       <c r="N42" s="7" t="inlineStr">
         <is>
-          <t>21.4%</t>
+          <t>21.2%</t>
         </is>
       </c>
       <c r="O42" s="7" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>12.5%</t>
         </is>
       </c>
       <c r="P42" s="7" t="inlineStr">
         <is>
-          <t>84.3%</t>
+          <t>84.5%</t>
         </is>
       </c>
       <c r="Q42" s="7" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>8.9%</t>
         </is>
       </c>
       <c r="R42" s="7" t="inlineStr">
         <is>
-          <t>7.2%</t>
+          <t>6.6%</t>
         </is>
       </c>
     </row>
@@ -4377,47 +4377,47 @@
       </c>
       <c r="J43" s="7" t="inlineStr">
         <is>
-          <t>4.70</t>
+          <t>4.63</t>
         </is>
       </c>
       <c r="K43" s="7" t="inlineStr">
         <is>
-          <t>3.55</t>
+          <t>3.72</t>
         </is>
       </c>
       <c r="L43" s="7" t="inlineStr">
         <is>
-          <t>1.72</t>
+          <t>1.73</t>
         </is>
       </c>
       <c r="M43" s="7" t="inlineStr">
         <is>
-          <t>19.8%</t>
+          <t>20.3%</t>
         </is>
       </c>
       <c r="N43" s="7" t="inlineStr">
         <is>
-          <t>26.2%</t>
+          <t>25.3%</t>
         </is>
       </c>
       <c r="O43" s="7" t="inlineStr">
         <is>
-          <t>54.0%</t>
+          <t>54.4%</t>
         </is>
       </c>
       <c r="P43" s="7" t="inlineStr">
         <is>
-          <t>24.7%</t>
+          <t>25.5%</t>
         </is>
       </c>
       <c r="Q43" s="7" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>16.7%</t>
         </is>
       </c>
       <c r="R43" s="7" t="inlineStr">
         <is>
-          <t>57.9%</t>
+          <t>57.8%</t>
         </is>
       </c>
     </row>
@@ -4467,47 +4467,47 @@
       </c>
       <c r="J44" s="7" t="inlineStr">
         <is>
-          <t>1.61</t>
+          <t>1.63</t>
         </is>
       </c>
       <c r="K44" s="7" t="inlineStr">
         <is>
-          <t>3.73</t>
+          <t>3.77</t>
         </is>
       </c>
       <c r="L44" s="7" t="inlineStr">
         <is>
-          <t>5.35</t>
+          <t>5.45</t>
         </is>
       </c>
       <c r="M44" s="7" t="inlineStr">
         <is>
-          <t>57.7%</t>
+          <t>57.8%</t>
         </is>
       </c>
       <c r="N44" s="7" t="inlineStr">
         <is>
-          <t>24.9%</t>
+          <t>25.0%</t>
         </is>
       </c>
       <c r="O44" s="7" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>17.3%</t>
         </is>
       </c>
       <c r="P44" s="7" t="inlineStr">
         <is>
-          <t>72.6%</t>
+          <t>74.9%</t>
         </is>
       </c>
       <c r="Q44" s="7" t="inlineStr">
         <is>
-          <t>11.3%</t>
+          <t>10.8%</t>
         </is>
       </c>
       <c r="R44" s="7" t="inlineStr">
         <is>
-          <t>16.1%</t>
+          <t>14.3%</t>
         </is>
       </c>
     </row>
@@ -4557,47 +4557,47 @@
       </c>
       <c r="J45" s="7" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>1.12</t>
         </is>
       </c>
       <c r="K45" s="7" t="inlineStr">
         <is>
-          <t>8.67</t>
+          <t>8.19</t>
         </is>
       </c>
       <c r="L45" s="7" t="inlineStr">
         <is>
-          <t>20.50</t>
+          <t>24.16</t>
         </is>
       </c>
       <c r="M45" s="7" t="inlineStr">
         <is>
-          <t>84.6%</t>
+          <t>84.5%</t>
         </is>
       </c>
       <c r="N45" s="7" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>11.6%</t>
         </is>
       </c>
       <c r="O45" s="7" t="inlineStr">
         <is>
-          <t>4.6%</t>
+          <t>3.9%</t>
         </is>
       </c>
       <c r="P45" s="7" t="inlineStr">
         <is>
-          <t>81.8%</t>
+          <t>81.7%</t>
         </is>
       </c>
       <c r="Q45" s="7" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>8.7%</t>
         </is>
       </c>
       <c r="R45" s="7" t="inlineStr">
         <is>
-          <t>8.9%</t>
+          <t>9.6%</t>
         </is>
       </c>
     </row>
@@ -4647,47 +4647,47 @@
       </c>
       <c r="J46" s="7" t="inlineStr">
         <is>
-          <t>2.08</t>
+          <t>2.12</t>
         </is>
       </c>
       <c r="K46" s="7" t="inlineStr">
         <is>
-          <t>3.37</t>
+          <t>3.44</t>
         </is>
       </c>
       <c r="L46" s="7" t="inlineStr">
         <is>
-          <t>3.37</t>
+          <t>3.34</t>
         </is>
       </c>
       <c r="M46" s="7" t="inlineStr">
         <is>
-          <t>44.8%</t>
+          <t>44.4%</t>
         </is>
       </c>
       <c r="N46" s="7" t="inlineStr">
         <is>
-          <t>27.6%</t>
+          <t>27.4%</t>
         </is>
       </c>
       <c r="O46" s="7" t="inlineStr">
         <is>
-          <t>27.6%</t>
+          <t>28.2%</t>
         </is>
       </c>
       <c r="P46" s="7" t="inlineStr">
         <is>
-          <t>45.5%</t>
+          <t>44.3%</t>
         </is>
       </c>
       <c r="Q46" s="7" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>16.2%</t>
         </is>
       </c>
       <c r="R46" s="7" t="inlineStr">
         <is>
-          <t>38.7%</t>
+          <t>39.5%</t>
         </is>
       </c>
     </row>
@@ -4737,12 +4737,12 @@
       </c>
       <c r="J47" s="7" t="inlineStr">
         <is>
-          <t>6.25</t>
+          <t>6.33</t>
         </is>
       </c>
       <c r="K47" s="7" t="inlineStr">
         <is>
-          <t>3.97</t>
+          <t>4.07</t>
         </is>
       </c>
       <c r="L47" s="7" t="inlineStr">
@@ -4752,32 +4752,32 @@
       </c>
       <c r="M47" s="7" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>14.8%</t>
         </is>
       </c>
       <c r="N47" s="7" t="inlineStr">
         <is>
-          <t>23.5%</t>
+          <t>23.1%</t>
         </is>
       </c>
       <c r="O47" s="7" t="inlineStr">
         <is>
-          <t>61.7%</t>
+          <t>62.1%</t>
         </is>
       </c>
       <c r="P47" s="7" t="inlineStr">
         <is>
-          <t>27.7%</t>
+          <t>28.2%</t>
         </is>
       </c>
       <c r="Q47" s="7" t="inlineStr">
         <is>
-          <t>13.1%</t>
+          <t>13.8%</t>
         </is>
       </c>
       <c r="R47" s="7" t="inlineStr">
         <is>
-          <t>59.2%</t>
+          <t>57.9%</t>
         </is>
       </c>
     </row>
@@ -4832,17 +4832,17 @@
       </c>
       <c r="K48" s="7" t="inlineStr">
         <is>
-          <t>6.17</t>
+          <t>6.21</t>
         </is>
       </c>
       <c r="L48" s="7" t="inlineStr">
         <is>
-          <t>9.92</t>
+          <t>11.20</t>
         </is>
       </c>
       <c r="M48" s="7" t="inlineStr">
         <is>
-          <t>75.4%</t>
+          <t>76.3%</t>
         </is>
       </c>
       <c r="N48" s="7" t="inlineStr">
@@ -4852,22 +4852,22 @@
       </c>
       <c r="O48" s="7" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>8.4%</t>
         </is>
       </c>
       <c r="P48" s="7" t="inlineStr">
         <is>
-          <t>68.0%</t>
+          <t>67.2%</t>
         </is>
       </c>
       <c r="Q48" s="7" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>17.3%</t>
         </is>
       </c>
       <c r="R48" s="7" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>15.5%</t>
         </is>
       </c>
     </row>
@@ -4917,47 +4917,47 @@
       </c>
       <c r="J49" s="7" t="inlineStr">
         <is>
-          <t>1.31</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="K49" s="7" t="inlineStr">
         <is>
-          <t>5.10</t>
+          <t>5.14</t>
         </is>
       </c>
       <c r="L49" s="7" t="inlineStr">
         <is>
-          <t>9.00</t>
+          <t>9.33</t>
         </is>
       </c>
       <c r="M49" s="7" t="inlineStr">
         <is>
-          <t>71.3%</t>
+          <t>71.5%</t>
         </is>
       </c>
       <c r="N49" s="7" t="inlineStr">
         <is>
-          <t>18.3%</t>
+          <t>18.4%</t>
         </is>
       </c>
       <c r="O49" s="7" t="inlineStr">
         <is>
-          <t>10.4%</t>
+          <t>10.1%</t>
         </is>
       </c>
       <c r="P49" s="7" t="inlineStr">
         <is>
-          <t>87.2%</t>
+          <t>88.1%</t>
         </is>
       </c>
       <c r="Q49" s="7" t="inlineStr">
         <is>
-          <t>7.2%</t>
+          <t>6.7%</t>
         </is>
       </c>
       <c r="R49" s="7" t="inlineStr">
         <is>
-          <t>5.6%</t>
+          <t>5.2%</t>
         </is>
       </c>
     </row>
@@ -5007,47 +5007,47 @@
       </c>
       <c r="J50" s="7" t="inlineStr">
         <is>
-          <t>6.17</t>
+          <t>6.32</t>
         </is>
       </c>
       <c r="K50" s="7" t="inlineStr">
         <is>
-          <t>3.87</t>
+          <t>3.85</t>
         </is>
       </c>
       <c r="L50" s="7" t="inlineStr">
         <is>
-          <t>1.52</t>
+          <t>1.55</t>
         </is>
       </c>
       <c r="M50" s="7" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>14.9%</t>
         </is>
       </c>
       <c r="N50" s="7" t="inlineStr">
         <is>
-          <t>24.0%</t>
+          <t>24.4%</t>
         </is>
       </c>
       <c r="O50" s="7" t="inlineStr">
         <is>
-          <t>61.0%</t>
+          <t>60.7%</t>
         </is>
       </c>
       <c r="P50" s="7" t="inlineStr">
         <is>
-          <t>19.8%</t>
+          <t>20.3%</t>
         </is>
       </c>
       <c r="Q50" s="7" t="inlineStr">
         <is>
-          <t>18.9%</t>
+          <t>18.8%</t>
         </is>
       </c>
       <c r="R50" s="7" t="inlineStr">
         <is>
-          <t>61.3%</t>
+          <t>60.9%</t>
         </is>
       </c>
     </row>
@@ -5087,12 +5087,12 @@
       </c>
       <c r="H51" s="10" t="inlineStr">
         <is>
-          <t>2-0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="I51" s="10" t="inlineStr">
         <is>
-          <t>2-0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J51" s="7" t="inlineStr">
@@ -5102,42 +5102,42 @@
       </c>
       <c r="K51" s="7" t="inlineStr">
         <is>
-          <t>4.16</t>
+          <t>4.17</t>
         </is>
       </c>
       <c r="L51" s="7" t="inlineStr">
         <is>
-          <t>7.08</t>
+          <t>7.34</t>
         </is>
       </c>
       <c r="M51" s="7" t="inlineStr">
         <is>
-          <t>64.4%</t>
+          <t>64.7%</t>
         </is>
       </c>
       <c r="N51" s="7" t="inlineStr">
         <is>
-          <t>22.4%</t>
+          <t>22.5%</t>
         </is>
       </c>
       <c r="O51" s="7" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>12.8%</t>
         </is>
       </c>
       <c r="P51" s="7" t="inlineStr">
         <is>
-          <t>79.4%</t>
+          <t>80.7%</t>
         </is>
       </c>
       <c r="Q51" s="7" t="inlineStr">
         <is>
+          <t>9.8%</t>
+        </is>
+      </c>
+      <c r="R51" s="7" t="inlineStr">
+        <is>
           <t>9.6%</t>
-        </is>
-      </c>
-      <c r="R51" s="7" t="inlineStr">
-        <is>
-          <t>11.1%</t>
         </is>
       </c>
     </row>
@@ -5162,12 +5162,12 @@
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>Bosnia and Herzegovina</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="F52" s="8" t="inlineStr">
         <is>
-          <t>Qatar</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="G52" s="8" t="inlineStr">
@@ -5187,47 +5187,47 @@
       </c>
       <c r="J52" s="7" t="inlineStr">
         <is>
-          <t>1.55</t>
+          <t>2.12</t>
         </is>
       </c>
       <c r="K52" s="7" t="inlineStr">
         <is>
-          <t>3.80</t>
+          <t>3.30</t>
         </is>
       </c>
       <c r="L52" s="7" t="inlineStr">
         <is>
-          <t>6.08</t>
+          <t>3.47</t>
         </is>
       </c>
       <c r="M52" s="7" t="inlineStr">
         <is>
-          <t>60.1%</t>
+          <t>44.4%</t>
         </is>
       </c>
       <c r="N52" s="7" t="inlineStr">
         <is>
-          <t>24.5%</t>
+          <t>28.5%</t>
         </is>
       </c>
       <c r="O52" s="7" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>27.1%</t>
         </is>
       </c>
       <c r="P52" s="7" t="inlineStr">
         <is>
-          <t>53.4%</t>
+          <t>58.1%</t>
         </is>
       </c>
       <c r="Q52" s="7" t="inlineStr">
         <is>
-          <t>18.0%</t>
+          <t>13.4%</t>
         </is>
       </c>
       <c r="R52" s="7" t="inlineStr">
         <is>
-          <t>28.6%</t>
+          <t>28.5%</t>
         </is>
       </c>
     </row>
@@ -5252,12 +5252,12 @@
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>Bosnia and Herzegovina</t>
         </is>
       </c>
       <c r="F53" s="8" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Qatar</t>
         </is>
       </c>
       <c r="G53" s="8" t="inlineStr">
@@ -5267,57 +5267,57 @@
       </c>
       <c r="H53" s="10" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="I53" s="10" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>2-0</t>
         </is>
       </c>
       <c r="J53" s="7" t="inlineStr">
         <is>
-          <t>2.08</t>
+          <t>1.63</t>
         </is>
       </c>
       <c r="K53" s="7" t="inlineStr">
         <is>
-          <t>3.28</t>
+          <t>3.67</t>
         </is>
       </c>
       <c r="L53" s="7" t="inlineStr">
         <is>
-          <t>3.42</t>
+          <t>5.55</t>
         </is>
       </c>
       <c r="M53" s="7" t="inlineStr">
         <is>
-          <t>44.6%</t>
+          <t>57.5%</t>
         </is>
       </c>
       <c r="N53" s="7" t="inlineStr">
         <is>
-          <t>28.3%</t>
+          <t>25.6%</t>
         </is>
       </c>
       <c r="O53" s="7" t="inlineStr">
         <is>
-          <t>27.1%</t>
+          <t>16.9%</t>
         </is>
       </c>
       <c r="P53" s="7" t="inlineStr">
         <is>
-          <t>45.9%</t>
+          <t>39.1%</t>
         </is>
       </c>
       <c r="Q53" s="7" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>16.7%</t>
         </is>
       </c>
       <c r="R53" s="7" t="inlineStr">
         <is>
-          <t>39.6%</t>
+          <t>44.2%</t>
         </is>
       </c>
     </row>
@@ -5367,12 +5367,12 @@
       </c>
       <c r="J54" s="7" t="inlineStr">
         <is>
-          <t>6.33</t>
+          <t>6.52</t>
         </is>
       </c>
       <c r="K54" s="7" t="inlineStr">
         <is>
-          <t>4.50</t>
+          <t>4.72</t>
         </is>
       </c>
       <c r="L54" s="7" t="inlineStr">
@@ -5382,32 +5382,32 @@
       </c>
       <c r="M54" s="7" t="inlineStr">
         <is>
-          <t>14.7%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="N54" s="7" t="inlineStr">
         <is>
-          <t>20.7%</t>
+          <t>20.0%</t>
         </is>
       </c>
       <c r="O54" s="7" t="inlineStr">
         <is>
-          <t>64.6%</t>
+          <t>65.5%</t>
         </is>
       </c>
       <c r="P54" s="7" t="inlineStr">
         <is>
-          <t>13.3%</t>
+          <t>13.8%</t>
         </is>
       </c>
       <c r="Q54" s="7" t="inlineStr">
         <is>
-          <t>13.3%</t>
+          <t>13.7%</t>
         </is>
       </c>
       <c r="R54" s="7" t="inlineStr">
         <is>
-          <t>73.4%</t>
+          <t>72.5%</t>
         </is>
       </c>
     </row>
@@ -5462,17 +5462,17 @@
       </c>
       <c r="K55" s="7" t="inlineStr">
         <is>
-          <t>5.03</t>
+          <t>5.06</t>
         </is>
       </c>
       <c r="L55" s="7" t="inlineStr">
         <is>
-          <t>8.67</t>
+          <t>9.43</t>
         </is>
       </c>
       <c r="M55" s="7" t="inlineStr">
         <is>
-          <t>70.7%</t>
+          <t>71.4%</t>
         </is>
       </c>
       <c r="N55" s="7" t="inlineStr">
@@ -5482,22 +5482,22 @@
       </c>
       <c r="O55" s="7" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>10.0%</t>
         </is>
       </c>
       <c r="P55" s="7" t="inlineStr">
         <is>
-          <t>79.3%</t>
+          <t>80.7%</t>
         </is>
       </c>
       <c r="Q55" s="7" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>9.9%</t>
         </is>
       </c>
       <c r="R55" s="7" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.4%</t>
         </is>
       </c>
     </row>
@@ -5547,22 +5547,22 @@
       </c>
       <c r="J56" s="7" t="inlineStr">
         <is>
-          <t>4.33</t>
+          <t>4.40</t>
         </is>
       </c>
       <c r="K56" s="7" t="inlineStr">
         <is>
-          <t>3.45</t>
+          <t>3.48</t>
         </is>
       </c>
       <c r="L56" s="7" t="inlineStr">
         <is>
-          <t>1.81</t>
+          <t>1.82</t>
         </is>
       </c>
       <c r="M56" s="7" t="inlineStr">
         <is>
-          <t>21.5%</t>
+          <t>21.4%</t>
         </is>
       </c>
       <c r="N56" s="7" t="inlineStr">
@@ -5572,22 +5572,22 @@
       </c>
       <c r="O56" s="7" t="inlineStr">
         <is>
-          <t>51.5%</t>
+          <t>51.6%</t>
         </is>
       </c>
       <c r="P56" s="7" t="inlineStr">
         <is>
-          <t>28.0%</t>
+          <t>25.4%</t>
         </is>
       </c>
       <c r="Q56" s="7" t="inlineStr">
         <is>
-          <t>17.0%</t>
+          <t>15.7%</t>
         </is>
       </c>
       <c r="R56" s="7" t="inlineStr">
         <is>
-          <t>55.1%</t>
+          <t>58.9%</t>
         </is>
       </c>
     </row>
@@ -5637,47 +5637,47 @@
       </c>
       <c r="J57" s="7" t="inlineStr">
         <is>
-          <t>3.83</t>
+          <t>5.50</t>
         </is>
       </c>
       <c r="K57" s="7" t="inlineStr">
         <is>
-          <t>3.37</t>
+          <t>3.88</t>
         </is>
       </c>
       <c r="L57" s="7" t="inlineStr">
         <is>
-          <t>1.92</t>
+          <t>1.60</t>
         </is>
       </c>
       <c r="M57" s="7" t="inlineStr">
         <is>
+          <t>17.1%</t>
+        </is>
+      </c>
+      <c r="N57" s="7" t="inlineStr">
+        <is>
           <t>24.2%</t>
         </is>
       </c>
-      <c r="N57" s="7" t="inlineStr">
-        <is>
-          <t>27.5%</t>
-        </is>
-      </c>
       <c r="O57" s="7" t="inlineStr">
         <is>
-          <t>48.3%</t>
+          <t>58.7%</t>
         </is>
       </c>
       <c r="P57" s="7" t="inlineStr">
         <is>
-          <t>19.4%</t>
+          <t>18.5%</t>
         </is>
       </c>
       <c r="Q57" s="7" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>15.6%</t>
         </is>
       </c>
       <c r="R57" s="7" t="inlineStr">
         <is>
-          <t>66.1%</t>
+          <t>65.9%</t>
         </is>
       </c>
     </row>
@@ -5727,12 +5727,12 @@
       </c>
       <c r="J58" s="7" t="inlineStr">
         <is>
-          <t>12.83</t>
+          <t>12.68</t>
         </is>
       </c>
       <c r="K58" s="7" t="inlineStr">
         <is>
-          <t>6.17</t>
+          <t>6.36</t>
         </is>
       </c>
       <c r="L58" s="7" t="inlineStr">
@@ -5742,32 +5742,32 @@
       </c>
       <c r="M58" s="7" t="inlineStr">
         <is>
-          <t>7.3%</t>
+          <t>7.4%</t>
         </is>
       </c>
       <c r="N58" s="7" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>14.8%</t>
         </is>
       </c>
       <c r="O58" s="7" t="inlineStr">
         <is>
-          <t>77.5%</t>
+          <t>77.8%</t>
         </is>
       </c>
       <c r="P58" s="7" t="inlineStr">
         <is>
-          <t>22.4%</t>
+          <t>22.2%</t>
         </is>
       </c>
       <c r="Q58" s="7" t="inlineStr">
         <is>
-          <t>18.4%</t>
+          <t>18.3%</t>
         </is>
       </c>
       <c r="R58" s="7" t="inlineStr">
         <is>
-          <t>59.3%</t>
+          <t>59.6%</t>
         </is>
       </c>
     </row>
@@ -5817,47 +5817,47 @@
       </c>
       <c r="J59" s="7" t="inlineStr">
         <is>
-          <t>4.77</t>
+          <t>4.64</t>
         </is>
       </c>
       <c r="K59" s="7" t="inlineStr">
         <is>
-          <t>3.70</t>
+          <t>3.71</t>
         </is>
       </c>
       <c r="L59" s="7" t="inlineStr">
         <is>
-          <t>1.68</t>
+          <t>1.73</t>
         </is>
       </c>
       <c r="M59" s="7" t="inlineStr">
         <is>
-          <t>19.5%</t>
+          <t>20.3%</t>
         </is>
       </c>
       <c r="N59" s="7" t="inlineStr">
         <is>
-          <t>25.1%</t>
+          <t>25.4%</t>
         </is>
       </c>
       <c r="O59" s="7" t="inlineStr">
         <is>
-          <t>55.4%</t>
+          <t>54.4%</t>
         </is>
       </c>
       <c r="P59" s="7" t="inlineStr">
         <is>
-          <t>34.0%</t>
+          <t>31.4%</t>
         </is>
       </c>
       <c r="Q59" s="7" t="inlineStr">
         <is>
-          <t>15.6%</t>
+          <t>19.1%</t>
         </is>
       </c>
       <c r="R59" s="7" t="inlineStr">
         <is>
-          <t>50.4%</t>
+          <t>49.4%</t>
         </is>
       </c>
     </row>
@@ -5907,17 +5907,17 @@
       </c>
       <c r="J60" s="7" t="inlineStr">
         <is>
-          <t>2.05</t>
+          <t>2.08</t>
         </is>
       </c>
       <c r="K60" s="7" t="inlineStr">
         <is>
-          <t>3.32</t>
+          <t>3.36</t>
         </is>
       </c>
       <c r="L60" s="7" t="inlineStr">
         <is>
-          <t>3.43</t>
+          <t>3.47</t>
         </is>
       </c>
       <c r="M60" s="7" t="inlineStr">
@@ -5937,17 +5937,17 @@
       </c>
       <c r="P60" s="7" t="inlineStr">
         <is>
-          <t>66.9%</t>
+          <t>67.4%</t>
         </is>
       </c>
       <c r="Q60" s="7" t="inlineStr">
         <is>
-          <t>11.3%</t>
+          <t>10.8%</t>
         </is>
       </c>
       <c r="R60" s="7" t="inlineStr">
         <is>
-          <t>21.9%</t>
+          <t>21.8%</t>
         </is>
       </c>
     </row>
@@ -5997,12 +5997,12 @@
       </c>
       <c r="J61" s="7" t="inlineStr">
         <is>
-          <t>6.08</t>
+          <t>6.36</t>
         </is>
       </c>
       <c r="K61" s="7" t="inlineStr">
         <is>
-          <t>4.13</t>
+          <t>4.21</t>
         </is>
       </c>
       <c r="L61" s="7" t="inlineStr">
@@ -6012,32 +6012,32 @@
       </c>
       <c r="M61" s="7" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>14.8%</t>
         </is>
       </c>
       <c r="N61" s="7" t="inlineStr">
         <is>
-          <t>22.6%</t>
+          <t>22.4%</t>
         </is>
       </c>
       <c r="O61" s="7" t="inlineStr">
         <is>
-          <t>62.1%</t>
+          <t>62.8%</t>
         </is>
       </c>
       <c r="P61" s="7" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="Q61" s="7" t="inlineStr">
         <is>
-          <t>13.7%</t>
+          <t>11.8%</t>
         </is>
       </c>
       <c r="R61" s="7" t="inlineStr">
         <is>
-          <t>71.0%</t>
+          <t>73.6%</t>
         </is>
       </c>
     </row>
@@ -6062,12 +6062,12 @@
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>Paraguay</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="F62" s="8" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="G62" s="8" t="inlineStr">
@@ -6087,47 +6087,47 @@
       </c>
       <c r="J62" s="7" t="inlineStr">
         <is>
-          <t>2.13</t>
+          <t>2.57</t>
         </is>
       </c>
       <c r="K62" s="7" t="inlineStr">
         <is>
-          <t>3.17</t>
+          <t>3.48</t>
         </is>
       </c>
       <c r="L62" s="7" t="inlineStr">
         <is>
-          <t>3.40</t>
+          <t>2.59</t>
         </is>
       </c>
       <c r="M62" s="7" t="inlineStr">
         <is>
-          <t>43.5%</t>
+          <t>36.6%</t>
         </is>
       </c>
       <c r="N62" s="7" t="inlineStr">
         <is>
-          <t>29.2%</t>
+          <t>27.0%</t>
         </is>
       </c>
       <c r="O62" s="7" t="inlineStr">
         <is>
-          <t>27.3%</t>
+          <t>36.3%</t>
         </is>
       </c>
       <c r="P62" s="7" t="inlineStr">
         <is>
-          <t>59.0%</t>
+          <t>64.0%</t>
         </is>
       </c>
       <c r="Q62" s="7" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>12.9%</t>
         </is>
       </c>
       <c r="R62" s="7" t="inlineStr">
         <is>
-          <t>24.2%</t>
+          <t>23.1%</t>
         </is>
       </c>
     </row>
@@ -6152,12 +6152,12 @@
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>Paraguay</t>
         </is>
       </c>
       <c r="F63" s="8" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="G63" s="8" t="inlineStr">
@@ -6167,57 +6167,57 @@
       </c>
       <c r="H63" s="10" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="I63" s="10" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="J63" s="7" t="inlineStr">
         <is>
-          <t>2.62</t>
+          <t>2.15</t>
         </is>
       </c>
       <c r="K63" s="7" t="inlineStr">
         <is>
-          <t>3.42</t>
+          <t>3.19</t>
         </is>
       </c>
       <c r="L63" s="7" t="inlineStr">
         <is>
-          <t>2.50</t>
+          <t>3.53</t>
         </is>
       </c>
       <c r="M63" s="7" t="inlineStr">
         <is>
-          <t>35.5%</t>
+          <t>43.8%</t>
         </is>
       </c>
       <c r="N63" s="7" t="inlineStr">
         <is>
-          <t>27.2%</t>
+          <t>29.5%</t>
         </is>
       </c>
       <c r="O63" s="7" t="inlineStr">
         <is>
-          <t>37.2%</t>
+          <t>26.7%</t>
         </is>
       </c>
       <c r="P63" s="7" t="inlineStr">
         <is>
-          <t>55.7%</t>
+          <t>37.6%</t>
         </is>
       </c>
       <c r="Q63" s="7" t="inlineStr">
         <is>
-          <t>14.2%</t>
+          <t>19.6%</t>
         </is>
       </c>
       <c r="R63" s="7" t="inlineStr">
         <is>
-          <t>30.1%</t>
+          <t>42.8%</t>
         </is>
       </c>
     </row>
@@ -6267,22 +6267,22 @@
       </c>
       <c r="J64" s="7" t="inlineStr">
         <is>
-          <t>4.23</t>
+          <t>4.29</t>
         </is>
       </c>
       <c r="K64" s="7" t="inlineStr">
         <is>
-          <t>3.50</t>
+          <t>3.56</t>
         </is>
       </c>
       <c r="L64" s="7" t="inlineStr">
         <is>
-          <t>1.80</t>
+          <t>1.83</t>
         </is>
       </c>
       <c r="M64" s="7" t="inlineStr">
         <is>
-          <t>21.9%</t>
+          <t>22.0%</t>
         </is>
       </c>
       <c r="N64" s="7" t="inlineStr">
@@ -6292,22 +6292,22 @@
       </c>
       <c r="O64" s="7" t="inlineStr">
         <is>
-          <t>51.6%</t>
+          <t>51.5%</t>
         </is>
       </c>
       <c r="P64" s="7" t="inlineStr">
         <is>
-          <t>19.4%</t>
+          <t>18.3%</t>
         </is>
       </c>
       <c r="Q64" s="7" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>12.6%</t>
         </is>
       </c>
       <c r="R64" s="7" t="inlineStr">
         <is>
-          <t>67.9%</t>
+          <t>69.1%</t>
         </is>
       </c>
     </row>
@@ -6357,47 +6357,47 @@
       </c>
       <c r="J65" s="7" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>1.40</t>
         </is>
       </c>
       <c r="K65" s="7" t="inlineStr">
         <is>
-          <t>4.40</t>
+          <t>4.55</t>
         </is>
       </c>
       <c r="L65" s="7" t="inlineStr">
         <is>
-          <t>7.08</t>
+          <t>7.86</t>
         </is>
       </c>
       <c r="M65" s="7" t="inlineStr">
         <is>
-          <t>65.6%</t>
+          <t>67.3%</t>
         </is>
       </c>
       <c r="N65" s="7" t="inlineStr">
         <is>
-          <t>21.2%</t>
+          <t>20.7%</t>
         </is>
       </c>
       <c r="O65" s="7" t="inlineStr">
         <is>
+          <t>12.0%</t>
+        </is>
+      </c>
+      <c r="P65" s="7" t="inlineStr">
+        <is>
+          <t>66.4%</t>
+        </is>
+      </c>
+      <c r="Q65" s="7" t="inlineStr">
+        <is>
           <t>13.2%</t>
         </is>
       </c>
-      <c r="P65" s="7" t="inlineStr">
-        <is>
-          <t>68.2%</t>
-        </is>
-      </c>
-      <c r="Q65" s="7" t="inlineStr">
-        <is>
-          <t>11.7%</t>
-        </is>
-      </c>
       <c r="R65" s="7" t="inlineStr">
         <is>
-          <t>20.1%</t>
+          <t>20.4%</t>
         </is>
       </c>
     </row>
@@ -6447,47 +6447,47 @@
       </c>
       <c r="J66" s="7" t="inlineStr">
         <is>
-          <t>2.52</t>
+          <t>2.40</t>
         </is>
       </c>
       <c r="K66" s="7" t="inlineStr">
         <is>
-          <t>3.25</t>
+          <t>3.36</t>
         </is>
       </c>
       <c r="L66" s="7" t="inlineStr">
         <is>
-          <t>2.69</t>
+          <t>2.88</t>
         </is>
       </c>
       <c r="M66" s="7" t="inlineStr">
         <is>
-          <t>36.9%</t>
+          <t>39.3%</t>
         </is>
       </c>
       <c r="N66" s="7" t="inlineStr">
         <is>
-          <t>28.6%</t>
+          <t>28.0%</t>
         </is>
       </c>
       <c r="O66" s="7" t="inlineStr">
         <is>
-          <t>34.5%</t>
+          <t>32.7%</t>
         </is>
       </c>
       <c r="P66" s="7" t="inlineStr">
         <is>
-          <t>26.3%</t>
+          <t>26.4%</t>
         </is>
       </c>
       <c r="Q66" s="7" t="inlineStr">
         <is>
-          <t>20.1%</t>
+          <t>19.0%</t>
         </is>
       </c>
       <c r="R66" s="7" t="inlineStr">
         <is>
-          <t>53.6%</t>
+          <t>54.6%</t>
         </is>
       </c>
     </row>
@@ -6537,17 +6537,17 @@
       </c>
       <c r="J67" s="7" t="inlineStr">
         <is>
-          <t>5.08</t>
+          <t>5.15</t>
         </is>
       </c>
       <c r="K67" s="7" t="inlineStr">
         <is>
-          <t>3.87</t>
+          <t>3.92</t>
         </is>
       </c>
       <c r="L67" s="7" t="inlineStr">
         <is>
-          <t>1.61</t>
+          <t>1.63</t>
         </is>
       </c>
       <c r="M67" s="7" t="inlineStr">
@@ -6567,17 +6567,17 @@
       </c>
       <c r="P67" s="7" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>15.1%</t>
         </is>
       </c>
       <c r="Q67" s="7" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>16.4%</t>
         </is>
       </c>
       <c r="R67" s="7" t="inlineStr">
         <is>
-          <t>68.2%</t>
+          <t>68.5%</t>
         </is>
       </c>
     </row>
@@ -6600,14 +6600,14 @@
           <t>G</t>
         </is>
       </c>
-      <c r="E68" s="8" t="inlineStr">
-        <is>
-          <t>New Zealand</t>
-        </is>
-      </c>
-      <c r="F68" s="9" t="inlineStr">
-        <is>
-          <t>Belgium</t>
+      <c r="E68" s="9" t="inlineStr">
+        <is>
+          <t>Egypt</t>
+        </is>
+      </c>
+      <c r="F68" s="8" t="inlineStr">
+        <is>
+          <t>Iran</t>
         </is>
       </c>
       <c r="G68" s="8" t="inlineStr">
@@ -6617,57 +6617,57 @@
       </c>
       <c r="H68" s="10" t="inlineStr">
         <is>
-          <t>0-2</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="I68" s="10" t="inlineStr">
         <is>
-          <t>0-2</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="J68" s="7" t="inlineStr">
         <is>
-          <t>8.83</t>
+          <t>2.23</t>
         </is>
       </c>
       <c r="K68" s="7" t="inlineStr">
         <is>
-          <t>5.58</t>
+          <t>2.99</t>
         </is>
       </c>
       <c r="L68" s="7" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t>3.56</t>
         </is>
       </c>
       <c r="M68" s="7" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>42.2%</t>
         </is>
       </c>
       <c r="N68" s="7" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>31.4%</t>
         </is>
       </c>
       <c r="O68" s="7" t="inlineStr">
         <is>
-          <t>72.6%</t>
+          <t>26.4%</t>
         </is>
       </c>
       <c r="P68" s="7" t="inlineStr">
         <is>
-          <t>13.4%</t>
+          <t>30.0%</t>
         </is>
       </c>
       <c r="Q68" s="7" t="inlineStr">
         <is>
-          <t>9.4%</t>
+          <t>17.6%</t>
         </is>
       </c>
       <c r="R68" s="7" t="inlineStr">
         <is>
-          <t>77.2%</t>
+          <t>52.4%</t>
         </is>
       </c>
     </row>
@@ -6690,14 +6690,14 @@
           <t>G</t>
         </is>
       </c>
-      <c r="E69" s="9" t="inlineStr">
-        <is>
-          <t>Egypt</t>
-        </is>
-      </c>
-      <c r="F69" s="8" t="inlineStr">
-        <is>
-          <t>Iran</t>
+      <c r="E69" s="8" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="F69" s="9" t="inlineStr">
+        <is>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="G69" s="8" t="inlineStr">
@@ -6707,57 +6707,57 @@
       </c>
       <c r="H69" s="10" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>0-2</t>
         </is>
       </c>
       <c r="I69" s="10" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>0-2</t>
         </is>
       </c>
       <c r="J69" s="7" t="inlineStr">
         <is>
-          <t>2.23</t>
+          <t>9.91</t>
         </is>
       </c>
       <c r="K69" s="7" t="inlineStr">
         <is>
-          <t>2.94</t>
+          <t>5.69</t>
         </is>
       </c>
       <c r="L69" s="7" t="inlineStr">
         <is>
-          <t>3.48</t>
+          <t>1.28</t>
         </is>
       </c>
       <c r="M69" s="7" t="inlineStr">
         <is>
-          <t>41.7%</t>
+          <t>9.5%</t>
         </is>
       </c>
       <c r="N69" s="7" t="inlineStr">
         <is>
-          <t>31.6%</t>
+          <t>16.6%</t>
         </is>
       </c>
       <c r="O69" s="7" t="inlineStr">
         <is>
-          <t>26.7%</t>
+          <t>73.8%</t>
         </is>
       </c>
       <c r="P69" s="7" t="inlineStr">
         <is>
-          <t>29.6%</t>
+          <t>12.1%</t>
         </is>
       </c>
       <c r="Q69" s="7" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>11.5%</t>
         </is>
       </c>
       <c r="R69" s="7" t="inlineStr">
         <is>
-          <t>53.6%</t>
+          <t>76.4%</t>
         </is>
       </c>
     </row>
@@ -6780,14 +6780,14 @@
           <t>L</t>
         </is>
       </c>
-      <c r="E70" s="9" t="inlineStr">
-        <is>
-          <t>Croatia</t>
-        </is>
-      </c>
-      <c r="F70" s="8" t="inlineStr">
-        <is>
-          <t>Ghana</t>
+      <c r="E70" s="8" t="inlineStr">
+        <is>
+          <t>Panama</t>
+        </is>
+      </c>
+      <c r="F70" s="9" t="inlineStr">
+        <is>
+          <t>England</t>
         </is>
       </c>
       <c r="G70" s="8" t="inlineStr">
@@ -6797,57 +6797,57 @@
       </c>
       <c r="H70" s="10" t="inlineStr">
         <is>
-          <t>2-0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="I70" s="10" t="inlineStr">
         <is>
-          <t>2-0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J70" s="7" t="inlineStr">
         <is>
-          <t>1.64</t>
+          <t>9.30</t>
         </is>
       </c>
       <c r="K70" s="7" t="inlineStr">
         <is>
-          <t>3.65</t>
+          <t>6.05</t>
         </is>
       </c>
       <c r="L70" s="7" t="inlineStr">
         <is>
-          <t>5.12</t>
+          <t>1.28</t>
         </is>
       </c>
       <c r="M70" s="7" t="inlineStr">
         <is>
-          <t>56.5%</t>
+          <t>10.2%</t>
         </is>
       </c>
       <c r="N70" s="7" t="inlineStr">
         <is>
-          <t>25.4%</t>
+          <t>15.7%</t>
         </is>
       </c>
       <c r="O70" s="7" t="inlineStr">
         <is>
-          <t>18.1%</t>
+          <t>74.1%</t>
         </is>
       </c>
       <c r="P70" s="7" t="inlineStr">
         <is>
-          <t>80.6%</t>
+          <t>11.6%</t>
         </is>
       </c>
       <c r="Q70" s="7" t="inlineStr">
         <is>
-          <t>10.3%</t>
+          <t>17.9%</t>
         </is>
       </c>
       <c r="R70" s="7" t="inlineStr">
         <is>
-          <t>9.0%</t>
+          <t>70.6%</t>
         </is>
       </c>
     </row>
@@ -6870,14 +6870,14 @@
           <t>L</t>
         </is>
       </c>
-      <c r="E71" s="8" t="inlineStr">
-        <is>
-          <t>Panama</t>
-        </is>
-      </c>
-      <c r="F71" s="9" t="inlineStr">
-        <is>
-          <t>England</t>
+      <c r="E71" s="9" t="inlineStr">
+        <is>
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="F71" s="8" t="inlineStr">
+        <is>
+          <t>Ghana</t>
         </is>
       </c>
       <c r="G71" s="8" t="inlineStr">
@@ -6887,57 +6887,57 @@
       </c>
       <c r="H71" s="10" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>2-0</t>
         </is>
       </c>
       <c r="I71" s="10" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>2-0</t>
         </is>
       </c>
       <c r="J71" s="7" t="inlineStr">
         <is>
-          <t>8.50</t>
+          <t>1.63</t>
         </is>
       </c>
       <c r="K71" s="7" t="inlineStr">
         <is>
-          <t>5.83</t>
+          <t>3.75</t>
         </is>
       </c>
       <c r="L71" s="7" t="inlineStr">
         <is>
-          <t>1.27</t>
+          <t>5.43</t>
         </is>
       </c>
       <c r="M71" s="7" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>57.6%</t>
         </is>
       </c>
       <c r="N71" s="7" t="inlineStr">
         <is>
-          <t>15.9%</t>
+          <t>25.1%</t>
         </is>
       </c>
       <c r="O71" s="7" t="inlineStr">
         <is>
-          <t>73.1%</t>
+          <t>17.3%</t>
         </is>
       </c>
       <c r="P71" s="7" t="inlineStr">
         <is>
-          <t>12.1%</t>
+          <t>79.3%</t>
         </is>
       </c>
       <c r="Q71" s="7" t="inlineStr">
         <is>
-          <t>17.0%</t>
+          <t>11.1%</t>
         </is>
       </c>
       <c r="R71" s="7" t="inlineStr">
         <is>
-          <t>70.9%</t>
+          <t>9.6%</t>
         </is>
       </c>
     </row>
@@ -6987,22 +6987,22 @@
       </c>
       <c r="J72" s="7" t="inlineStr">
         <is>
-          <t>3.37</t>
+          <t>3.48</t>
         </is>
       </c>
       <c r="K72" s="7" t="inlineStr">
         <is>
-          <t>3.23</t>
+          <t>3.28</t>
         </is>
       </c>
       <c r="L72" s="7" t="inlineStr">
         <is>
-          <t>2.12</t>
+          <t>2.13</t>
         </is>
       </c>
       <c r="M72" s="7" t="inlineStr">
         <is>
-          <t>27.5%</t>
+          <t>27.1%</t>
         </is>
       </c>
       <c r="N72" s="7" t="inlineStr">
@@ -7012,22 +7012,22 @@
       </c>
       <c r="O72" s="7" t="inlineStr">
         <is>
-          <t>43.8%</t>
+          <t>44.2%</t>
         </is>
       </c>
       <c r="P72" s="7" t="inlineStr">
         <is>
-          <t>41.2%</t>
+          <t>36.6%</t>
         </is>
       </c>
       <c r="Q72" s="7" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>17.9%</t>
         </is>
       </c>
       <c r="R72" s="7" t="inlineStr">
         <is>
-          <t>43.5%</t>
+          <t>45.5%</t>
         </is>
       </c>
     </row>
@@ -7082,42 +7082,42 @@
       </c>
       <c r="K73" s="7" t="inlineStr">
         <is>
-          <t>3.25</t>
+          <t>3.31</t>
         </is>
       </c>
       <c r="L73" s="7" t="inlineStr">
         <is>
-          <t>2.98</t>
+          <t>3.06</t>
         </is>
       </c>
       <c r="M73" s="7" t="inlineStr">
         <is>
-          <t>40.3%</t>
+          <t>40.9%</t>
         </is>
       </c>
       <c r="N73" s="7" t="inlineStr">
         <is>
-          <t>28.5%</t>
+          <t>28.4%</t>
         </is>
       </c>
       <c r="O73" s="7" t="inlineStr">
         <is>
-          <t>31.1%</t>
+          <t>30.7%</t>
         </is>
       </c>
       <c r="P73" s="7" t="inlineStr">
         <is>
-          <t>32.4%</t>
+          <t>33.2%</t>
         </is>
       </c>
       <c r="Q73" s="7" t="inlineStr">
         <is>
-          <t>15.9%</t>
+          <t>17.1%</t>
         </is>
       </c>
       <c r="R73" s="7" t="inlineStr">
         <is>
-          <t>51.6%</t>
+          <t>49.6%</t>
         </is>
       </c>
     </row>
@@ -7167,47 +7167,47 @@
       </c>
       <c r="J74" s="7" t="inlineStr">
         <is>
-          <t>3.50</t>
+          <t>3.66</t>
         </is>
       </c>
       <c r="K74" s="7" t="inlineStr">
         <is>
-          <t>3.13</t>
+          <t>3.09</t>
         </is>
       </c>
       <c r="L74" s="7" t="inlineStr">
         <is>
-          <t>2.12</t>
+          <t>2.16</t>
         </is>
       </c>
       <c r="M74" s="7" t="inlineStr">
         <is>
-          <t>26.5%</t>
+          <t>25.8%</t>
         </is>
       </c>
       <c r="N74" s="7" t="inlineStr">
         <is>
-          <t>29.7%</t>
+          <t>30.5%</t>
         </is>
       </c>
       <c r="O74" s="7" t="inlineStr">
         <is>
-          <t>43.8%</t>
+          <t>43.7%</t>
         </is>
       </c>
       <c r="P74" s="7" t="inlineStr">
         <is>
-          <t>35.8%</t>
+          <t>35.9%</t>
         </is>
       </c>
       <c r="Q74" s="7" t="inlineStr">
         <is>
-          <t>18.1%</t>
+          <t>19.9%</t>
         </is>
       </c>
       <c r="R74" s="7" t="inlineStr">
         <is>
-          <t>46.1%</t>
+          <t>44.2%</t>
         </is>
       </c>
     </row>
@@ -7257,42 +7257,42 @@
       </c>
       <c r="J75" s="7" t="inlineStr">
         <is>
-          <t>13.00</t>
+          <t>14.37</t>
         </is>
       </c>
       <c r="K75" s="7" t="inlineStr">
         <is>
-          <t>6.67</t>
+          <t>7.04</t>
         </is>
       </c>
       <c r="L75" s="7" t="inlineStr">
         <is>
-          <t>1.19</t>
+          <t>1.18</t>
         </is>
       </c>
       <c r="M75" s="7" t="inlineStr">
         <is>
-          <t>7.2%</t>
+          <t>6.6%</t>
         </is>
       </c>
       <c r="N75" s="7" t="inlineStr">
         <is>
-          <t>14.0%</t>
+          <t>13.4%</t>
         </is>
       </c>
       <c r="O75" s="7" t="inlineStr">
         <is>
-          <t>78.7%</t>
+          <t>80.0%</t>
         </is>
       </c>
       <c r="P75" s="7" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>10.4%</t>
         </is>
       </c>
       <c r="Q75" s="7" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>11.4%</t>
         </is>
       </c>
       <c r="R75" s="7" t="inlineStr">
@@ -7373,7 +7373,7 @@
       </c>
       <c r="P76" s="11" t="inlineStr">
         <is>
-          <t>41.5%</t>
+          <t>46.0%</t>
         </is>
       </c>
       <c r="Q76" s="11" t="inlineStr">
@@ -7383,7 +7383,7 @@
       </c>
       <c r="R76" s="11" t="inlineStr">
         <is>
-          <t>58.5%</t>
+          <t>54.0%</t>
         </is>
       </c>
     </row>
@@ -7459,7 +7459,7 @@
       </c>
       <c r="P77" s="11" t="inlineStr">
         <is>
-          <t>64.4%</t>
+          <t>64.7%</t>
         </is>
       </c>
       <c r="Q77" s="11" t="inlineStr">
@@ -7469,7 +7469,7 @@
       </c>
       <c r="R77" s="11" t="inlineStr">
         <is>
-          <t>35.6%</t>
+          <t>35.3%</t>
         </is>
       </c>
     </row>
@@ -7545,7 +7545,7 @@
       </c>
       <c r="P78" s="11" t="inlineStr">
         <is>
-          <t>68.8%</t>
+          <t>69.3%</t>
         </is>
       </c>
       <c r="Q78" s="11" t="inlineStr">
@@ -7555,7 +7555,7 @@
       </c>
       <c r="R78" s="11" t="inlineStr">
         <is>
-          <t>31.2%</t>
+          <t>30.7%</t>
         </is>
       </c>
     </row>
@@ -7631,7 +7631,7 @@
       </c>
       <c r="P79" s="11" t="inlineStr">
         <is>
-          <t>67.2%</t>
+          <t>67.3%</t>
         </is>
       </c>
       <c r="Q79" s="11" t="inlineStr">
@@ -7641,7 +7641,7 @@
       </c>
       <c r="R79" s="11" t="inlineStr">
         <is>
-          <t>32.8%</t>
+          <t>32.7%</t>
         </is>
       </c>
     </row>
@@ -7717,7 +7717,7 @@
       </c>
       <c r="P80" s="11" t="inlineStr">
         <is>
-          <t>55.2%</t>
+          <t>55.4%</t>
         </is>
       </c>
       <c r="Q80" s="11" t="inlineStr">
@@ -7727,7 +7727,7 @@
       </c>
       <c r="R80" s="11" t="inlineStr">
         <is>
-          <t>44.8%</t>
+          <t>44.6%</t>
         </is>
       </c>
     </row>
@@ -7803,7 +7803,7 @@
       </c>
       <c r="P81" s="11" t="inlineStr">
         <is>
-          <t>84.9%</t>
+          <t>85.0%</t>
         </is>
       </c>
       <c r="Q81" s="11" t="inlineStr">
@@ -7813,7 +7813,7 @@
       </c>
       <c r="R81" s="11" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>15.0%</t>
         </is>
       </c>
     </row>
@@ -7889,7 +7889,7 @@
       </c>
       <c r="P82" s="11" t="inlineStr">
         <is>
-          <t>61.4%</t>
+          <t>63.1%</t>
         </is>
       </c>
       <c r="Q82" s="11" t="inlineStr">
@@ -7899,7 +7899,7 @@
       </c>
       <c r="R82" s="11" t="inlineStr">
         <is>
-          <t>38.6%</t>
+          <t>36.9%</t>
         </is>
       </c>
     </row>
@@ -7975,7 +7975,7 @@
       </c>
       <c r="P83" s="11" t="inlineStr">
         <is>
-          <t>87.4%</t>
+          <t>87.6%</t>
         </is>
       </c>
       <c r="Q83" s="11" t="inlineStr">
@@ -7985,7 +7985,7 @@
       </c>
       <c r="R83" s="11" t="inlineStr">
         <is>
-          <t>12.6%</t>
+          <t>12.4%</t>
         </is>
       </c>
     </row>
@@ -8011,7 +8011,7 @@
       </c>
       <c r="F84" s="12" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>Algeria</t>
         </is>
       </c>
       <c r="G84" s="12" t="inlineStr">
@@ -8061,7 +8061,7 @@
       </c>
       <c r="P84" s="11" t="inlineStr">
         <is>
-          <t>73.2%</t>
+          <t>72.2%</t>
         </is>
       </c>
       <c r="Q84" s="11" t="inlineStr">
@@ -8071,7 +8071,7 @@
       </c>
       <c r="R84" s="11" t="inlineStr">
         <is>
-          <t>26.8%</t>
+          <t>27.8%</t>
         </is>
       </c>
     </row>
@@ -8097,7 +8097,7 @@
       </c>
       <c r="F85" s="12" t="inlineStr">
         <is>
-          <t>Algeria</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="G85" s="12" t="inlineStr">
@@ -8147,7 +8147,7 @@
       </c>
       <c r="P85" s="11" t="inlineStr">
         <is>
-          <t>71.2%</t>
+          <t>75.3%</t>
         </is>
       </c>
       <c r="Q85" s="11" t="inlineStr">
@@ -8157,7 +8157,7 @@
       </c>
       <c r="R85" s="11" t="inlineStr">
         <is>
-          <t>28.8%</t>
+          <t>24.7%</t>
         </is>
       </c>
     </row>
@@ -8233,7 +8233,7 @@
       </c>
       <c r="P86" s="11" t="inlineStr">
         <is>
-          <t>87.9%</t>
+          <t>88.1%</t>
         </is>
       </c>
       <c r="Q86" s="11" t="inlineStr">
@@ -8243,7 +8243,7 @@
       </c>
       <c r="R86" s="11" t="inlineStr">
         <is>
-          <t>12.1%</t>
+          <t>11.9%</t>
         </is>
       </c>
     </row>
@@ -8405,7 +8405,7 @@
       </c>
       <c r="P88" s="11" t="inlineStr">
         <is>
-          <t>71.8%</t>
+          <t>72.4%</t>
         </is>
       </c>
       <c r="Q88" s="11" t="inlineStr">
@@ -8415,7 +8415,7 @@
       </c>
       <c r="R88" s="11" t="inlineStr">
         <is>
-          <t>28.2%</t>
+          <t>27.6%</t>
         </is>
       </c>
     </row>
@@ -8491,7 +8491,7 @@
       </c>
       <c r="P89" s="11" t="inlineStr">
         <is>
-          <t>61.5%</t>
+          <t>60.7%</t>
         </is>
       </c>
       <c r="Q89" s="11" t="inlineStr">
@@ -8501,7 +8501,7 @@
       </c>
       <c r="R89" s="11" t="inlineStr">
         <is>
-          <t>38.5%</t>
+          <t>39.3%</t>
         </is>
       </c>
     </row>
@@ -8663,7 +8663,7 @@
       </c>
       <c r="P91" s="11" t="inlineStr">
         <is>
-          <t>89.8%</t>
+          <t>90.2%</t>
         </is>
       </c>
       <c r="Q91" s="11" t="inlineStr">
@@ -8673,7 +8673,7 @@
       </c>
       <c r="R91" s="11" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>9.8%</t>
         </is>
       </c>
     </row>
@@ -8749,7 +8749,7 @@
       </c>
       <c r="P92" s="15" t="inlineStr">
         <is>
-          <t>32.6%</t>
+          <t>32.0%</t>
         </is>
       </c>
       <c r="Q92" s="15" t="inlineStr">
@@ -8759,7 +8759,7 @@
       </c>
       <c r="R92" s="15" t="inlineStr">
         <is>
-          <t>67.4%</t>
+          <t>68.0%</t>
         </is>
       </c>
     </row>
@@ -8921,7 +8921,7 @@
       </c>
       <c r="P94" s="15" t="inlineStr">
         <is>
-          <t>34.4%</t>
+          <t>34.6%</t>
         </is>
       </c>
       <c r="Q94" s="15" t="inlineStr">
@@ -8931,7 +8931,7 @@
       </c>
       <c r="R94" s="15" t="inlineStr">
         <is>
-          <t>65.6%</t>
+          <t>65.4%</t>
         </is>
       </c>
     </row>
@@ -9007,7 +9007,7 @@
       </c>
       <c r="P95" s="15" t="inlineStr">
         <is>
-          <t>36.2%</t>
+          <t>37.7%</t>
         </is>
       </c>
       <c r="Q95" s="15" t="inlineStr">
@@ -9017,7 +9017,7 @@
       </c>
       <c r="R95" s="15" t="inlineStr">
         <is>
-          <t>63.8%</t>
+          <t>62.3%</t>
         </is>
       </c>
     </row>
@@ -9093,7 +9093,7 @@
       </c>
       <c r="P96" s="15" t="inlineStr">
         <is>
-          <t>75.6%</t>
+          <t>75.9%</t>
         </is>
       </c>
       <c r="Q96" s="15" t="inlineStr">
@@ -9103,7 +9103,7 @@
       </c>
       <c r="R96" s="15" t="inlineStr">
         <is>
-          <t>24.4%</t>
+          <t>24.1%</t>
         </is>
       </c>
     </row>
@@ -9179,7 +9179,7 @@
       </c>
       <c r="P97" s="15" t="inlineStr">
         <is>
-          <t>51.2%</t>
+          <t>50.8%</t>
         </is>
       </c>
       <c r="Q97" s="15" t="inlineStr">
@@ -9189,7 +9189,7 @@
       </c>
       <c r="R97" s="15" t="inlineStr">
         <is>
-          <t>48.8%</t>
+          <t>49.2%</t>
         </is>
       </c>
     </row>
@@ -9265,7 +9265,7 @@
       </c>
       <c r="P98" s="15" t="inlineStr">
         <is>
-          <t>24.1%</t>
+          <t>23.4%</t>
         </is>
       </c>
       <c r="Q98" s="15" t="inlineStr">
@@ -9275,7 +9275,7 @@
       </c>
       <c r="R98" s="15" t="inlineStr">
         <is>
-          <t>75.9%</t>
+          <t>76.6%</t>
         </is>
       </c>
     </row>
@@ -9351,7 +9351,7 @@
       </c>
       <c r="P99" s="15" t="inlineStr">
         <is>
-          <t>25.5%</t>
+          <t>26.0%</t>
         </is>
       </c>
       <c r="Q99" s="15" t="inlineStr">
@@ -9361,7 +9361,7 @@
       </c>
       <c r="R99" s="15" t="inlineStr">
         <is>
-          <t>74.5%</t>
+          <t>74.0%</t>
         </is>
       </c>
     </row>
@@ -9437,7 +9437,7 @@
       </c>
       <c r="P100" s="19" t="inlineStr">
         <is>
-          <t>43.2%</t>
+          <t>43.1%</t>
         </is>
       </c>
       <c r="Q100" s="19" t="inlineStr">
@@ -9447,7 +9447,7 @@
       </c>
       <c r="R100" s="19" t="inlineStr">
         <is>
-          <t>56.8%</t>
+          <t>56.9%</t>
         </is>
       </c>
     </row>
@@ -9609,7 +9609,7 @@
       </c>
       <c r="P102" s="19" t="inlineStr">
         <is>
-          <t>56.3%</t>
+          <t>55.9%</t>
         </is>
       </c>
       <c r="Q102" s="19" t="inlineStr">
@@ -9619,7 +9619,7 @@
       </c>
       <c r="R102" s="19" t="inlineStr">
         <is>
-          <t>43.7%</t>
+          <t>44.1%</t>
         </is>
       </c>
     </row>
@@ -9695,7 +9695,7 @@
       </c>
       <c r="P103" s="19" t="inlineStr">
         <is>
-          <t>33.4%</t>
+          <t>33.7%</t>
         </is>
       </c>
       <c r="Q103" s="19" t="inlineStr">
@@ -9705,7 +9705,7 @@
       </c>
       <c r="R103" s="19" t="inlineStr">
         <is>
-          <t>66.6%</t>
+          <t>66.3%</t>
         </is>
       </c>
     </row>
@@ -9867,7 +9867,7 @@
       </c>
       <c r="P105" s="23" t="inlineStr">
         <is>
-          <t>45.2%</t>
+          <t>45.3%</t>
         </is>
       </c>
       <c r="Q105" s="23" t="inlineStr">
@@ -9877,7 +9877,7 @@
       </c>
       <c r="R105" s="23" t="inlineStr">
         <is>
-          <t>54.8%</t>
+          <t>54.7%</t>
         </is>
       </c>
     </row>
@@ -9953,7 +9953,7 @@
       </c>
       <c r="P106" s="27" t="inlineStr">
         <is>
-          <t>39.8%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="Q106" s="27" t="inlineStr">
@@ -9963,7 +9963,7 @@
       </c>
       <c r="R106" s="27" t="inlineStr">
         <is>
-          <t>60.2%</t>
+          <t>60.0%</t>
         </is>
       </c>
     </row>
@@ -10039,7 +10039,7 @@
       </c>
       <c r="P107" s="18" t="inlineStr">
         <is>
-          <t>58.5%</t>
+          <t>58.8%</t>
         </is>
       </c>
       <c r="Q107" s="18" t="inlineStr">
@@ -10049,7 +10049,7 @@
       </c>
       <c r="R107" s="18" t="inlineStr">
         <is>
-          <t>41.5%</t>
+          <t>41.2%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix incremental Soccerbase refresh
</commit_message>
<xml_diff>
--- a/github_vercel_app/public/files/Scorito_scores_met_kansen_latest.xlsx
+++ b/github_vercel_app/public/files/Scorito_scores_met_kansen_latest.xlsx
@@ -897,17 +897,17 @@
       </c>
       <c r="P4" s="7" t="inlineStr">
         <is>
-          <t>88.1%</t>
+          <t>87.6%</t>
         </is>
       </c>
       <c r="Q4" s="7" t="inlineStr">
         <is>
-          <t>6.6%</t>
+          <t>6.9%</t>
         </is>
       </c>
       <c r="R4" s="7" t="inlineStr">
         <is>
-          <t>5.3%</t>
+          <t>5.5%</t>
         </is>
       </c>
     </row>
@@ -987,17 +987,17 @@
       </c>
       <c r="P5" s="7" t="inlineStr">
         <is>
-          <t>62.5%</t>
+          <t>62.1%</t>
         </is>
       </c>
       <c r="Q5" s="7" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>15.4%</t>
         </is>
       </c>
       <c r="R5" s="7" t="inlineStr">
         <is>
-          <t>21.8%</t>
+          <t>22.5%</t>
         </is>
       </c>
     </row>
@@ -1020,7 +1020,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>Canada</t>
         </is>
@@ -1042,7 +1042,7 @@
       </c>
       <c r="I6" s="10" t="inlineStr">
         <is>
-          <t>2-0</t>
+          <t>1-1</t>
         </is>
       </c>
       <c r="J6" s="7" t="inlineStr">
@@ -1077,17 +1077,17 @@
       </c>
       <c r="P6" s="7" t="inlineStr">
         <is>
-          <t>76.1%</t>
+          <t>73.9%</t>
         </is>
       </c>
       <c r="Q6" s="7" t="inlineStr">
         <is>
-          <t>12.8%</t>
+          <t>13.4%</t>
         </is>
       </c>
       <c r="R6" s="7" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>12.7%</t>
         </is>
       </c>
     </row>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="I7" s="10" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>4-1</t>
         </is>
       </c>
       <c r="J7" s="7" t="inlineStr">
@@ -1167,17 +1167,17 @@
       </c>
       <c r="P7" s="7" t="inlineStr">
         <is>
-          <t>44.5%</t>
+          <t>53.3%</t>
         </is>
       </c>
       <c r="Q7" s="7" t="inlineStr">
         <is>
-          <t>18.2%</t>
+          <t>16.6%</t>
         </is>
       </c>
       <c r="R7" s="7" t="inlineStr">
         <is>
-          <t>37.3%</t>
+          <t>30.1%</t>
         </is>
       </c>
     </row>
@@ -1257,17 +1257,17 @@
       </c>
       <c r="P8" s="7" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>10.7%</t>
         </is>
       </c>
       <c r="Q8" s="7" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.9%</t>
         </is>
       </c>
       <c r="R8" s="7" t="inlineStr">
         <is>
-          <t>77.2%</t>
+          <t>76.5%</t>
         </is>
       </c>
     </row>
@@ -1347,17 +1347,17 @@
       </c>
       <c r="P9" s="7" t="inlineStr">
         <is>
-          <t>52.0%</t>
+          <t>51.9%</t>
         </is>
       </c>
       <c r="Q9" s="7" t="inlineStr">
         <is>
-          <t>18.0%</t>
+          <t>17.8%</t>
         </is>
       </c>
       <c r="R9" s="7" t="inlineStr">
         <is>
-          <t>30.0%</t>
+          <t>30.3%</t>
         </is>
       </c>
     </row>
@@ -1437,12 +1437,12 @@
       </c>
       <c r="P10" s="7" t="inlineStr">
         <is>
-          <t>20.2%</t>
+          <t>20.4%</t>
         </is>
       </c>
       <c r="Q10" s="7" t="inlineStr">
         <is>
-          <t>19.7%</t>
+          <t>19.5%</t>
         </is>
       </c>
       <c r="R10" s="7" t="inlineStr">
@@ -1527,17 +1527,17 @@
       </c>
       <c r="P11" s="7" t="inlineStr">
         <is>
-          <t>26.5%</t>
+          <t>27.4%</t>
         </is>
       </c>
       <c r="Q11" s="7" t="inlineStr">
         <is>
-          <t>16.5%</t>
+          <t>16.9%</t>
         </is>
       </c>
       <c r="R11" s="7" t="inlineStr">
         <is>
-          <t>57.0%</t>
+          <t>55.7%</t>
         </is>
       </c>
     </row>
@@ -1617,17 +1617,17 @@
       </c>
       <c r="P12" s="7" t="inlineStr">
         <is>
-          <t>83.5%</t>
+          <t>83.3%</t>
         </is>
       </c>
       <c r="Q12" s="7" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>8.9%</t>
         </is>
       </c>
       <c r="R12" s="7" t="inlineStr">
         <is>
-          <t>7.2%</t>
+          <t>7.7%</t>
         </is>
       </c>
     </row>
@@ -1707,17 +1707,17 @@
       </c>
       <c r="P13" s="7" t="inlineStr">
         <is>
-          <t>48.6%</t>
+          <t>46.7%</t>
         </is>
       </c>
       <c r="Q13" s="7" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>13.1%</t>
         </is>
       </c>
       <c r="R13" s="7" t="inlineStr">
         <is>
-          <t>38.2%</t>
+          <t>40.2%</t>
         </is>
       </c>
     </row>
@@ -1797,17 +1797,17 @@
       </c>
       <c r="P14" s="7" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>13.9%</t>
         </is>
       </c>
       <c r="Q14" s="7" t="inlineStr">
         <is>
-          <t>16.6%</t>
+          <t>15.9%</t>
         </is>
       </c>
       <c r="R14" s="7" t="inlineStr">
         <is>
-          <t>69.1%</t>
+          <t>70.2%</t>
         </is>
       </c>
     </row>
@@ -1887,17 +1887,17 @@
       </c>
       <c r="P15" s="7" t="inlineStr">
         <is>
-          <t>41.4%</t>
+          <t>41.7%</t>
         </is>
       </c>
       <c r="Q15" s="7" t="inlineStr">
         <is>
-          <t>16.5%</t>
+          <t>16.0%</t>
         </is>
       </c>
       <c r="R15" s="7" t="inlineStr">
         <is>
-          <t>42.1%</t>
+          <t>42.3%</t>
         </is>
       </c>
     </row>
@@ -1937,12 +1937,12 @@
       </c>
       <c r="H16" s="10" t="inlineStr">
         <is>
-          <t>2-0</t>
+          <t>3-0</t>
         </is>
       </c>
       <c r="I16" s="10" t="inlineStr">
         <is>
-          <t>2-0</t>
+          <t>3-0</t>
         </is>
       </c>
       <c r="J16" s="7" t="inlineStr">
@@ -1977,17 +1977,17 @@
       </c>
       <c r="P16" s="7" t="inlineStr">
         <is>
-          <t>89.0%</t>
+          <t>88.8%</t>
         </is>
       </c>
       <c r="Q16" s="7" t="inlineStr">
         <is>
-          <t>6.2%</t>
+          <t>6.3%</t>
         </is>
       </c>
       <c r="R16" s="7" t="inlineStr">
         <is>
-          <t>4.8%</t>
+          <t>4.9%</t>
         </is>
       </c>
     </row>
@@ -2067,17 +2067,17 @@
       </c>
       <c r="P17" s="7" t="inlineStr">
         <is>
-          <t>53.8%</t>
+          <t>54.0%</t>
         </is>
       </c>
       <c r="Q17" s="7" t="inlineStr">
         <is>
-          <t>12.1%</t>
+          <t>11.8%</t>
         </is>
       </c>
       <c r="R17" s="7" t="inlineStr">
         <is>
-          <t>34.1%</t>
+          <t>34.2%</t>
         </is>
       </c>
     </row>
@@ -2157,17 +2157,17 @@
       </c>
       <c r="P18" s="7" t="inlineStr">
         <is>
-          <t>13.5%</t>
+          <t>13.4%</t>
         </is>
       </c>
       <c r="Q18" s="7" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>15.0%</t>
         </is>
       </c>
       <c r="R18" s="7" t="inlineStr">
         <is>
-          <t>70.8%</t>
+          <t>71.6%</t>
         </is>
       </c>
     </row>
@@ -2247,17 +2247,17 @@
       </c>
       <c r="P19" s="7" t="inlineStr">
         <is>
-          <t>69.5%</t>
+          <t>70.3%</t>
         </is>
       </c>
       <c r="Q19" s="7" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>10.7%</t>
         </is>
       </c>
       <c r="R19" s="7" t="inlineStr">
         <is>
-          <t>19.4%</t>
+          <t>18.9%</t>
         </is>
       </c>
     </row>
@@ -2337,17 +2337,17 @@
       </c>
       <c r="P20" s="7" t="inlineStr">
         <is>
-          <t>64.7%</t>
+          <t>64.5%</t>
         </is>
       </c>
       <c r="Q20" s="7" t="inlineStr">
         <is>
-          <t>13.4%</t>
+          <t>13.3%</t>
         </is>
       </c>
       <c r="R20" s="7" t="inlineStr">
         <is>
-          <t>21.9%</t>
+          <t>22.1%</t>
         </is>
       </c>
     </row>
@@ -2427,17 +2427,17 @@
       </c>
       <c r="P21" s="7" t="inlineStr">
         <is>
-          <t>16.1%</t>
+          <t>16.2%</t>
         </is>
       </c>
       <c r="Q21" s="7" t="inlineStr">
         <is>
-          <t>14.8%</t>
+          <t>14.9%</t>
         </is>
       </c>
       <c r="R21" s="7" t="inlineStr">
         <is>
-          <t>69.2%</t>
+          <t>68.9%</t>
         </is>
       </c>
     </row>
@@ -2517,12 +2517,12 @@
       </c>
       <c r="P22" s="7" t="inlineStr">
         <is>
-          <t>77.0%</t>
+          <t>76.8%</t>
         </is>
       </c>
       <c r="Q22" s="7" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>11.1%</t>
         </is>
       </c>
       <c r="R22" s="7" t="inlineStr">
@@ -2612,12 +2612,12 @@
       </c>
       <c r="Q23" s="7" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>14.8%</t>
         </is>
       </c>
       <c r="R23" s="7" t="inlineStr">
         <is>
-          <t>24.1%</t>
+          <t>23.9%</t>
         </is>
       </c>
     </row>
@@ -2697,17 +2697,17 @@
       </c>
       <c r="P24" s="7" t="inlineStr">
         <is>
-          <t>75.6%</t>
+          <t>76.3%</t>
         </is>
       </c>
       <c r="Q24" s="7" t="inlineStr">
         <is>
-          <t>14.0%</t>
+          <t>13.6%</t>
         </is>
       </c>
       <c r="R24" s="7" t="inlineStr">
         <is>
-          <t>10.4%</t>
+          <t>10.1%</t>
         </is>
       </c>
     </row>
@@ -2787,17 +2787,17 @@
       </c>
       <c r="P25" s="7" t="inlineStr">
         <is>
-          <t>52.7%</t>
+          <t>53.9%</t>
         </is>
       </c>
       <c r="Q25" s="7" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>16.4%</t>
         </is>
       </c>
       <c r="R25" s="7" t="inlineStr">
         <is>
-          <t>29.9%</t>
+          <t>29.7%</t>
         </is>
       </c>
     </row>
@@ -2877,17 +2877,17 @@
       </c>
       <c r="P26" s="7" t="inlineStr">
         <is>
-          <t>23.2%</t>
+          <t>22.5%</t>
         </is>
       </c>
       <c r="Q26" s="7" t="inlineStr">
         <is>
-          <t>13.4%</t>
+          <t>13.7%</t>
         </is>
       </c>
       <c r="R26" s="7" t="inlineStr">
         <is>
-          <t>63.4%</t>
+          <t>63.8%</t>
         </is>
       </c>
     </row>
@@ -2967,17 +2967,17 @@
       </c>
       <c r="P27" s="7" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>17.8%</t>
         </is>
       </c>
       <c r="Q27" s="7" t="inlineStr">
         <is>
-          <t>16.2%</t>
+          <t>15.5%</t>
         </is>
       </c>
       <c r="R27" s="7" t="inlineStr">
         <is>
-          <t>66.3%</t>
+          <t>66.7%</t>
         </is>
       </c>
     </row>
@@ -3057,17 +3057,17 @@
       </c>
       <c r="P28" s="7" t="inlineStr">
         <is>
-          <t>50.8%</t>
+          <t>52.4%</t>
         </is>
       </c>
       <c r="Q28" s="7" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>14.2%</t>
         </is>
       </c>
       <c r="R28" s="7" t="inlineStr">
         <is>
-          <t>34.7%</t>
+          <t>33.4%</t>
         </is>
       </c>
     </row>
@@ -3147,17 +3147,17 @@
       </c>
       <c r="P29" s="7" t="inlineStr">
         <is>
-          <t>77.0%</t>
+          <t>76.4%</t>
         </is>
       </c>
       <c r="Q29" s="7" t="inlineStr">
         <is>
-          <t>10.4%</t>
+          <t>10.9%</t>
         </is>
       </c>
       <c r="R29" s="7" t="inlineStr">
         <is>
-          <t>12.6%</t>
+          <t>12.7%</t>
         </is>
       </c>
     </row>
@@ -3237,17 +3237,17 @@
       </c>
       <c r="P30" s="7" t="inlineStr">
         <is>
-          <t>81.9%</t>
+          <t>82.0%</t>
         </is>
       </c>
       <c r="Q30" s="7" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>9.9%</t>
         </is>
       </c>
       <c r="R30" s="7" t="inlineStr">
         <is>
-          <t>8.4%</t>
+          <t>8.1%</t>
         </is>
       </c>
     </row>
@@ -3332,12 +3332,12 @@
       </c>
       <c r="Q31" s="7" t="inlineStr">
         <is>
-          <t>16.3%</t>
+          <t>16.1%</t>
         </is>
       </c>
       <c r="R31" s="7" t="inlineStr">
         <is>
-          <t>20.9%</t>
+          <t>21.1%</t>
         </is>
       </c>
     </row>
@@ -3417,17 +3417,17 @@
       </c>
       <c r="P32" s="7" t="inlineStr">
         <is>
-          <t>54.0%</t>
+          <t>58.7%</t>
         </is>
       </c>
       <c r="Q32" s="7" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>16.2%</t>
         </is>
       </c>
       <c r="R32" s="7" t="inlineStr">
         <is>
-          <t>28.9%</t>
+          <t>25.1%</t>
         </is>
       </c>
     </row>
@@ -3507,7 +3507,7 @@
       </c>
       <c r="P33" s="7" t="inlineStr">
         <is>
-          <t>24.5%</t>
+          <t>25.3%</t>
         </is>
       </c>
       <c r="Q33" s="7" t="inlineStr">
@@ -3517,7 +3517,7 @@
       </c>
       <c r="R33" s="7" t="inlineStr">
         <is>
-          <t>59.5%</t>
+          <t>58.7%</t>
         </is>
       </c>
     </row>
@@ -3597,17 +3597,17 @@
       </c>
       <c r="P34" s="7" t="inlineStr">
         <is>
-          <t>87.6%</t>
+          <t>87.0%</t>
         </is>
       </c>
       <c r="Q34" s="7" t="inlineStr">
         <is>
+          <t>6.6%</t>
+        </is>
+      </c>
+      <c r="R34" s="7" t="inlineStr">
+        <is>
           <t>6.4%</t>
-        </is>
-      </c>
-      <c r="R34" s="7" t="inlineStr">
-        <is>
-          <t>6.0%</t>
         </is>
       </c>
     </row>
@@ -3647,12 +3647,12 @@
       </c>
       <c r="H35" s="10" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="I35" s="10" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J35" s="7" t="inlineStr">
@@ -3687,17 +3687,17 @@
       </c>
       <c r="P35" s="7" t="inlineStr">
         <is>
-          <t>39.7%</t>
+          <t>43.7%</t>
         </is>
       </c>
       <c r="Q35" s="7" t="inlineStr">
         <is>
-          <t>16.6%</t>
+          <t>16.2%</t>
         </is>
       </c>
       <c r="R35" s="7" t="inlineStr">
         <is>
-          <t>43.7%</t>
+          <t>40.1%</t>
         </is>
       </c>
     </row>
@@ -3737,12 +3737,12 @@
       </c>
       <c r="H36" s="10" t="inlineStr">
         <is>
-          <t>2-0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="I36" s="10" t="inlineStr">
         <is>
-          <t>2-0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J36" s="7" t="inlineStr">
@@ -3777,17 +3777,17 @@
       </c>
       <c r="P36" s="7" t="inlineStr">
         <is>
-          <t>67.4%</t>
+          <t>66.4%</t>
         </is>
       </c>
       <c r="Q36" s="7" t="inlineStr">
         <is>
-          <t>12.6%</t>
+          <t>13.9%</t>
         </is>
       </c>
       <c r="R36" s="7" t="inlineStr">
         <is>
-          <t>20.0%</t>
+          <t>19.7%</t>
         </is>
       </c>
     </row>
@@ -3867,17 +3867,17 @@
       </c>
       <c r="P37" s="7" t="inlineStr">
         <is>
-          <t>68.9%</t>
+          <t>68.4%</t>
         </is>
       </c>
       <c r="Q37" s="7" t="inlineStr">
         <is>
-          <t>13.6%</t>
+          <t>13.8%</t>
         </is>
       </c>
       <c r="R37" s="7" t="inlineStr">
         <is>
-          <t>17.6%</t>
+          <t>17.8%</t>
         </is>
       </c>
     </row>
@@ -3957,17 +3957,17 @@
       </c>
       <c r="P38" s="7" t="inlineStr">
         <is>
-          <t>87.4%</t>
+          <t>87.1%</t>
         </is>
       </c>
       <c r="Q38" s="7" t="inlineStr">
         <is>
-          <t>6.3%</t>
+          <t>6.1%</t>
         </is>
       </c>
       <c r="R38" s="7" t="inlineStr">
         <is>
-          <t>6.3%</t>
+          <t>6.8%</t>
         </is>
       </c>
     </row>
@@ -4047,17 +4047,17 @@
       </c>
       <c r="P39" s="7" t="inlineStr">
         <is>
-          <t>17.0%</t>
+          <t>16.9%</t>
         </is>
       </c>
       <c r="Q39" s="7" t="inlineStr">
         <is>
-          <t>17.2%</t>
+          <t>16.6%</t>
         </is>
       </c>
       <c r="R39" s="7" t="inlineStr">
         <is>
-          <t>65.8%</t>
+          <t>66.5%</t>
         </is>
       </c>
     </row>
@@ -4137,7 +4137,7 @@
       </c>
       <c r="P40" s="7" t="inlineStr">
         <is>
-          <t>89.2%</t>
+          <t>89.3%</t>
         </is>
       </c>
       <c r="Q40" s="7" t="inlineStr">
@@ -4147,7 +4147,7 @@
       </c>
       <c r="R40" s="7" t="inlineStr">
         <is>
-          <t>3.9%</t>
+          <t>3.8%</t>
         </is>
       </c>
     </row>
@@ -4227,17 +4227,17 @@
       </c>
       <c r="P41" s="7" t="inlineStr">
         <is>
-          <t>49.0%</t>
+          <t>48.8%</t>
         </is>
       </c>
       <c r="Q41" s="7" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>12.5%</t>
         </is>
       </c>
       <c r="R41" s="7" t="inlineStr">
         <is>
-          <t>38.0%</t>
+          <t>38.8%</t>
         </is>
       </c>
     </row>
@@ -4317,17 +4317,17 @@
       </c>
       <c r="P42" s="7" t="inlineStr">
         <is>
-          <t>84.5%</t>
+          <t>84.0%</t>
         </is>
       </c>
       <c r="Q42" s="7" t="inlineStr">
         <is>
-          <t>8.9%</t>
+          <t>9.0%</t>
         </is>
       </c>
       <c r="R42" s="7" t="inlineStr">
         <is>
-          <t>6.6%</t>
+          <t>6.9%</t>
         </is>
       </c>
     </row>
@@ -4407,17 +4407,17 @@
       </c>
       <c r="P43" s="7" t="inlineStr">
         <is>
-          <t>25.5%</t>
+          <t>25.7%</t>
         </is>
       </c>
       <c r="Q43" s="7" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>17.0%</t>
         </is>
       </c>
       <c r="R43" s="7" t="inlineStr">
         <is>
-          <t>57.8%</t>
+          <t>57.3%</t>
         </is>
       </c>
     </row>
@@ -4497,17 +4497,17 @@
       </c>
       <c r="P44" s="7" t="inlineStr">
         <is>
-          <t>74.9%</t>
+          <t>74.1%</t>
         </is>
       </c>
       <c r="Q44" s="7" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>11.2%</t>
         </is>
       </c>
       <c r="R44" s="7" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.7%</t>
         </is>
       </c>
     </row>
@@ -4587,12 +4587,12 @@
       </c>
       <c r="P45" s="7" t="inlineStr">
         <is>
-          <t>81.7%</t>
+          <t>81.5%</t>
         </is>
       </c>
       <c r="Q45" s="7" t="inlineStr">
         <is>
-          <t>8.7%</t>
+          <t>8.9%</t>
         </is>
       </c>
       <c r="R45" s="7" t="inlineStr">
@@ -4677,17 +4677,17 @@
       </c>
       <c r="P46" s="7" t="inlineStr">
         <is>
-          <t>44.3%</t>
+          <t>45.0%</t>
         </is>
       </c>
       <c r="Q46" s="7" t="inlineStr">
         <is>
-          <t>16.2%</t>
+          <t>15.9%</t>
         </is>
       </c>
       <c r="R46" s="7" t="inlineStr">
         <is>
-          <t>39.5%</t>
+          <t>39.1%</t>
         </is>
       </c>
     </row>
@@ -4767,17 +4767,17 @@
       </c>
       <c r="P47" s="7" t="inlineStr">
         <is>
-          <t>28.2%</t>
+          <t>27.0%</t>
         </is>
       </c>
       <c r="Q47" s="7" t="inlineStr">
         <is>
-          <t>13.8%</t>
+          <t>14.3%</t>
         </is>
       </c>
       <c r="R47" s="7" t="inlineStr">
         <is>
-          <t>57.9%</t>
+          <t>58.7%</t>
         </is>
       </c>
     </row>
@@ -4817,12 +4817,12 @@
       </c>
       <c r="H48" s="10" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>2-0</t>
         </is>
       </c>
       <c r="I48" s="10" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>2-0</t>
         </is>
       </c>
       <c r="J48" s="7" t="inlineStr">
@@ -4862,12 +4862,12 @@
       </c>
       <c r="Q48" s="7" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>17.4%</t>
         </is>
       </c>
       <c r="R48" s="7" t="inlineStr">
         <is>
-          <t>15.5%</t>
+          <t>15.4%</t>
         </is>
       </c>
     </row>
@@ -4947,17 +4947,17 @@
       </c>
       <c r="P49" s="7" t="inlineStr">
         <is>
-          <t>88.1%</t>
+          <t>87.9%</t>
         </is>
       </c>
       <c r="Q49" s="7" t="inlineStr">
         <is>
-          <t>6.7%</t>
+          <t>6.8%</t>
         </is>
       </c>
       <c r="R49" s="7" t="inlineStr">
         <is>
-          <t>5.2%</t>
+          <t>5.3%</t>
         </is>
       </c>
     </row>
@@ -5037,17 +5037,17 @@
       </c>
       <c r="P50" s="7" t="inlineStr">
         <is>
-          <t>20.3%</t>
+          <t>19.8%</t>
         </is>
       </c>
       <c r="Q50" s="7" t="inlineStr">
         <is>
-          <t>18.8%</t>
+          <t>19.3%</t>
         </is>
       </c>
       <c r="R50" s="7" t="inlineStr">
         <is>
-          <t>60.9%</t>
+          <t>60.8%</t>
         </is>
       </c>
     </row>
@@ -5127,17 +5127,17 @@
       </c>
       <c r="P51" s="7" t="inlineStr">
         <is>
-          <t>80.7%</t>
+          <t>81.0%</t>
         </is>
       </c>
       <c r="Q51" s="7" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>9.6%</t>
         </is>
       </c>
       <c r="R51" s="7" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.4%</t>
         </is>
       </c>
     </row>
@@ -5217,17 +5217,17 @@
       </c>
       <c r="P52" s="7" t="inlineStr">
         <is>
-          <t>58.1%</t>
+          <t>59.9%</t>
         </is>
       </c>
       <c r="Q52" s="7" t="inlineStr">
         <is>
-          <t>13.4%</t>
+          <t>12.8%</t>
         </is>
       </c>
       <c r="R52" s="7" t="inlineStr">
         <is>
-          <t>28.5%</t>
+          <t>27.3%</t>
         </is>
       </c>
     </row>
@@ -5267,12 +5267,12 @@
       </c>
       <c r="H53" s="10" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="I53" s="10" t="inlineStr">
         <is>
-          <t>2-0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J53" s="7" t="inlineStr">
@@ -5307,17 +5307,17 @@
       </c>
       <c r="P53" s="7" t="inlineStr">
         <is>
-          <t>39.1%</t>
+          <t>41.9%</t>
         </is>
       </c>
       <c r="Q53" s="7" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>17.4%</t>
         </is>
       </c>
       <c r="R53" s="7" t="inlineStr">
         <is>
-          <t>44.2%</t>
+          <t>40.8%</t>
         </is>
       </c>
     </row>
@@ -5397,7 +5397,7 @@
       </c>
       <c r="P54" s="7" t="inlineStr">
         <is>
-          <t>13.8%</t>
+          <t>14.0%</t>
         </is>
       </c>
       <c r="Q54" s="7" t="inlineStr">
@@ -5407,7 +5407,7 @@
       </c>
       <c r="R54" s="7" t="inlineStr">
         <is>
-          <t>72.5%</t>
+          <t>72.3%</t>
         </is>
       </c>
     </row>
@@ -5487,7 +5487,7 @@
       </c>
       <c r="P55" s="7" t="inlineStr">
         <is>
-          <t>80.7%</t>
+          <t>80.6%</t>
         </is>
       </c>
       <c r="Q55" s="7" t="inlineStr">
@@ -5577,17 +5577,17 @@
       </c>
       <c r="P56" s="7" t="inlineStr">
         <is>
-          <t>25.4%</t>
+          <t>25.7%</t>
         </is>
       </c>
       <c r="Q56" s="7" t="inlineStr">
         <is>
-          <t>15.7%</t>
+          <t>15.5%</t>
         </is>
       </c>
       <c r="R56" s="7" t="inlineStr">
         <is>
-          <t>58.9%</t>
+          <t>58.8%</t>
         </is>
       </c>
     </row>
@@ -5667,17 +5667,17 @@
       </c>
       <c r="P57" s="7" t="inlineStr">
         <is>
-          <t>18.5%</t>
+          <t>19.4%</t>
         </is>
       </c>
       <c r="Q57" s="7" t="inlineStr">
         <is>
-          <t>15.6%</t>
+          <t>14.8%</t>
         </is>
       </c>
       <c r="R57" s="7" t="inlineStr">
         <is>
-          <t>65.9%</t>
+          <t>65.8%</t>
         </is>
       </c>
     </row>
@@ -5757,17 +5757,17 @@
       </c>
       <c r="P58" s="7" t="inlineStr">
         <is>
-          <t>22.2%</t>
+          <t>22.0%</t>
         </is>
       </c>
       <c r="Q58" s="7" t="inlineStr">
         <is>
-          <t>18.3%</t>
+          <t>18.6%</t>
         </is>
       </c>
       <c r="R58" s="7" t="inlineStr">
         <is>
-          <t>59.6%</t>
+          <t>59.4%</t>
         </is>
       </c>
     </row>
@@ -5847,17 +5847,17 @@
       </c>
       <c r="P59" s="7" t="inlineStr">
         <is>
-          <t>31.4%</t>
+          <t>33.0%</t>
         </is>
       </c>
       <c r="Q59" s="7" t="inlineStr">
         <is>
-          <t>19.1%</t>
+          <t>17.5%</t>
         </is>
       </c>
       <c r="R59" s="7" t="inlineStr">
         <is>
-          <t>49.4%</t>
+          <t>49.6%</t>
         </is>
       </c>
     </row>
@@ -5937,7 +5937,7 @@
       </c>
       <c r="P60" s="7" t="inlineStr">
         <is>
-          <t>67.4%</t>
+          <t>68.0%</t>
         </is>
       </c>
       <c r="Q60" s="7" t="inlineStr">
@@ -5947,7 +5947,7 @@
       </c>
       <c r="R60" s="7" t="inlineStr">
         <is>
-          <t>21.8%</t>
+          <t>21.2%</t>
         </is>
       </c>
     </row>
@@ -6027,17 +6027,17 @@
       </c>
       <c r="P61" s="7" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>14.1%</t>
         </is>
       </c>
       <c r="Q61" s="7" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>12.4%</t>
         </is>
       </c>
       <c r="R61" s="7" t="inlineStr">
         <is>
-          <t>73.6%</t>
+          <t>73.4%</t>
         </is>
       </c>
     </row>
@@ -6117,17 +6117,17 @@
       </c>
       <c r="P62" s="7" t="inlineStr">
         <is>
-          <t>64.0%</t>
+          <t>59.9%</t>
         </is>
       </c>
       <c r="Q62" s="7" t="inlineStr">
         <is>
-          <t>12.9%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="R62" s="7" t="inlineStr">
         <is>
-          <t>23.1%</t>
+          <t>25.6%</t>
         </is>
       </c>
     </row>
@@ -6207,17 +6207,17 @@
       </c>
       <c r="P63" s="7" t="inlineStr">
         <is>
-          <t>37.6%</t>
+          <t>36.6%</t>
         </is>
       </c>
       <c r="Q63" s="7" t="inlineStr">
         <is>
-          <t>19.6%</t>
+          <t>18.9%</t>
         </is>
       </c>
       <c r="R63" s="7" t="inlineStr">
         <is>
-          <t>42.8%</t>
+          <t>44.5%</t>
         </is>
       </c>
     </row>
@@ -6297,17 +6297,17 @@
       </c>
       <c r="P64" s="7" t="inlineStr">
         <is>
-          <t>18.3%</t>
+          <t>17.9%</t>
         </is>
       </c>
       <c r="Q64" s="7" t="inlineStr">
         <is>
-          <t>12.6%</t>
+          <t>12.1%</t>
         </is>
       </c>
       <c r="R64" s="7" t="inlineStr">
         <is>
-          <t>69.1%</t>
+          <t>70.0%</t>
         </is>
       </c>
     </row>
@@ -6387,17 +6387,17 @@
       </c>
       <c r="P65" s="7" t="inlineStr">
         <is>
-          <t>66.4%</t>
+          <t>65.2%</t>
         </is>
       </c>
       <c r="Q65" s="7" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>13.1%</t>
         </is>
       </c>
       <c r="R65" s="7" t="inlineStr">
         <is>
-          <t>20.4%</t>
+          <t>21.7%</t>
         </is>
       </c>
     </row>
@@ -6477,17 +6477,17 @@
       </c>
       <c r="P66" s="7" t="inlineStr">
         <is>
-          <t>26.4%</t>
+          <t>26.0%</t>
         </is>
       </c>
       <c r="Q66" s="7" t="inlineStr">
         <is>
-          <t>19.0%</t>
+          <t>20.3%</t>
         </is>
       </c>
       <c r="R66" s="7" t="inlineStr">
         <is>
-          <t>54.6%</t>
+          <t>53.7%</t>
         </is>
       </c>
     </row>
@@ -6567,17 +6567,17 @@
       </c>
       <c r="P67" s="7" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>14.0%</t>
         </is>
       </c>
       <c r="Q67" s="7" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>16.3%</t>
         </is>
       </c>
       <c r="R67" s="7" t="inlineStr">
         <is>
-          <t>68.5%</t>
+          <t>69.6%</t>
         </is>
       </c>
     </row>
@@ -6657,17 +6657,17 @@
       </c>
       <c r="P68" s="7" t="inlineStr">
         <is>
-          <t>30.0%</t>
+          <t>29.1%</t>
         </is>
       </c>
       <c r="Q68" s="7" t="inlineStr">
         <is>
-          <t>17.6%</t>
+          <t>16.8%</t>
         </is>
       </c>
       <c r="R68" s="7" t="inlineStr">
         <is>
-          <t>52.4%</t>
+          <t>54.1%</t>
         </is>
       </c>
     </row>
@@ -6747,17 +6747,17 @@
       </c>
       <c r="P69" s="7" t="inlineStr">
         <is>
-          <t>12.1%</t>
+          <t>13.4%</t>
         </is>
       </c>
       <c r="Q69" s="7" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.4%</t>
         </is>
       </c>
       <c r="R69" s="7" t="inlineStr">
         <is>
-          <t>76.4%</t>
+          <t>75.2%</t>
         </is>
       </c>
     </row>
@@ -6837,17 +6837,17 @@
       </c>
       <c r="P70" s="7" t="inlineStr">
         <is>
-          <t>11.6%</t>
+          <t>11.1%</t>
         </is>
       </c>
       <c r="Q70" s="7" t="inlineStr">
         <is>
-          <t>17.9%</t>
+          <t>19.5%</t>
         </is>
       </c>
       <c r="R70" s="7" t="inlineStr">
         <is>
-          <t>70.6%</t>
+          <t>69.4%</t>
         </is>
       </c>
     </row>
@@ -6927,12 +6927,12 @@
       </c>
       <c r="P71" s="7" t="inlineStr">
         <is>
-          <t>79.3%</t>
+          <t>79.0%</t>
         </is>
       </c>
       <c r="Q71" s="7" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>11.3%</t>
         </is>
       </c>
       <c r="R71" s="7" t="inlineStr">
@@ -7017,17 +7017,17 @@
       </c>
       <c r="P72" s="7" t="inlineStr">
         <is>
-          <t>36.6%</t>
+          <t>40.5%</t>
         </is>
       </c>
       <c r="Q72" s="7" t="inlineStr">
         <is>
-          <t>17.9%</t>
+          <t>16.8%</t>
         </is>
       </c>
       <c r="R72" s="7" t="inlineStr">
         <is>
-          <t>45.5%</t>
+          <t>42.7%</t>
         </is>
       </c>
     </row>
@@ -7107,17 +7107,17 @@
       </c>
       <c r="P73" s="7" t="inlineStr">
         <is>
-          <t>33.2%</t>
+          <t>33.7%</t>
         </is>
       </c>
       <c r="Q73" s="7" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>17.3%</t>
         </is>
       </c>
       <c r="R73" s="7" t="inlineStr">
         <is>
-          <t>49.6%</t>
+          <t>49.0%</t>
         </is>
       </c>
     </row>
@@ -7197,17 +7197,17 @@
       </c>
       <c r="P74" s="7" t="inlineStr">
         <is>
-          <t>35.9%</t>
+          <t>37.2%</t>
         </is>
       </c>
       <c r="Q74" s="7" t="inlineStr">
         <is>
-          <t>19.9%</t>
+          <t>19.8%</t>
         </is>
       </c>
       <c r="R74" s="7" t="inlineStr">
         <is>
-          <t>44.2%</t>
+          <t>43.0%</t>
         </is>
       </c>
     </row>
@@ -7287,17 +7287,17 @@
       </c>
       <c r="P75" s="7" t="inlineStr">
         <is>
+          <t>11.6%</t>
+        </is>
+      </c>
+      <c r="Q75" s="7" t="inlineStr">
+        <is>
           <t>10.4%</t>
         </is>
       </c>
-      <c r="Q75" s="7" t="inlineStr">
-        <is>
-          <t>11.4%</t>
-        </is>
-      </c>
       <c r="R75" s="7" t="inlineStr">
         <is>
-          <t>78.2%</t>
+          <t>78.1%</t>
         </is>
       </c>
     </row>
@@ -7316,12 +7316,12 @@
         </is>
       </c>
       <c r="D76" s="11" t="inlineStr"/>
-      <c r="E76" s="12" t="inlineStr">
+      <c r="E76" s="13" t="inlineStr">
         <is>
           <t>South Korea</t>
         </is>
       </c>
-      <c r="F76" s="13" t="inlineStr">
+      <c r="F76" s="12" t="inlineStr">
         <is>
           <t>Canada</t>
         </is>
@@ -7333,12 +7333,12 @@
       </c>
       <c r="H76" s="14" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="I76" s="14" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="J76" s="11" t="inlineStr">
@@ -7373,7 +7373,7 @@
       </c>
       <c r="P76" s="11" t="inlineStr">
         <is>
-          <t>46.0%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="Q76" s="11" t="inlineStr">
@@ -7383,7 +7383,7 @@
       </c>
       <c r="R76" s="11" t="inlineStr">
         <is>
-          <t>54.0%</t>
+          <t>50.0%</t>
         </is>
       </c>
     </row>
@@ -7459,7 +7459,7 @@
       </c>
       <c r="P77" s="11" t="inlineStr">
         <is>
-          <t>64.7%</t>
+          <t>64.5%</t>
         </is>
       </c>
       <c r="Q77" s="11" t="inlineStr">
@@ -7469,7 +7469,7 @@
       </c>
       <c r="R77" s="11" t="inlineStr">
         <is>
-          <t>35.3%</t>
+          <t>35.5%</t>
         </is>
       </c>
     </row>
@@ -7495,7 +7495,7 @@
       </c>
       <c r="F78" s="12" t="inlineStr">
         <is>
-          <t>Paraguay</t>
+          <t>Scotland</t>
         </is>
       </c>
       <c r="G78" s="12" t="inlineStr">
@@ -7545,7 +7545,7 @@
       </c>
       <c r="P78" s="11" t="inlineStr">
         <is>
-          <t>69.3%</t>
+          <t>75.6%</t>
         </is>
       </c>
       <c r="Q78" s="11" t="inlineStr">
@@ -7555,7 +7555,7 @@
       </c>
       <c r="R78" s="11" t="inlineStr">
         <is>
-          <t>30.7%</t>
+          <t>24.4%</t>
         </is>
       </c>
     </row>
@@ -7717,7 +7717,7 @@
       </c>
       <c r="P80" s="11" t="inlineStr">
         <is>
-          <t>55.4%</t>
+          <t>55.3%</t>
         </is>
       </c>
       <c r="Q80" s="11" t="inlineStr">
@@ -7727,7 +7727,7 @@
       </c>
       <c r="R80" s="11" t="inlineStr">
         <is>
-          <t>44.6%</t>
+          <t>44.7%</t>
         </is>
       </c>
     </row>
@@ -7839,7 +7839,7 @@
       </c>
       <c r="F82" s="12" t="inlineStr">
         <is>
-          <t>Senegal</t>
+          <t>Ivory Coast</t>
         </is>
       </c>
       <c r="G82" s="12" t="inlineStr">
@@ -7849,12 +7849,12 @@
       </c>
       <c r="H82" s="14" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="I82" s="14" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J82" s="11" t="inlineStr">
@@ -7889,7 +7889,7 @@
       </c>
       <c r="P82" s="11" t="inlineStr">
         <is>
-          <t>63.1%</t>
+          <t>81.0%</t>
         </is>
       </c>
       <c r="Q82" s="11" t="inlineStr">
@@ -7899,7 +7899,7 @@
       </c>
       <c r="R82" s="11" t="inlineStr">
         <is>
-          <t>36.9%</t>
+          <t>19.0%</t>
         </is>
       </c>
     </row>
@@ -7925,7 +7925,7 @@
       </c>
       <c r="F83" s="12" t="inlineStr">
         <is>
-          <t>Ivory Coast</t>
+          <t>Senegal</t>
         </is>
       </c>
       <c r="G83" s="12" t="inlineStr">
@@ -7935,12 +7935,12 @@
       </c>
       <c r="H83" s="14" t="inlineStr">
         <is>
-          <t>2-0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="I83" s="14" t="inlineStr">
         <is>
-          <t>2-0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J83" s="11" t="inlineStr">
@@ -7975,7 +7975,7 @@
       </c>
       <c r="P83" s="11" t="inlineStr">
         <is>
-          <t>87.6%</t>
+          <t>74.1%</t>
         </is>
       </c>
       <c r="Q83" s="11" t="inlineStr">
@@ -7985,7 +7985,7 @@
       </c>
       <c r="R83" s="11" t="inlineStr">
         <is>
-          <t>12.4%</t>
+          <t>25.9%</t>
         </is>
       </c>
     </row>
@@ -8061,7 +8061,7 @@
       </c>
       <c r="P84" s="11" t="inlineStr">
         <is>
-          <t>72.2%</t>
+          <t>72.0%</t>
         </is>
       </c>
       <c r="Q84" s="11" t="inlineStr">
@@ -8071,7 +8071,7 @@
       </c>
       <c r="R84" s="11" t="inlineStr">
         <is>
-          <t>27.8%</t>
+          <t>28.0%</t>
         </is>
       </c>
     </row>
@@ -8092,12 +8092,12 @@
       <c r="D85" s="11" t="inlineStr"/>
       <c r="E85" s="13" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F85" s="12" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Bosnia and Herzegovina</t>
         </is>
       </c>
       <c r="G85" s="12" t="inlineStr">
@@ -8147,7 +8147,7 @@
       </c>
       <c r="P85" s="11" t="inlineStr">
         <is>
-          <t>75.3%</t>
+          <t>76.8%</t>
         </is>
       </c>
       <c r="Q85" s="11" t="inlineStr">
@@ -8157,7 +8157,7 @@
       </c>
       <c r="R85" s="11" t="inlineStr">
         <is>
-          <t>24.7%</t>
+          <t>23.2%</t>
         </is>
       </c>
     </row>
@@ -8355,7 +8355,7 @@
       </c>
       <c r="F88" s="12" t="inlineStr">
         <is>
-          <t>Scotland</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="G88" s="12" t="inlineStr">
@@ -8405,7 +8405,7 @@
       </c>
       <c r="P88" s="11" t="inlineStr">
         <is>
-          <t>72.4%</t>
+          <t>77.9%</t>
         </is>
       </c>
       <c r="Q88" s="11" t="inlineStr">
@@ -8415,7 +8415,7 @@
       </c>
       <c r="R88" s="11" t="inlineStr">
         <is>
-          <t>27.6%</t>
+          <t>22.1%</t>
         </is>
       </c>
     </row>
@@ -8436,7 +8436,7 @@
       <c r="D89" s="11" t="inlineStr"/>
       <c r="E89" s="13" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="F89" s="12" t="inlineStr">
@@ -8451,12 +8451,12 @@
       </c>
       <c r="H89" s="14" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="I89" s="14" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J89" s="11" t="inlineStr">
@@ -8491,7 +8491,7 @@
       </c>
       <c r="P89" s="11" t="inlineStr">
         <is>
-          <t>60.7%</t>
+          <t>75.0%</t>
         </is>
       </c>
       <c r="Q89" s="11" t="inlineStr">
@@ -8501,7 +8501,7 @@
       </c>
       <c r="R89" s="11" t="inlineStr">
         <is>
-          <t>39.3%</t>
+          <t>25.0%</t>
         </is>
       </c>
     </row>
@@ -8613,7 +8613,7 @@
       </c>
       <c r="F91" s="12" t="inlineStr">
         <is>
-          <t>Bosnia and Herzegovina</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="G91" s="12" t="inlineStr">
@@ -8623,12 +8623,12 @@
       </c>
       <c r="H91" s="14" t="inlineStr">
         <is>
-          <t>2-0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="I91" s="14" t="inlineStr">
         <is>
-          <t>2-0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J91" s="11" t="inlineStr">
@@ -8663,7 +8663,7 @@
       </c>
       <c r="P91" s="11" t="inlineStr">
         <is>
-          <t>90.2%</t>
+          <t>78.7%</t>
         </is>
       </c>
       <c r="Q91" s="11" t="inlineStr">
@@ -8673,7 +8673,7 @@
       </c>
       <c r="R91" s="11" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>21.3%</t>
         </is>
       </c>
     </row>
@@ -8694,7 +8694,7 @@
       <c r="D92" s="15" t="inlineStr"/>
       <c r="E92" s="16" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="F92" s="17" t="inlineStr">
@@ -8749,7 +8749,7 @@
       </c>
       <c r="P92" s="15" t="inlineStr">
         <is>
-          <t>32.0%</t>
+          <t>28.7%</t>
         </is>
       </c>
       <c r="Q92" s="15" t="inlineStr">
@@ -8759,7 +8759,7 @@
       </c>
       <c r="R92" s="15" t="inlineStr">
         <is>
-          <t>68.0%</t>
+          <t>71.3%</t>
         </is>
       </c>
     </row>
@@ -8921,7 +8921,7 @@
       </c>
       <c r="P94" s="15" t="inlineStr">
         <is>
-          <t>34.6%</t>
+          <t>34.7%</t>
         </is>
       </c>
       <c r="Q94" s="15" t="inlineStr">
@@ -8931,7 +8931,7 @@
       </c>
       <c r="R94" s="15" t="inlineStr">
         <is>
-          <t>65.4%</t>
+          <t>65.3%</t>
         </is>
       </c>
     </row>
@@ -9007,7 +9007,7 @@
       </c>
       <c r="P95" s="15" t="inlineStr">
         <is>
-          <t>37.7%</t>
+          <t>37.5%</t>
         </is>
       </c>
       <c r="Q95" s="15" t="inlineStr">
@@ -9017,7 +9017,7 @@
       </c>
       <c r="R95" s="15" t="inlineStr">
         <is>
-          <t>62.3%</t>
+          <t>62.5%</t>
         </is>
       </c>
     </row>
@@ -9129,7 +9129,7 @@
       </c>
       <c r="F97" s="16" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="G97" s="16" t="inlineStr">
@@ -9179,7 +9179,7 @@
       </c>
       <c r="P97" s="15" t="inlineStr">
         <is>
-          <t>50.8%</t>
+          <t>60.4%</t>
         </is>
       </c>
       <c r="Q97" s="15" t="inlineStr">
@@ -9189,7 +9189,7 @@
       </c>
       <c r="R97" s="15" t="inlineStr">
         <is>
-          <t>49.2%</t>
+          <t>39.6%</t>
         </is>
       </c>
     </row>
@@ -9210,7 +9210,7 @@
       <c r="D98" s="15" t="inlineStr"/>
       <c r="E98" s="16" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="F98" s="17" t="inlineStr">
@@ -9225,12 +9225,12 @@
       </c>
       <c r="H98" s="18" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="I98" s="18" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="J98" s="15" t="inlineStr">
@@ -9265,7 +9265,7 @@
       </c>
       <c r="P98" s="15" t="inlineStr">
         <is>
-          <t>23.4%</t>
+          <t>37.2%</t>
         </is>
       </c>
       <c r="Q98" s="15" t="inlineStr">
@@ -9275,7 +9275,7 @@
       </c>
       <c r="R98" s="15" t="inlineStr">
         <is>
-          <t>76.6%</t>
+          <t>62.8%</t>
         </is>
       </c>
     </row>
@@ -9351,7 +9351,7 @@
       </c>
       <c r="P99" s="15" t="inlineStr">
         <is>
-          <t>26.0%</t>
+          <t>26.1%</t>
         </is>
       </c>
       <c r="Q99" s="15" t="inlineStr">
@@ -9361,7 +9361,7 @@
       </c>
       <c r="R99" s="15" t="inlineStr">
         <is>
-          <t>74.0%</t>
+          <t>73.9%</t>
         </is>
       </c>
     </row>
@@ -9437,7 +9437,7 @@
       </c>
       <c r="P100" s="19" t="inlineStr">
         <is>
-          <t>43.1%</t>
+          <t>43.0%</t>
         </is>
       </c>
       <c r="Q100" s="19" t="inlineStr">
@@ -9447,7 +9447,7 @@
       </c>
       <c r="R100" s="19" t="inlineStr">
         <is>
-          <t>56.9%</t>
+          <t>57.0%</t>
         </is>
       </c>
     </row>
@@ -9523,7 +9523,7 @@
       </c>
       <c r="P101" s="19" t="inlineStr">
         <is>
-          <t>82.0%</t>
+          <t>82.1%</t>
         </is>
       </c>
       <c r="Q101" s="19" t="inlineStr">
@@ -9533,7 +9533,7 @@
       </c>
       <c r="R101" s="19" t="inlineStr">
         <is>
-          <t>18.0%</t>
+          <t>17.9%</t>
         </is>
       </c>
     </row>
@@ -9609,7 +9609,7 @@
       </c>
       <c r="P102" s="19" t="inlineStr">
         <is>
-          <t>55.9%</t>
+          <t>55.7%</t>
         </is>
       </c>
       <c r="Q102" s="19" t="inlineStr">
@@ -9619,7 +9619,7 @@
       </c>
       <c r="R102" s="19" t="inlineStr">
         <is>
-          <t>44.1%</t>
+          <t>44.3%</t>
         </is>
       </c>
     </row>
@@ -9781,7 +9781,7 @@
       </c>
       <c r="P104" s="23" t="inlineStr">
         <is>
-          <t>27.9%</t>
+          <t>27.8%</t>
         </is>
       </c>
       <c r="Q104" s="23" t="inlineStr">
@@ -9791,7 +9791,7 @@
       </c>
       <c r="R104" s="23" t="inlineStr">
         <is>
-          <t>72.1%</t>
+          <t>72.2%</t>
         </is>
       </c>
     </row>
@@ -10039,7 +10039,7 @@
       </c>
       <c r="P107" s="18" t="inlineStr">
         <is>
-          <t>58.8%</t>
+          <t>58.9%</t>
         </is>
       </c>
       <c r="Q107" s="18" t="inlineStr">
@@ -10049,7 +10049,7 @@
       </c>
       <c r="R107" s="18" t="inlineStr">
         <is>
-          <t>41.2%</t>
+          <t>41.1%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix dashboard playoff fixtures and locked scores
</commit_message>
<xml_diff>
--- a/github_vercel_app/public/files/Scorito_scores_met_kansen_latest.xlsx
+++ b/github_vercel_app/public/files/Scorito_scores_met_kansen_latest.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="WK 2026 Voorspellingen" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WK 2026 Voorspellingen" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -897,17 +897,17 @@
       </c>
       <c r="P4" s="7" t="inlineStr">
         <is>
-          <t>88.3%</t>
+          <t>87.4%</t>
         </is>
       </c>
       <c r="Q4" s="7" t="inlineStr">
         <is>
-          <t>6.7%</t>
+          <t>7.1%</t>
         </is>
       </c>
       <c r="R4" s="7" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>5.4%</t>
         </is>
       </c>
     </row>
@@ -937,7 +937,7 @@
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>Winner UEFA Playoff D</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="G5" s="8" t="inlineStr">
@@ -947,12 +947,12 @@
       </c>
       <c r="H5" s="10" t="inlineStr">
         <is>
-          <t>4-0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="I5" s="10" t="inlineStr">
         <is>
-          <t>4-0</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
@@ -987,17 +987,17 @@
       </c>
       <c r="P5" s="7" t="inlineStr">
         <is>
-          <t>92.9%</t>
+          <t>62.0%</t>
         </is>
       </c>
       <c r="Q5" s="7" t="inlineStr">
         <is>
-          <t>3.7%</t>
+          <t>15.2%</t>
         </is>
       </c>
       <c r="R5" s="7" t="inlineStr">
         <is>
-          <t>3.4%</t>
+          <t>22.8%</t>
         </is>
       </c>
     </row>
@@ -1020,14 +1020,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>Canada</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>Winner UEFA Playoff A</t>
+          <t>Bosnia and Herzegovina</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
@@ -1037,12 +1037,12 @@
       </c>
       <c r="H6" s="10" t="inlineStr">
         <is>
-          <t>3-0</t>
+          <t>2-0</t>
         </is>
       </c>
       <c r="I6" s="10" t="inlineStr">
         <is>
-          <t>3-0</t>
+          <t>1-1</t>
         </is>
       </c>
       <c r="J6" s="7" t="inlineStr">
@@ -1077,17 +1077,17 @@
       </c>
       <c r="P6" s="7" t="inlineStr">
         <is>
-          <t>93.0%</t>
+          <t>73.4%</t>
         </is>
       </c>
       <c r="Q6" s="7" t="inlineStr">
         <is>
-          <t>3.7%</t>
+          <t>13.7%</t>
         </is>
       </c>
       <c r="R6" s="7" t="inlineStr">
         <is>
-          <t>3.2%</t>
+          <t>12.8%</t>
         </is>
       </c>
     </row>
@@ -1167,17 +1167,17 @@
       </c>
       <c r="P7" s="7" t="inlineStr">
         <is>
-          <t>54.2%</t>
+          <t>54.1%</t>
         </is>
       </c>
       <c r="Q7" s="7" t="inlineStr">
         <is>
-          <t>17.8%</t>
+          <t>16.9%</t>
         </is>
       </c>
       <c r="R7" s="7" t="inlineStr">
         <is>
-          <t>28.0%</t>
+          <t>29.1%</t>
         </is>
       </c>
     </row>
@@ -1257,17 +1257,17 @@
       </c>
       <c r="P8" s="7" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.4%</t>
         </is>
       </c>
       <c r="Q8" s="7" t="inlineStr">
         <is>
-          <t>16.3%</t>
+          <t>17.4%</t>
         </is>
       </c>
       <c r="R8" s="7" t="inlineStr">
         <is>
-          <t>72.5%</t>
+          <t>71.2%</t>
         </is>
       </c>
     </row>
@@ -1347,17 +1347,17 @@
       </c>
       <c r="P9" s="7" t="inlineStr">
         <is>
-          <t>51.2%</t>
+          <t>51.1%</t>
         </is>
       </c>
       <c r="Q9" s="7" t="inlineStr">
         <is>
-          <t>19.0%</t>
+          <t>18.9%</t>
         </is>
       </c>
       <c r="R9" s="7" t="inlineStr">
         <is>
-          <t>29.8%</t>
+          <t>30.0%</t>
         </is>
       </c>
     </row>
@@ -1407,47 +1407,47 @@
       </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
-          <t>5.51</t>
+          <t>5.49</t>
         </is>
       </c>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>4.33</t>
+          <t>4.30</t>
         </is>
       </c>
       <c r="L10" s="7" t="inlineStr">
         <is>
-          <t>1.57</t>
+          <t>1.59</t>
         </is>
       </c>
       <c r="M10" s="7" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>17.5%</t>
         </is>
       </c>
       <c r="N10" s="7" t="inlineStr">
         <is>
-          <t>22.0%</t>
+          <t>22.3%</t>
         </is>
       </c>
       <c r="O10" s="7" t="inlineStr">
         <is>
-          <t>60.7%</t>
+          <t>60.3%</t>
         </is>
       </c>
       <c r="P10" s="7" t="inlineStr">
         <is>
-          <t>17.7%</t>
+          <t>18.7%</t>
         </is>
       </c>
       <c r="Q10" s="7" t="inlineStr">
         <is>
-          <t>16.2%</t>
+          <t>15.8%</t>
         </is>
       </c>
       <c r="R10" s="7" t="inlineStr">
         <is>
-          <t>66.1%</t>
+          <t>65.5%</t>
         </is>
       </c>
     </row>
@@ -1497,17 +1497,17 @@
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>5.34</t>
+          <t>5.37</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
         <is>
-          <t>3.69</t>
+          <t>3.67</t>
         </is>
       </c>
       <c r="L11" s="7" t="inlineStr">
         <is>
-          <t>1.69</t>
+          <t>1.70</t>
         </is>
       </c>
       <c r="M11" s="7" t="inlineStr">
@@ -1517,27 +1517,27 @@
       </c>
       <c r="N11" s="7" t="inlineStr">
         <is>
-          <t>25.8%</t>
+          <t>26.0%</t>
         </is>
       </c>
       <c r="O11" s="7" t="inlineStr">
         <is>
-          <t>56.4%</t>
+          <t>56.2%</t>
         </is>
       </c>
       <c r="P11" s="7" t="inlineStr">
         <is>
-          <t>36.7%</t>
+          <t>37.2%</t>
         </is>
       </c>
       <c r="Q11" s="7" t="inlineStr">
         <is>
-          <t>19.8%</t>
+          <t>20.4%</t>
         </is>
       </c>
       <c r="R11" s="7" t="inlineStr">
         <is>
-          <t>43.5%</t>
+          <t>42.5%</t>
         </is>
       </c>
     </row>
@@ -1592,42 +1592,42 @@
       </c>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>17.38</t>
+          <t>18.60</t>
         </is>
       </c>
       <c r="L12" s="7" t="inlineStr">
         <is>
-          <t>36.25</t>
+          <t>41.95</t>
         </is>
       </c>
       <c r="M12" s="7" t="inlineStr">
         <is>
-          <t>91.9%</t>
+          <t>92.5%</t>
         </is>
       </c>
       <c r="N12" s="7" t="inlineStr">
         <is>
-          <t>5.5%</t>
+          <t>5.2%</t>
         </is>
       </c>
       <c r="O12" s="7" t="inlineStr">
         <is>
-          <t>2.6%</t>
+          <t>2.3%</t>
         </is>
       </c>
       <c r="P12" s="7" t="inlineStr">
         <is>
-          <t>83.3%</t>
+          <t>84.2%</t>
         </is>
       </c>
       <c r="Q12" s="7" t="inlineStr">
         <is>
-          <t>7.9%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="R12" s="7" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>7.3%</t>
         </is>
       </c>
     </row>
@@ -1677,27 +1677,27 @@
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>2.03</t>
+          <t>2.07</t>
         </is>
       </c>
       <c r="K13" s="7" t="inlineStr">
         <is>
-          <t>3.48</t>
+          <t>3.47</t>
         </is>
       </c>
       <c r="L13" s="7" t="inlineStr">
         <is>
-          <t>3.61</t>
+          <t>3.66</t>
         </is>
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
-          <t>46.6%</t>
+          <t>46.3%</t>
         </is>
       </c>
       <c r="N13" s="7" t="inlineStr">
         <is>
-          <t>27.2%</t>
+          <t>27.6%</t>
         </is>
       </c>
       <c r="O13" s="7" t="inlineStr">
@@ -1707,17 +1707,17 @@
       </c>
       <c r="P13" s="7" t="inlineStr">
         <is>
-          <t>46.0%</t>
+          <t>47.6%</t>
         </is>
       </c>
       <c r="Q13" s="7" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>12.8%</t>
         </is>
       </c>
       <c r="R13" s="7" t="inlineStr">
         <is>
-          <t>41.0%</t>
+          <t>39.7%</t>
         </is>
       </c>
     </row>
@@ -1767,47 +1767,47 @@
       </c>
       <c r="J14" s="7" t="inlineStr">
         <is>
-          <t>3.31</t>
+          <t>3.27</t>
         </is>
       </c>
       <c r="K14" s="7" t="inlineStr">
         <is>
-          <t>2.81</t>
+          <t>2.84</t>
         </is>
       </c>
       <c r="L14" s="7" t="inlineStr">
         <is>
-          <t>2.53</t>
+          <t>2.58</t>
         </is>
       </c>
       <c r="M14" s="7" t="inlineStr">
         <is>
-          <t>28.7%</t>
+          <t>29.2%</t>
         </is>
       </c>
       <c r="N14" s="7" t="inlineStr">
         <is>
-          <t>33.8%</t>
+          <t>33.7%</t>
         </is>
       </c>
       <c r="O14" s="7" t="inlineStr">
         <is>
-          <t>37.5%</t>
+          <t>37.1%</t>
         </is>
       </c>
       <c r="P14" s="7" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>13.9%</t>
         </is>
       </c>
       <c r="Q14" s="7" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>16.4%</t>
         </is>
       </c>
       <c r="R14" s="7" t="inlineStr">
         <is>
-          <t>68.2%</t>
+          <t>69.7%</t>
         </is>
       </c>
     </row>
@@ -1847,57 +1847,57 @@
       </c>
       <c r="H15" s="10" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="I15" s="10" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
-          <t>1.94</t>
+          <t>1.96</t>
         </is>
       </c>
       <c r="K15" s="7" t="inlineStr">
         <is>
-          <t>3.36</t>
+          <t>3.37</t>
         </is>
       </c>
       <c r="L15" s="7" t="inlineStr">
         <is>
-          <t>4.10</t>
+          <t>4.14</t>
         </is>
       </c>
       <c r="M15" s="7" t="inlineStr">
         <is>
-          <t>48.8%</t>
+          <t>48.7%</t>
         </is>
       </c>
       <c r="N15" s="7" t="inlineStr">
         <is>
-          <t>28.2%</t>
+          <t>28.3%</t>
         </is>
       </c>
       <c r="O15" s="7" t="inlineStr">
         <is>
-          <t>23.1%</t>
+          <t>23.0%</t>
         </is>
       </c>
       <c r="P15" s="7" t="inlineStr">
         <is>
-          <t>42.6%</t>
+          <t>41.7%</t>
         </is>
       </c>
       <c r="Q15" s="7" t="inlineStr">
         <is>
-          <t>16.1%</t>
+          <t>16.3%</t>
         </is>
       </c>
       <c r="R15" s="7" t="inlineStr">
         <is>
-          <t>41.3%</t>
+          <t>42.0%</t>
         </is>
       </c>
     </row>
@@ -1952,42 +1952,42 @@
       </c>
       <c r="K16" s="7" t="inlineStr">
         <is>
-          <t>11.13</t>
+          <t>10.96</t>
         </is>
       </c>
       <c r="L16" s="7" t="inlineStr">
         <is>
-          <t>24.00</t>
+          <t>24.26</t>
         </is>
       </c>
       <c r="M16" s="7" t="inlineStr">
         <is>
-          <t>87.5%</t>
+          <t>87.4%</t>
         </is>
       </c>
       <c r="N16" s="7" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>8.7%</t>
         </is>
       </c>
       <c r="O16" s="7" t="inlineStr">
         <is>
-          <t>4.0%</t>
+          <t>3.9%</t>
         </is>
       </c>
       <c r="P16" s="7" t="inlineStr">
         <is>
-          <t>89.9%</t>
+          <t>89.4%</t>
         </is>
       </c>
       <c r="Q16" s="7" t="inlineStr">
         <is>
-          <t>6.0%</t>
+          <t>6.2%</t>
         </is>
       </c>
       <c r="R16" s="7" t="inlineStr">
         <is>
-          <t>4.1%</t>
+          <t>4.4%</t>
         </is>
       </c>
     </row>
@@ -2037,22 +2037,22 @@
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
-          <t>1.60</t>
+          <t>1.62</t>
         </is>
       </c>
       <c r="K17" s="7" t="inlineStr">
         <is>
-          <t>3.88</t>
+          <t>3.91</t>
         </is>
       </c>
       <c r="L17" s="7" t="inlineStr">
         <is>
-          <t>5.60</t>
+          <t>5.64</t>
         </is>
       </c>
       <c r="M17" s="7" t="inlineStr">
         <is>
-          <t>58.9%</t>
+          <t>58.8%</t>
         </is>
       </c>
       <c r="N17" s="7" t="inlineStr">
@@ -2062,22 +2062,22 @@
       </c>
       <c r="O17" s="7" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>16.9%</t>
         </is>
       </c>
       <c r="P17" s="7" t="inlineStr">
         <is>
-          <t>54.7%</t>
+          <t>53.3%</t>
         </is>
       </c>
       <c r="Q17" s="7" t="inlineStr">
         <is>
-          <t>13.1%</t>
+          <t>12.3%</t>
         </is>
       </c>
       <c r="R17" s="7" t="inlineStr">
         <is>
-          <t>32.2%</t>
+          <t>34.4%</t>
         </is>
       </c>
     </row>
@@ -2127,47 +2127,47 @@
       </c>
       <c r="J18" s="7" t="inlineStr">
         <is>
-          <t>7.69</t>
+          <t>7.84</t>
         </is>
       </c>
       <c r="K18" s="7" t="inlineStr">
         <is>
-          <t>4.39</t>
+          <t>4.31</t>
         </is>
       </c>
       <c r="L18" s="7" t="inlineStr">
         <is>
-          <t>1.44</t>
+          <t>1.45</t>
         </is>
       </c>
       <c r="M18" s="7" t="inlineStr">
         <is>
-          <t>12.4%</t>
+          <t>12.2%</t>
         </is>
       </c>
       <c r="N18" s="7" t="inlineStr">
         <is>
-          <t>21.6%</t>
+          <t>22.1%</t>
         </is>
       </c>
       <c r="O18" s="7" t="inlineStr">
         <is>
-          <t>66.0%</t>
+          <t>65.7%</t>
         </is>
       </c>
       <c r="P18" s="7" t="inlineStr">
         <is>
-          <t>13.2%</t>
+          <t>13.3%</t>
         </is>
       </c>
       <c r="Q18" s="7" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>14.7%</t>
         </is>
       </c>
       <c r="R18" s="7" t="inlineStr">
         <is>
-          <t>72.9%</t>
+          <t>72.0%</t>
         </is>
       </c>
     </row>
@@ -2207,12 +2207,12 @@
       </c>
       <c r="H19" s="10" t="inlineStr">
         <is>
-          <t>2-0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="I19" s="10" t="inlineStr">
         <is>
-          <t>2-0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J19" s="7" t="inlineStr">
@@ -2222,37 +2222,37 @@
       </c>
       <c r="K19" s="7" t="inlineStr">
         <is>
-          <t>3.41</t>
+          <t>3.45</t>
         </is>
       </c>
       <c r="L19" s="7" t="inlineStr">
         <is>
-          <t>4.71</t>
+          <t>4.67</t>
         </is>
       </c>
       <c r="M19" s="7" t="inlineStr">
         <is>
-          <t>51.9%</t>
+          <t>52.0%</t>
         </is>
       </c>
       <c r="N19" s="7" t="inlineStr">
         <is>
-          <t>27.9%</t>
+          <t>27.6%</t>
         </is>
       </c>
       <c r="O19" s="7" t="inlineStr">
         <is>
-          <t>20.2%</t>
+          <t>20.4%</t>
         </is>
       </c>
       <c r="P19" s="7" t="inlineStr">
         <is>
-          <t>68.9%</t>
+          <t>69.2%</t>
         </is>
       </c>
       <c r="Q19" s="7" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>10.5%</t>
         </is>
       </c>
       <c r="R19" s="7" t="inlineStr">
@@ -2312,42 +2312,42 @@
       </c>
       <c r="K20" s="7" t="inlineStr">
         <is>
-          <t>4.37</t>
+          <t>4.35</t>
         </is>
       </c>
       <c r="L20" s="7" t="inlineStr">
         <is>
-          <t>7.00</t>
+          <t>7.12</t>
         </is>
       </c>
       <c r="M20" s="7" t="inlineStr">
         <is>
-          <t>64.7%</t>
+          <t>64.8%</t>
         </is>
       </c>
       <c r="N20" s="7" t="inlineStr">
         <is>
+          <t>21.9%</t>
+        </is>
+      </c>
+      <c r="O20" s="7" t="inlineStr">
+        <is>
+          <t>13.4%</t>
+        </is>
+      </c>
+      <c r="P20" s="7" t="inlineStr">
+        <is>
+          <t>64.2%</t>
+        </is>
+      </c>
+      <c r="Q20" s="7" t="inlineStr">
+        <is>
+          <t>13.9%</t>
+        </is>
+      </c>
+      <c r="R20" s="7" t="inlineStr">
+        <is>
           <t>21.8%</t>
-        </is>
-      </c>
-      <c r="O20" s="7" t="inlineStr">
-        <is>
-          <t>13.6%</t>
-        </is>
-      </c>
-      <c r="P20" s="7" t="inlineStr">
-        <is>
-          <t>65.9%</t>
-        </is>
-      </c>
-      <c r="Q20" s="7" t="inlineStr">
-        <is>
-          <t>12.6%</t>
-        </is>
-      </c>
-      <c r="R20" s="7" t="inlineStr">
-        <is>
-          <t>21.5%</t>
         </is>
       </c>
     </row>
@@ -2397,12 +2397,12 @@
       </c>
       <c r="J21" s="7" t="inlineStr">
         <is>
-          <t>14.00</t>
+          <t>15.16</t>
         </is>
       </c>
       <c r="K21" s="7" t="inlineStr">
         <is>
-          <t>7.00</t>
+          <t>7.09</t>
         </is>
       </c>
       <c r="L21" s="7" t="inlineStr">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="M21" s="7" t="inlineStr">
         <is>
-          <t>6.8%</t>
+          <t>6.3%</t>
         </is>
       </c>
       <c r="N21" s="7" t="inlineStr">
@@ -2422,22 +2422,22 @@
       </c>
       <c r="O21" s="7" t="inlineStr">
         <is>
-          <t>79.7%</t>
+          <t>80.2%</t>
         </is>
       </c>
       <c r="P21" s="7" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>15.7%</t>
         </is>
       </c>
       <c r="Q21" s="7" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>14.6%</t>
         </is>
       </c>
       <c r="R21" s="7" t="inlineStr">
         <is>
-          <t>68.7%</t>
+          <t>69.7%</t>
         </is>
       </c>
     </row>
@@ -2487,47 +2487,47 @@
       </c>
       <c r="J22" s="7" t="inlineStr">
         <is>
-          <t>1.39</t>
+          <t>1.40</t>
         </is>
       </c>
       <c r="K22" s="7" t="inlineStr">
         <is>
-          <t>4.61</t>
+          <t>4.49</t>
         </is>
       </c>
       <c r="L22" s="7" t="inlineStr">
         <is>
-          <t>8.63</t>
+          <t>8.92</t>
         </is>
       </c>
       <c r="M22" s="7" t="inlineStr">
         <is>
-          <t>68.4%</t>
+          <t>68.1%</t>
         </is>
       </c>
       <c r="N22" s="7" t="inlineStr">
         <is>
-          <t>20.6%</t>
+          <t>21.2%</t>
         </is>
       </c>
       <c r="O22" s="7" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>10.7%</t>
         </is>
       </c>
       <c r="P22" s="7" t="inlineStr">
         <is>
-          <t>77.6%</t>
+          <t>74.7%</t>
         </is>
       </c>
       <c r="Q22" s="7" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>12.0%</t>
         </is>
       </c>
       <c r="R22" s="7" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>13.3%</t>
         </is>
       </c>
     </row>
@@ -2582,42 +2582,42 @@
       </c>
       <c r="K23" s="7" t="inlineStr">
         <is>
-          <t>5.35</t>
+          <t>5.24</t>
         </is>
       </c>
       <c r="L23" s="7" t="inlineStr">
         <is>
-          <t>8.69</t>
+          <t>9.06</t>
         </is>
       </c>
       <c r="M23" s="7" t="inlineStr">
         <is>
-          <t>71.3%</t>
+          <t>71.4%</t>
         </is>
       </c>
       <c r="N23" s="7" t="inlineStr">
         <is>
-          <t>17.7%</t>
+          <t>18.1%</t>
         </is>
       </c>
       <c r="O23" s="7" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>10.5%</t>
         </is>
       </c>
       <c r="P23" s="7" t="inlineStr">
         <is>
-          <t>61.0%</t>
+          <t>62.0%</t>
         </is>
       </c>
       <c r="Q23" s="7" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>15.6%</t>
         </is>
       </c>
       <c r="R23" s="7" t="inlineStr">
         <is>
-          <t>23.7%</t>
+          <t>22.4%</t>
         </is>
       </c>
     </row>
@@ -2667,27 +2667,27 @@
       </c>
       <c r="J24" s="7" t="inlineStr">
         <is>
-          <t>1.28</t>
+          <t>1.29</t>
         </is>
       </c>
       <c r="K24" s="7" t="inlineStr">
         <is>
-          <t>5.74</t>
+          <t>5.48</t>
         </is>
       </c>
       <c r="L24" s="7" t="inlineStr">
         <is>
-          <t>10.44</t>
+          <t>10.46</t>
         </is>
       </c>
       <c r="M24" s="7" t="inlineStr">
         <is>
-          <t>74.3%</t>
+          <t>73.6%</t>
         </is>
       </c>
       <c r="N24" s="7" t="inlineStr">
         <is>
-          <t>16.6%</t>
+          <t>17.3%</t>
         </is>
       </c>
       <c r="O24" s="7" t="inlineStr">
@@ -2697,17 +2697,17 @@
       </c>
       <c r="P24" s="7" t="inlineStr">
         <is>
-          <t>74.8%</t>
+          <t>75.6%</t>
         </is>
       </c>
       <c r="Q24" s="7" t="inlineStr">
         <is>
-          <t>14.4%</t>
+          <t>14.2%</t>
         </is>
       </c>
       <c r="R24" s="7" t="inlineStr">
         <is>
-          <t>10.9%</t>
+          <t>10.2%</t>
         </is>
       </c>
     </row>
@@ -2762,22 +2762,22 @@
       </c>
       <c r="K25" s="7" t="inlineStr">
         <is>
-          <t>3.72</t>
+          <t>3.77</t>
         </is>
       </c>
       <c r="L25" s="7" t="inlineStr">
         <is>
-          <t>4.89</t>
+          <t>4.90</t>
         </is>
       </c>
       <c r="M25" s="7" t="inlineStr">
         <is>
-          <t>55.1%</t>
+          <t>55.3%</t>
         </is>
       </c>
       <c r="N25" s="7" t="inlineStr">
         <is>
-          <t>25.5%</t>
+          <t>25.2%</t>
         </is>
       </c>
       <c r="O25" s="7" t="inlineStr">
@@ -2787,17 +2787,17 @@
       </c>
       <c r="P25" s="7" t="inlineStr">
         <is>
-          <t>53.9%</t>
+          <t>52.8%</t>
         </is>
       </c>
       <c r="Q25" s="7" t="inlineStr">
         <is>
-          <t>18.2%</t>
+          <t>16.9%</t>
         </is>
       </c>
       <c r="R25" s="7" t="inlineStr">
         <is>
-          <t>27.9%</t>
+          <t>30.3%</t>
         </is>
       </c>
     </row>
@@ -2847,47 +2847,47 @@
       </c>
       <c r="J26" s="7" t="inlineStr">
         <is>
-          <t>2.15</t>
+          <t>2.16</t>
         </is>
       </c>
       <c r="K26" s="7" t="inlineStr">
         <is>
-          <t>3.38</t>
+          <t>3.41</t>
         </is>
       </c>
       <c r="L26" s="7" t="inlineStr">
         <is>
-          <t>3.43</t>
+          <t>3.39</t>
         </is>
       </c>
       <c r="M26" s="7" t="inlineStr">
         <is>
-          <t>44.2%</t>
+          <t>44.0%</t>
         </is>
       </c>
       <c r="N26" s="7" t="inlineStr">
         <is>
+          <t>27.9%</t>
+        </is>
+      </c>
+      <c r="O26" s="7" t="inlineStr">
+        <is>
           <t>28.1%</t>
         </is>
       </c>
-      <c r="O26" s="7" t="inlineStr">
-        <is>
-          <t>27.7%</t>
-        </is>
-      </c>
       <c r="P26" s="7" t="inlineStr">
         <is>
-          <t>21.2%</t>
+          <t>21.3%</t>
         </is>
       </c>
       <c r="Q26" s="7" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="R26" s="7" t="inlineStr">
         <is>
-          <t>64.4%</t>
+          <t>64.2%</t>
         </is>
       </c>
     </row>
@@ -2937,12 +2937,12 @@
       </c>
       <c r="J27" s="7" t="inlineStr">
         <is>
-          <t>8.81</t>
+          <t>8.75</t>
         </is>
       </c>
       <c r="K27" s="7" t="inlineStr">
         <is>
-          <t>4.66</t>
+          <t>4.59</t>
         </is>
       </c>
       <c r="L27" s="7" t="inlineStr">
@@ -2952,32 +2952,32 @@
       </c>
       <c r="M27" s="7" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>10.9%</t>
         </is>
       </c>
       <c r="N27" s="7" t="inlineStr">
         <is>
-          <t>20.5%</t>
+          <t>20.7%</t>
         </is>
       </c>
       <c r="O27" s="7" t="inlineStr">
         <is>
-          <t>68.7%</t>
+          <t>68.4%</t>
         </is>
       </c>
       <c r="P27" s="7" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>17.2%</t>
         </is>
       </c>
       <c r="Q27" s="7" t="inlineStr">
         <is>
-          <t>15.9%</t>
+          <t>17.1%</t>
         </is>
       </c>
       <c r="R27" s="7" t="inlineStr">
         <is>
-          <t>69.2%</t>
+          <t>65.7%</t>
         </is>
       </c>
     </row>
@@ -3027,47 +3027,47 @@
       </c>
       <c r="J28" s="7" t="inlineStr">
         <is>
-          <t>1.76</t>
+          <t>1.78</t>
         </is>
       </c>
       <c r="K28" s="7" t="inlineStr">
         <is>
-          <t>3.70</t>
+          <t>3.73</t>
         </is>
       </c>
       <c r="L28" s="7" t="inlineStr">
         <is>
-          <t>4.60</t>
+          <t>4.50</t>
         </is>
       </c>
       <c r="M28" s="7" t="inlineStr">
         <is>
-          <t>53.8%</t>
+          <t>53.4%</t>
         </is>
       </c>
       <c r="N28" s="7" t="inlineStr">
         <is>
-          <t>25.6%</t>
+          <t>25.5%</t>
         </is>
       </c>
       <c r="O28" s="7" t="inlineStr">
         <is>
-          <t>20.6%</t>
+          <t>21.1%</t>
         </is>
       </c>
       <c r="P28" s="7" t="inlineStr">
         <is>
-          <t>51.3%</t>
+          <t>50.6%</t>
         </is>
       </c>
       <c r="Q28" s="7" t="inlineStr">
         <is>
-          <t>16.0%</t>
+          <t>15.2%</t>
         </is>
       </c>
       <c r="R28" s="7" t="inlineStr">
         <is>
-          <t>32.7%</t>
+          <t>34.2%</t>
         </is>
       </c>
     </row>
@@ -3127,12 +3127,12 @@
       </c>
       <c r="L29" s="7" t="inlineStr">
         <is>
-          <t>5.75</t>
+          <t>5.88</t>
         </is>
       </c>
       <c r="M29" s="7" t="inlineStr">
         <is>
-          <t>59.9%</t>
+          <t>60.1%</t>
         </is>
       </c>
       <c r="N29" s="7" t="inlineStr">
@@ -3142,22 +3142,22 @@
       </c>
       <c r="O29" s="7" t="inlineStr">
         <is>
-          <t>16.5%</t>
+          <t>16.2%</t>
         </is>
       </c>
       <c r="P29" s="7" t="inlineStr">
         <is>
-          <t>75.5%</t>
+          <t>75.3%</t>
         </is>
       </c>
       <c r="Q29" s="7" t="inlineStr">
         <is>
-          <t>11.5%</t>
+          <t>11.1%</t>
         </is>
       </c>
       <c r="R29" s="7" t="inlineStr">
         <is>
-          <t>13.0%</t>
+          <t>13.6%</t>
         </is>
       </c>
     </row>
@@ -3207,47 +3207,47 @@
       </c>
       <c r="J30" s="7" t="inlineStr">
         <is>
-          <t>1.27</t>
+          <t>1.28</t>
         </is>
       </c>
       <c r="K30" s="7" t="inlineStr">
         <is>
-          <t>5.64</t>
+          <t>5.53</t>
         </is>
       </c>
       <c r="L30" s="7" t="inlineStr">
         <is>
-          <t>11.00</t>
+          <t>11.27</t>
         </is>
       </c>
       <c r="M30" s="7" t="inlineStr">
         <is>
-          <t>74.6%</t>
+          <t>74.3%</t>
         </is>
       </c>
       <c r="N30" s="7" t="inlineStr">
         <is>
-          <t>16.8%</t>
+          <t>17.2%</t>
         </is>
       </c>
       <c r="O30" s="7" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>8.4%</t>
         </is>
       </c>
       <c r="P30" s="7" t="inlineStr">
         <is>
-          <t>81.9%</t>
+          <t>80.9%</t>
         </is>
       </c>
       <c r="Q30" s="7" t="inlineStr">
         <is>
-          <t>10.4%</t>
+          <t>10.7%</t>
         </is>
       </c>
       <c r="R30" s="7" t="inlineStr">
         <is>
-          <t>7.7%</t>
+          <t>8.4%</t>
         </is>
       </c>
     </row>
@@ -3297,47 +3297,47 @@
       </c>
       <c r="J31" s="7" t="inlineStr">
         <is>
-          <t>1.97</t>
+          <t>1.98</t>
         </is>
       </c>
       <c r="K31" s="7" t="inlineStr">
         <is>
-          <t>3.28</t>
+          <t>3.30</t>
         </is>
       </c>
       <c r="L31" s="7" t="inlineStr">
         <is>
-          <t>4.16</t>
+          <t>4.09</t>
         </is>
       </c>
       <c r="M31" s="7" t="inlineStr">
         <is>
-          <t>48.2%</t>
+          <t>48.0%</t>
         </is>
       </c>
       <c r="N31" s="7" t="inlineStr">
         <is>
-          <t>29.0%</t>
+          <t>28.8%</t>
         </is>
       </c>
       <c r="O31" s="7" t="inlineStr">
         <is>
-          <t>22.8%</t>
+          <t>23.2%</t>
         </is>
       </c>
       <c r="P31" s="7" t="inlineStr">
         <is>
-          <t>63.8%</t>
+          <t>61.4%</t>
         </is>
       </c>
       <c r="Q31" s="7" t="inlineStr">
         <is>
-          <t>16.5%</t>
+          <t>16.7%</t>
         </is>
       </c>
       <c r="R31" s="7" t="inlineStr">
         <is>
-          <t>19.7%</t>
+          <t>21.9%</t>
         </is>
       </c>
     </row>
@@ -3387,17 +3387,17 @@
       </c>
       <c r="J32" s="7" t="inlineStr">
         <is>
-          <t>1.59</t>
+          <t>1.60</t>
         </is>
       </c>
       <c r="K32" s="7" t="inlineStr">
         <is>
-          <t>4.13</t>
+          <t>4.18</t>
         </is>
       </c>
       <c r="L32" s="7" t="inlineStr">
         <is>
-          <t>5.39</t>
+          <t>5.36</t>
         </is>
       </c>
       <c r="M32" s="7" t="inlineStr">
@@ -3407,27 +3407,27 @@
       </c>
       <c r="N32" s="7" t="inlineStr">
         <is>
-          <t>22.9%</t>
+          <t>22.8%</t>
         </is>
       </c>
       <c r="O32" s="7" t="inlineStr">
         <is>
-          <t>17.6%</t>
+          <t>17.8%</t>
         </is>
       </c>
       <c r="P32" s="7" t="inlineStr">
         <is>
-          <t>53.2%</t>
+          <t>53.3%</t>
         </is>
       </c>
       <c r="Q32" s="7" t="inlineStr">
         <is>
-          <t>16.3%</t>
+          <t>16.9%</t>
         </is>
       </c>
       <c r="R32" s="7" t="inlineStr">
         <is>
-          <t>30.5%</t>
+          <t>29.8%</t>
         </is>
       </c>
     </row>
@@ -3477,7 +3477,7 @@
       </c>
       <c r="J33" s="7" t="inlineStr">
         <is>
-          <t>4.86</t>
+          <t>4.85</t>
         </is>
       </c>
       <c r="K33" s="7" t="inlineStr">
@@ -3487,27 +3487,27 @@
       </c>
       <c r="L33" s="7" t="inlineStr">
         <is>
-          <t>1.76</t>
+          <t>1.77</t>
         </is>
       </c>
       <c r="M33" s="7" t="inlineStr">
         <is>
-          <t>19.5%</t>
+          <t>19.6%</t>
         </is>
       </c>
       <c r="N33" s="7" t="inlineStr">
         <is>
-          <t>26.7%</t>
+          <t>26.8%</t>
         </is>
       </c>
       <c r="O33" s="7" t="inlineStr">
         <is>
-          <t>53.8%</t>
+          <t>53.6%</t>
         </is>
       </c>
       <c r="P33" s="7" t="inlineStr">
         <is>
-          <t>25.5%</t>
+          <t>25.7%</t>
         </is>
       </c>
       <c r="Q33" s="7" t="inlineStr">
@@ -3517,7 +3517,7 @@
       </c>
       <c r="R33" s="7" t="inlineStr">
         <is>
-          <t>58.8%</t>
+          <t>58.6%</t>
         </is>
       </c>
     </row>
@@ -3567,47 +3567,47 @@
       </c>
       <c r="J34" s="7" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>1.10</t>
         </is>
       </c>
       <c r="K34" s="7" t="inlineStr">
         <is>
-          <t>9.94</t>
+          <t>10.04</t>
         </is>
       </c>
       <c r="L34" s="7" t="inlineStr">
         <is>
-          <t>20.13</t>
+          <t>22.25</t>
         </is>
       </c>
       <c r="M34" s="7" t="inlineStr">
         <is>
-          <t>85.7%</t>
+          <t>86.3%</t>
         </is>
       </c>
       <c r="N34" s="7" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.5%</t>
         </is>
       </c>
       <c r="O34" s="7" t="inlineStr">
         <is>
-          <t>4.7%</t>
+          <t>4.3%</t>
         </is>
       </c>
       <c r="P34" s="7" t="inlineStr">
         <is>
-          <t>87.0%</t>
+          <t>87.4%</t>
         </is>
       </c>
       <c r="Q34" s="7" t="inlineStr">
         <is>
-          <t>6.9%</t>
+          <t>6.6%</t>
         </is>
       </c>
       <c r="R34" s="7" t="inlineStr">
         <is>
-          <t>6.1%</t>
+          <t>5.9%</t>
         </is>
       </c>
     </row>
@@ -3657,47 +3657,47 @@
       </c>
       <c r="J35" s="7" t="inlineStr">
         <is>
-          <t>2.00</t>
+          <t>2.04</t>
         </is>
       </c>
       <c r="K35" s="7" t="inlineStr">
         <is>
-          <t>3.30</t>
+          <t>3.28</t>
         </is>
       </c>
       <c r="L35" s="7" t="inlineStr">
         <is>
-          <t>3.97</t>
+          <t>3.90</t>
         </is>
       </c>
       <c r="M35" s="7" t="inlineStr">
         <is>
-          <t>47.4%</t>
+          <t>46.6%</t>
         </is>
       </c>
       <c r="N35" s="7" t="inlineStr">
         <is>
-          <t>28.7%</t>
+          <t>29.0%</t>
         </is>
       </c>
       <c r="O35" s="7" t="inlineStr">
         <is>
-          <t>23.9%</t>
+          <t>24.4%</t>
         </is>
       </c>
       <c r="P35" s="7" t="inlineStr">
         <is>
-          <t>39.7%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="Q35" s="7" t="inlineStr">
         <is>
-          <t>16.2%</t>
+          <t>14.9%</t>
         </is>
       </c>
       <c r="R35" s="7" t="inlineStr">
         <is>
-          <t>44.1%</t>
+          <t>45.1%</t>
         </is>
       </c>
     </row>
@@ -3752,42 +3752,42 @@
       </c>
       <c r="K36" s="7" t="inlineStr">
         <is>
-          <t>3.93</t>
+          <t>4.01</t>
         </is>
       </c>
       <c r="L36" s="7" t="inlineStr">
         <is>
-          <t>4.96</t>
+          <t>5.19</t>
         </is>
       </c>
       <c r="M36" s="7" t="inlineStr">
         <is>
-          <t>57.4%</t>
+          <t>58.1%</t>
         </is>
       </c>
       <c r="N36" s="7" t="inlineStr">
         <is>
-          <t>23.8%</t>
+          <t>23.6%</t>
         </is>
       </c>
       <c r="O36" s="7" t="inlineStr">
         <is>
-          <t>18.9%</t>
+          <t>18.3%</t>
         </is>
       </c>
       <c r="P36" s="7" t="inlineStr">
         <is>
-          <t>69.9%</t>
+          <t>67.7%</t>
         </is>
       </c>
       <c r="Q36" s="7" t="inlineStr">
         <is>
-          <t>12.1%</t>
+          <t>12.8%</t>
         </is>
       </c>
       <c r="R36" s="7" t="inlineStr">
         <is>
-          <t>18.0%</t>
+          <t>19.5%</t>
         </is>
       </c>
     </row>
@@ -3837,27 +3837,27 @@
       </c>
       <c r="J37" s="7" t="inlineStr">
         <is>
-          <t>1.53</t>
+          <t>1.55</t>
         </is>
       </c>
       <c r="K37" s="7" t="inlineStr">
         <is>
-          <t>4.18</t>
+          <t>4.26</t>
         </is>
       </c>
       <c r="L37" s="7" t="inlineStr">
         <is>
-          <t>5.56</t>
+          <t>5.62</t>
         </is>
       </c>
       <c r="M37" s="7" t="inlineStr">
         <is>
-          <t>60.9%</t>
+          <t>61.0%</t>
         </is>
       </c>
       <c r="N37" s="7" t="inlineStr">
         <is>
-          <t>22.3%</t>
+          <t>22.2%</t>
         </is>
       </c>
       <c r="O37" s="7" t="inlineStr">
@@ -3867,17 +3867,17 @@
       </c>
       <c r="P37" s="7" t="inlineStr">
         <is>
-          <t>69.7%</t>
+          <t>69.2%</t>
         </is>
       </c>
       <c r="Q37" s="7" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>13.7%</t>
         </is>
       </c>
       <c r="R37" s="7" t="inlineStr">
         <is>
-          <t>17.8%</t>
+          <t>17.2%</t>
         </is>
       </c>
     </row>
@@ -3932,17 +3932,17 @@
       </c>
       <c r="K38" s="7" t="inlineStr">
         <is>
-          <t>6.81</t>
+          <t>6.90</t>
         </is>
       </c>
       <c r="L38" s="7" t="inlineStr">
         <is>
-          <t>12.50</t>
+          <t>15.28</t>
         </is>
       </c>
       <c r="M38" s="7" t="inlineStr">
         <is>
-          <t>78.7%</t>
+          <t>80.0%</t>
         </is>
       </c>
       <c r="N38" s="7" t="inlineStr">
@@ -3952,22 +3952,22 @@
       </c>
       <c r="O38" s="7" t="inlineStr">
         <is>
-          <t>7.5%</t>
+          <t>6.2%</t>
         </is>
       </c>
       <c r="P38" s="7" t="inlineStr">
         <is>
-          <t>86.4%</t>
+          <t>87.8%</t>
         </is>
       </c>
       <c r="Q38" s="7" t="inlineStr">
         <is>
-          <t>6.7%</t>
+          <t>5.6%</t>
         </is>
       </c>
       <c r="R38" s="7" t="inlineStr">
         <is>
-          <t>6.8%</t>
+          <t>6.6%</t>
         </is>
       </c>
     </row>
@@ -4017,47 +4017,47 @@
       </c>
       <c r="J39" s="7" t="inlineStr">
         <is>
-          <t>5.29</t>
+          <t>5.42</t>
         </is>
       </c>
       <c r="K39" s="7" t="inlineStr">
         <is>
-          <t>3.51</t>
+          <t>3.60</t>
         </is>
       </c>
       <c r="L39" s="7" t="inlineStr">
         <is>
-          <t>1.67</t>
+          <t>1.69</t>
         </is>
       </c>
       <c r="M39" s="7" t="inlineStr">
         <is>
-          <t>17.6%</t>
+          <t>17.5%</t>
         </is>
       </c>
       <c r="N39" s="7" t="inlineStr">
         <is>
-          <t>26.6%</t>
+          <t>26.4%</t>
         </is>
       </c>
       <c r="O39" s="7" t="inlineStr">
         <is>
-          <t>55.8%</t>
+          <t>56.1%</t>
         </is>
       </c>
       <c r="P39" s="7" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>17.2%</t>
         </is>
       </c>
       <c r="Q39" s="7" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>16.4%</t>
         </is>
       </c>
       <c r="R39" s="7" t="inlineStr">
         <is>
-          <t>66.5%</t>
+          <t>66.4%</t>
         </is>
       </c>
     </row>
@@ -4112,42 +4112,42 @@
       </c>
       <c r="K40" s="7" t="inlineStr">
         <is>
-          <t>9.63</t>
+          <t>9.30</t>
         </is>
       </c>
       <c r="L40" s="7" t="inlineStr">
         <is>
-          <t>21.63</t>
+          <t>24.32</t>
         </is>
       </c>
       <c r="M40" s="7" t="inlineStr">
         <is>
-          <t>85.8%</t>
+          <t>85.9%</t>
         </is>
       </c>
       <c r="N40" s="7" t="inlineStr">
         <is>
-          <t>9.8%</t>
+          <t>10.2%</t>
         </is>
       </c>
       <c r="O40" s="7" t="inlineStr">
         <is>
-          <t>4.4%</t>
+          <t>3.9%</t>
         </is>
       </c>
       <c r="P40" s="7" t="inlineStr">
         <is>
-          <t>89.4%</t>
+          <t>89.0%</t>
         </is>
       </c>
       <c r="Q40" s="7" t="inlineStr">
         <is>
-          <t>6.7%</t>
+          <t>7.0%</t>
         </is>
       </c>
       <c r="R40" s="7" t="inlineStr">
         <is>
-          <t>3.9%</t>
+          <t>4.0%</t>
         </is>
       </c>
     </row>
@@ -4197,47 +4197,47 @@
       </c>
       <c r="J41" s="7" t="inlineStr">
         <is>
-          <t>1.39</t>
+          <t>1.40</t>
         </is>
       </c>
       <c r="K41" s="7" t="inlineStr">
         <is>
-          <t>4.65</t>
+          <t>4.58</t>
         </is>
       </c>
       <c r="L41" s="7" t="inlineStr">
         <is>
-          <t>7.56</t>
+          <t>7.76</t>
         </is>
       </c>
       <c r="M41" s="7" t="inlineStr">
         <is>
-          <t>67.4%</t>
+          <t>67.3%</t>
         </is>
       </c>
       <c r="N41" s="7" t="inlineStr">
         <is>
-          <t>20.2%</t>
+          <t>20.6%</t>
         </is>
       </c>
       <c r="O41" s="7" t="inlineStr">
         <is>
-          <t>12.4%</t>
+          <t>12.1%</t>
         </is>
       </c>
       <c r="P41" s="7" t="inlineStr">
         <is>
-          <t>45.3%</t>
+          <t>49.6%</t>
         </is>
       </c>
       <c r="Q41" s="7" t="inlineStr">
         <is>
-          <t>13.4%</t>
+          <t>12.9%</t>
         </is>
       </c>
       <c r="R41" s="7" t="inlineStr">
         <is>
-          <t>41.2%</t>
+          <t>37.5%</t>
         </is>
       </c>
     </row>
@@ -4292,42 +4292,42 @@
       </c>
       <c r="K42" s="7" t="inlineStr">
         <is>
-          <t>4.41</t>
+          <t>4.37</t>
         </is>
       </c>
       <c r="L42" s="7" t="inlineStr">
         <is>
-          <t>7.06</t>
+          <t>7.35</t>
         </is>
       </c>
       <c r="M42" s="7" t="inlineStr">
         <is>
-          <t>65.5%</t>
+          <t>65.7%</t>
         </is>
       </c>
       <c r="N42" s="7" t="inlineStr">
         <is>
-          <t>21.2%</t>
+          <t>21.5%</t>
         </is>
       </c>
       <c r="O42" s="7" t="inlineStr">
         <is>
-          <t>13.3%</t>
+          <t>12.8%</t>
         </is>
       </c>
       <c r="P42" s="7" t="inlineStr">
         <is>
-          <t>85.7%</t>
+          <t>84.6%</t>
         </is>
       </c>
       <c r="Q42" s="7" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>8.8%</t>
         </is>
       </c>
       <c r="R42" s="7" t="inlineStr">
         <is>
-          <t>6.0%</t>
+          <t>6.6%</t>
         </is>
       </c>
     </row>
@@ -4377,47 +4377,47 @@
       </c>
       <c r="J43" s="7" t="inlineStr">
         <is>
-          <t>4.75</t>
+          <t>4.66</t>
         </is>
       </c>
       <c r="K43" s="7" t="inlineStr">
         <is>
-          <t>3.60</t>
+          <t>3.69</t>
         </is>
       </c>
       <c r="L43" s="7" t="inlineStr">
         <is>
-          <t>1.73</t>
+          <t>1.74</t>
         </is>
       </c>
       <c r="M43" s="7" t="inlineStr">
         <is>
-          <t>19.7%</t>
+          <t>20.2%</t>
         </is>
       </c>
       <c r="N43" s="7" t="inlineStr">
         <is>
+          <t>25.6%</t>
+        </is>
+      </c>
+      <c r="O43" s="7" t="inlineStr">
+        <is>
+          <t>54.2%</t>
+        </is>
+      </c>
+      <c r="P43" s="7" t="inlineStr">
+        <is>
           <t>26.0%</t>
         </is>
       </c>
-      <c r="O43" s="7" t="inlineStr">
-        <is>
-          <t>54.2%</t>
-        </is>
-      </c>
-      <c r="P43" s="7" t="inlineStr">
-        <is>
-          <t>25.5%</t>
-        </is>
-      </c>
       <c r="Q43" s="7" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>16.6%</t>
         </is>
       </c>
       <c r="R43" s="7" t="inlineStr">
         <is>
-          <t>57.1%</t>
+          <t>57.4%</t>
         </is>
       </c>
     </row>
@@ -4472,37 +4472,37 @@
       </c>
       <c r="K44" s="7" t="inlineStr">
         <is>
-          <t>3.78</t>
+          <t>3.77</t>
         </is>
       </c>
       <c r="L44" s="7" t="inlineStr">
         <is>
-          <t>5.41</t>
+          <t>5.60</t>
         </is>
       </c>
       <c r="M44" s="7" t="inlineStr">
         <is>
-          <t>58.0%</t>
+          <t>58.3%</t>
         </is>
       </c>
       <c r="N44" s="7" t="inlineStr">
         <is>
-          <t>24.7%</t>
+          <t>24.9%</t>
         </is>
       </c>
       <c r="O44" s="7" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>16.8%</t>
         </is>
       </c>
       <c r="P44" s="7" t="inlineStr">
         <is>
-          <t>73.5%</t>
+          <t>73.3%</t>
         </is>
       </c>
       <c r="Q44" s="7" t="inlineStr">
         <is>
-          <t>11.3%</t>
+          <t>11.5%</t>
         </is>
       </c>
       <c r="R44" s="7" t="inlineStr">
@@ -4562,12 +4562,12 @@
       </c>
       <c r="K45" s="7" t="inlineStr">
         <is>
-          <t>8.81</t>
+          <t>8.37</t>
         </is>
       </c>
       <c r="L45" s="7" t="inlineStr">
         <is>
-          <t>21.88</t>
+          <t>25.04</t>
         </is>
       </c>
       <c r="M45" s="7" t="inlineStr">
@@ -4577,27 +4577,27 @@
       </c>
       <c r="N45" s="7" t="inlineStr">
         <is>
-          <t>10.7%</t>
+          <t>11.3%</t>
         </is>
       </c>
       <c r="O45" s="7" t="inlineStr">
         <is>
-          <t>4.3%</t>
+          <t>3.8%</t>
         </is>
       </c>
       <c r="P45" s="7" t="inlineStr">
         <is>
-          <t>81.5%</t>
+          <t>81.4%</t>
         </is>
       </c>
       <c r="Q45" s="7" t="inlineStr">
         <is>
-          <t>9.3%</t>
+          <t>8.8%</t>
         </is>
       </c>
       <c r="R45" s="7" t="inlineStr">
         <is>
-          <t>9.2%</t>
+          <t>9.9%</t>
         </is>
       </c>
     </row>
@@ -4647,27 +4647,27 @@
       </c>
       <c r="J46" s="7" t="inlineStr">
         <is>
-          <t>2.10</t>
+          <t>2.11</t>
         </is>
       </c>
       <c r="K46" s="7" t="inlineStr">
         <is>
-          <t>3.38</t>
+          <t>3.43</t>
         </is>
       </c>
       <c r="L46" s="7" t="inlineStr">
         <is>
-          <t>3.35</t>
+          <t>3.37</t>
         </is>
       </c>
       <c r="M46" s="7" t="inlineStr">
         <is>
-          <t>44.5%</t>
+          <t>44.6%</t>
         </is>
       </c>
       <c r="N46" s="7" t="inlineStr">
         <is>
-          <t>27.6%</t>
+          <t>27.4%</t>
         </is>
       </c>
       <c r="O46" s="7" t="inlineStr">
@@ -4677,17 +4677,17 @@
       </c>
       <c r="P46" s="7" t="inlineStr">
         <is>
-          <t>45.5%</t>
+          <t>44.1%</t>
         </is>
       </c>
       <c r="Q46" s="7" t="inlineStr">
         <is>
-          <t>16.1%</t>
+          <t>15.8%</t>
         </is>
       </c>
       <c r="R46" s="7" t="inlineStr">
         <is>
-          <t>38.4%</t>
+          <t>40.1%</t>
         </is>
       </c>
     </row>
@@ -4737,17 +4737,17 @@
       </c>
       <c r="J47" s="7" t="inlineStr">
         <is>
-          <t>6.69</t>
+          <t>6.68</t>
         </is>
       </c>
       <c r="K47" s="7" t="inlineStr">
         <is>
-          <t>4.05</t>
+          <t>4.12</t>
         </is>
       </c>
       <c r="L47" s="7" t="inlineStr">
         <is>
-          <t>1.50</t>
+          <t>1.49</t>
         </is>
       </c>
       <c r="M47" s="7" t="inlineStr">
@@ -4757,27 +4757,27 @@
       </c>
       <c r="N47" s="7" t="inlineStr">
         <is>
-          <t>23.2%</t>
+          <t>22.8%</t>
         </is>
       </c>
       <c r="O47" s="7" t="inlineStr">
         <is>
-          <t>62.7%</t>
+          <t>63.1%</t>
         </is>
       </c>
       <c r="P47" s="7" t="inlineStr">
         <is>
-          <t>25.9%</t>
+          <t>26.5%</t>
         </is>
       </c>
       <c r="Q47" s="7" t="inlineStr">
         <is>
-          <t>16.5%</t>
+          <t>14.9%</t>
         </is>
       </c>
       <c r="R47" s="7" t="inlineStr">
         <is>
-          <t>57.6%</t>
+          <t>58.6%</t>
         </is>
       </c>
     </row>
@@ -4832,42 +4832,42 @@
       </c>
       <c r="K48" s="7" t="inlineStr">
         <is>
-          <t>6.13</t>
+          <t>6.12</t>
         </is>
       </c>
       <c r="L48" s="7" t="inlineStr">
         <is>
-          <t>10.25</t>
+          <t>11.30</t>
         </is>
       </c>
       <c r="M48" s="7" t="inlineStr">
         <is>
-          <t>75.6%</t>
+          <t>76.2%</t>
         </is>
       </c>
       <c r="N48" s="7" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>15.4%</t>
         </is>
       </c>
       <c r="O48" s="7" t="inlineStr">
         <is>
-          <t>9.1%</t>
+          <t>8.4%</t>
         </is>
       </c>
       <c r="P48" s="7" t="inlineStr">
         <is>
-          <t>67.8%</t>
+          <t>67.2%</t>
         </is>
       </c>
       <c r="Q48" s="7" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>18.2%</t>
         </is>
       </c>
       <c r="R48" s="7" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>14.6%</t>
         </is>
       </c>
     </row>
@@ -4922,22 +4922,22 @@
       </c>
       <c r="K49" s="7" t="inlineStr">
         <is>
-          <t>5.10</t>
+          <t>5.17</t>
         </is>
       </c>
       <c r="L49" s="7" t="inlineStr">
         <is>
-          <t>9.25</t>
+          <t>9.28</t>
         </is>
       </c>
       <c r="M49" s="7" t="inlineStr">
         <is>
-          <t>71.5%</t>
+          <t>71.7%</t>
         </is>
       </c>
       <c r="N49" s="7" t="inlineStr">
         <is>
-          <t>18.4%</t>
+          <t>18.2%</t>
         </is>
       </c>
       <c r="O49" s="7" t="inlineStr">
@@ -4947,17 +4947,17 @@
       </c>
       <c r="P49" s="7" t="inlineStr">
         <is>
-          <t>87.4%</t>
+          <t>88.0%</t>
         </is>
       </c>
       <c r="Q49" s="7" t="inlineStr">
         <is>
-          <t>7.7%</t>
+          <t>6.9%</t>
         </is>
       </c>
       <c r="R49" s="7" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>5.1%</t>
         </is>
       </c>
     </row>
@@ -5012,42 +5012,42 @@
       </c>
       <c r="K50" s="7" t="inlineStr">
         <is>
-          <t>3.93</t>
+          <t>3.86</t>
         </is>
       </c>
       <c r="L50" s="7" t="inlineStr">
         <is>
-          <t>1.52</t>
+          <t>1.55</t>
         </is>
       </c>
       <c r="M50" s="7" t="inlineStr">
         <is>
-          <t>14.8%</t>
+          <t>14.9%</t>
         </is>
       </c>
       <c r="N50" s="7" t="inlineStr">
         <is>
-          <t>23.8%</t>
+          <t>24.4%</t>
         </is>
       </c>
       <c r="O50" s="7" t="inlineStr">
         <is>
-          <t>61.4%</t>
+          <t>60.7%</t>
         </is>
       </c>
       <c r="P50" s="7" t="inlineStr">
         <is>
-          <t>20.1%</t>
+          <t>21.1%</t>
         </is>
       </c>
       <c r="Q50" s="7" t="inlineStr">
         <is>
-          <t>17.7%</t>
+          <t>19.1%</t>
         </is>
       </c>
       <c r="R50" s="7" t="inlineStr">
         <is>
-          <t>62.2%</t>
+          <t>59.7%</t>
         </is>
       </c>
     </row>
@@ -5097,47 +5097,47 @@
       </c>
       <c r="J51" s="7" t="inlineStr">
         <is>
-          <t>1.46</t>
+          <t>1.45</t>
         </is>
       </c>
       <c r="K51" s="7" t="inlineStr">
         <is>
-          <t>4.15</t>
+          <t>4.22</t>
         </is>
       </c>
       <c r="L51" s="7" t="inlineStr">
         <is>
-          <t>7.06</t>
+          <t>7.43</t>
         </is>
       </c>
       <c r="M51" s="7" t="inlineStr">
         <is>
-          <t>64.2%</t>
+          <t>65.0%</t>
         </is>
       </c>
       <c r="N51" s="7" t="inlineStr">
         <is>
-          <t>22.6%</t>
+          <t>22.3%</t>
         </is>
       </c>
       <c r="O51" s="7" t="inlineStr">
         <is>
-          <t>13.3%</t>
+          <t>12.7%</t>
         </is>
       </c>
       <c r="P51" s="7" t="inlineStr">
         <is>
-          <t>79.6%</t>
+          <t>79.5%</t>
         </is>
       </c>
       <c r="Q51" s="7" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.8%</t>
         </is>
       </c>
       <c r="R51" s="7" t="inlineStr">
         <is>
-          <t>10.8%</t>
+          <t>10.7%</t>
         </is>
       </c>
     </row>
@@ -5187,7 +5187,7 @@
       </c>
       <c r="J52" s="7" t="inlineStr">
         <is>
-          <t>2.09</t>
+          <t>2.10</t>
         </is>
       </c>
       <c r="K52" s="7" t="inlineStr">
@@ -5197,7 +5197,7 @@
       </c>
       <c r="L52" s="7" t="inlineStr">
         <is>
-          <t>3.46</t>
+          <t>3.47</t>
         </is>
       </c>
       <c r="M52" s="7" t="inlineStr">
@@ -5207,7 +5207,7 @@
       </c>
       <c r="N52" s="7" t="inlineStr">
         <is>
-          <t>28.2%</t>
+          <t>28.3%</t>
         </is>
       </c>
       <c r="O52" s="7" t="inlineStr">
@@ -5217,17 +5217,17 @@
       </c>
       <c r="P52" s="7" t="inlineStr">
         <is>
-          <t>58.7%</t>
+          <t>57.4%</t>
         </is>
       </c>
       <c r="Q52" s="7" t="inlineStr">
         <is>
-          <t>11.9%</t>
+          <t>12.8%</t>
         </is>
       </c>
       <c r="R52" s="7" t="inlineStr">
         <is>
-          <t>29.4%</t>
+          <t>29.8%</t>
         </is>
       </c>
     </row>
@@ -5277,47 +5277,47 @@
       </c>
       <c r="J53" s="7" t="inlineStr">
         <is>
-          <t>1.52</t>
+          <t>1.54</t>
         </is>
       </c>
       <c r="K53" s="7" t="inlineStr">
         <is>
-          <t>4.01</t>
+          <t>3.95</t>
         </is>
       </c>
       <c r="L53" s="7" t="inlineStr">
         <is>
-          <t>6.25</t>
+          <t>6.17</t>
         </is>
       </c>
       <c r="M53" s="7" t="inlineStr">
         <is>
-          <t>61.6%</t>
+          <t>61.0%</t>
         </is>
       </c>
       <c r="N53" s="7" t="inlineStr">
         <is>
-          <t>23.4%</t>
+          <t>23.8%</t>
         </is>
       </c>
       <c r="O53" s="7" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>15.2%</t>
         </is>
       </c>
       <c r="P53" s="7" t="inlineStr">
         <is>
-          <t>41.1%</t>
+          <t>39.0%</t>
         </is>
       </c>
       <c r="Q53" s="7" t="inlineStr">
         <is>
-          <t>17.3%</t>
+          <t>17.1%</t>
         </is>
       </c>
       <c r="R53" s="7" t="inlineStr">
         <is>
-          <t>41.6%</t>
+          <t>43.8%</t>
         </is>
       </c>
     </row>
@@ -5367,17 +5367,17 @@
       </c>
       <c r="J54" s="7" t="inlineStr">
         <is>
-          <t>6.63</t>
+          <t>6.72</t>
         </is>
       </c>
       <c r="K54" s="7" t="inlineStr">
         <is>
-          <t>4.83</t>
+          <t>4.75</t>
         </is>
       </c>
       <c r="L54" s="7" t="inlineStr">
         <is>
-          <t>1.40</t>
+          <t>1.43</t>
         </is>
       </c>
       <c r="M54" s="7" t="inlineStr">
@@ -5387,22 +5387,22 @@
       </c>
       <c r="N54" s="7" t="inlineStr">
         <is>
-          <t>19.3%</t>
+          <t>19.9%</t>
         </is>
       </c>
       <c r="O54" s="7" t="inlineStr">
         <is>
-          <t>66.6%</t>
+          <t>66.1%</t>
         </is>
       </c>
       <c r="P54" s="7" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.4%</t>
         </is>
       </c>
       <c r="Q54" s="7" t="inlineStr">
         <is>
-          <t>13.1%</t>
+          <t>13.0%</t>
         </is>
       </c>
       <c r="R54" s="7" t="inlineStr">
@@ -5457,47 +5457,47 @@
       </c>
       <c r="J55" s="7" t="inlineStr">
         <is>
-          <t>1.30</t>
+          <t>1.29</t>
         </is>
       </c>
       <c r="K55" s="7" t="inlineStr">
         <is>
-          <t>5.28</t>
+          <t>5.33</t>
         </is>
       </c>
       <c r="L55" s="7" t="inlineStr">
         <is>
-          <t>9.50</t>
+          <t>9.83</t>
         </is>
       </c>
       <c r="M55" s="7" t="inlineStr">
         <is>
-          <t>72.3%</t>
+          <t>72.8%</t>
         </is>
       </c>
       <c r="N55" s="7" t="inlineStr">
         <is>
-          <t>17.8%</t>
+          <t>17.6%</t>
         </is>
       </c>
       <c r="O55" s="7" t="inlineStr">
         <is>
-          <t>9.9%</t>
+          <t>9.6%</t>
         </is>
       </c>
       <c r="P55" s="7" t="inlineStr">
         <is>
-          <t>80.8%</t>
+          <t>81.5%</t>
         </is>
       </c>
       <c r="Q55" s="7" t="inlineStr">
         <is>
-          <t>9.5%</t>
+          <t>9.1%</t>
         </is>
       </c>
       <c r="R55" s="7" t="inlineStr">
         <is>
-          <t>9.7%</t>
+          <t>9.4%</t>
         </is>
       </c>
     </row>
@@ -5547,12 +5547,12 @@
       </c>
       <c r="J56" s="7" t="inlineStr">
         <is>
-          <t>4.51</t>
+          <t>4.50</t>
         </is>
       </c>
       <c r="K56" s="7" t="inlineStr">
         <is>
-          <t>3.48</t>
+          <t>3.49</t>
         </is>
       </c>
       <c r="L56" s="7" t="inlineStr">
@@ -5562,12 +5562,12 @@
       </c>
       <c r="M56" s="7" t="inlineStr">
         <is>
-          <t>20.8%</t>
+          <t>20.9%</t>
         </is>
       </c>
       <c r="N56" s="7" t="inlineStr">
         <is>
-          <t>27.0%</t>
+          <t>26.9%</t>
         </is>
       </c>
       <c r="O56" s="7" t="inlineStr">
@@ -5577,17 +5577,17 @@
       </c>
       <c r="P56" s="7" t="inlineStr">
         <is>
-          <t>24.6%</t>
+          <t>25.5%</t>
         </is>
       </c>
       <c r="Q56" s="7" t="inlineStr">
         <is>
-          <t>14.7%</t>
+          <t>15.6%</t>
         </is>
       </c>
       <c r="R56" s="7" t="inlineStr">
         <is>
-          <t>60.6%</t>
+          <t>58.9%</t>
         </is>
       </c>
     </row>
@@ -5637,47 +5637,47 @@
       </c>
       <c r="J57" s="7" t="inlineStr">
         <is>
-          <t>5.46</t>
+          <t>5.41</t>
         </is>
       </c>
       <c r="K57" s="7" t="inlineStr">
         <is>
-          <t>3.93</t>
+          <t>3.84</t>
         </is>
       </c>
       <c r="L57" s="7" t="inlineStr">
         <is>
-          <t>1.59</t>
+          <t>1.60</t>
         </is>
       </c>
       <c r="M57" s="7" t="inlineStr">
         <is>
-          <t>17.2%</t>
+          <t>17.3%</t>
         </is>
       </c>
       <c r="N57" s="7" t="inlineStr">
         <is>
-          <t>23.9%</t>
+          <t>24.3%</t>
         </is>
       </c>
       <c r="O57" s="7" t="inlineStr">
         <is>
-          <t>59.0%</t>
+          <t>58.4%</t>
         </is>
       </c>
       <c r="P57" s="7" t="inlineStr">
         <is>
-          <t>19.4%</t>
+          <t>18.1%</t>
         </is>
       </c>
       <c r="Q57" s="7" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>17.6%</t>
         </is>
       </c>
       <c r="R57" s="7" t="inlineStr">
         <is>
-          <t>63.2%</t>
+          <t>64.3%</t>
         </is>
       </c>
     </row>
@@ -5727,12 +5727,12 @@
       </c>
       <c r="J58" s="7" t="inlineStr">
         <is>
-          <t>12.50</t>
+          <t>12.65</t>
         </is>
       </c>
       <c r="K58" s="7" t="inlineStr">
         <is>
-          <t>6.31</t>
+          <t>6.27</t>
         </is>
       </c>
       <c r="L58" s="7" t="inlineStr">
@@ -5742,12 +5742,12 @@
       </c>
       <c r="M58" s="7" t="inlineStr">
         <is>
-          <t>7.6%</t>
+          <t>7.5%</t>
         </is>
       </c>
       <c r="N58" s="7" t="inlineStr">
         <is>
-          <t>15.0%</t>
+          <t>15.1%</t>
         </is>
       </c>
       <c r="O58" s="7" t="inlineStr">
@@ -5757,17 +5757,17 @@
       </c>
       <c r="P58" s="7" t="inlineStr">
         <is>
-          <t>20.6%</t>
+          <t>22.1%</t>
         </is>
       </c>
       <c r="Q58" s="7" t="inlineStr">
         <is>
-          <t>18.6%</t>
+          <t>18.4%</t>
         </is>
       </c>
       <c r="R58" s="7" t="inlineStr">
         <is>
-          <t>60.7%</t>
+          <t>59.5%</t>
         </is>
       </c>
     </row>
@@ -5817,32 +5817,32 @@
       </c>
       <c r="J59" s="7" t="inlineStr">
         <is>
-          <t>4.85</t>
+          <t>4.61</t>
         </is>
       </c>
       <c r="K59" s="7" t="inlineStr">
         <is>
-          <t>3.75</t>
+          <t>3.70</t>
         </is>
       </c>
       <c r="L59" s="7" t="inlineStr">
         <is>
-          <t>1.69</t>
+          <t>1.73</t>
         </is>
       </c>
       <c r="M59" s="7" t="inlineStr">
         <is>
-          <t>19.4%</t>
+          <t>20.4%</t>
         </is>
       </c>
       <c r="N59" s="7" t="inlineStr">
         <is>
-          <t>25.0%</t>
+          <t>25.4%</t>
         </is>
       </c>
       <c r="O59" s="7" t="inlineStr">
         <is>
-          <t>55.6%</t>
+          <t>54.3%</t>
         </is>
       </c>
       <c r="P59" s="7" t="inlineStr">
@@ -5852,12 +5852,12 @@
       </c>
       <c r="Q59" s="7" t="inlineStr">
         <is>
-          <t>17.2%</t>
+          <t>16.5%</t>
         </is>
       </c>
       <c r="R59" s="7" t="inlineStr">
         <is>
-          <t>51.0%</t>
+          <t>51.8%</t>
         </is>
       </c>
     </row>
@@ -5907,27 +5907,27 @@
       </c>
       <c r="J60" s="7" t="inlineStr">
         <is>
-          <t>2.05</t>
+          <t>2.07</t>
         </is>
       </c>
       <c r="K60" s="7" t="inlineStr">
         <is>
-          <t>3.36</t>
+          <t>3.35</t>
         </is>
       </c>
       <c r="L60" s="7" t="inlineStr">
         <is>
-          <t>3.48</t>
+          <t>3.50</t>
         </is>
       </c>
       <c r="M60" s="7" t="inlineStr">
         <is>
-          <t>45.5%</t>
+          <t>45.3%</t>
         </is>
       </c>
       <c r="N60" s="7" t="inlineStr">
         <is>
-          <t>27.7%</t>
+          <t>28.0%</t>
         </is>
       </c>
       <c r="O60" s="7" t="inlineStr">
@@ -5937,17 +5937,17 @@
       </c>
       <c r="P60" s="7" t="inlineStr">
         <is>
-          <t>70.5%</t>
+          <t>67.5%</t>
         </is>
       </c>
       <c r="Q60" s="7" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>11.2%</t>
         </is>
       </c>
       <c r="R60" s="7" t="inlineStr">
         <is>
-          <t>19.0%</t>
+          <t>21.3%</t>
         </is>
       </c>
     </row>
@@ -5997,47 +5997,47 @@
       </c>
       <c r="J61" s="7" t="inlineStr">
         <is>
-          <t>6.19</t>
+          <t>6.48</t>
         </is>
       </c>
       <c r="K61" s="7" t="inlineStr">
         <is>
-          <t>4.15</t>
+          <t>4.22</t>
         </is>
       </c>
       <c r="L61" s="7" t="inlineStr">
         <is>
-          <t>1.50</t>
+          <t>1.48</t>
         </is>
       </c>
       <c r="M61" s="7" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>14.5%</t>
         </is>
       </c>
       <c r="N61" s="7" t="inlineStr">
         <is>
-          <t>22.5%</t>
+          <t>22.2%</t>
         </is>
       </c>
       <c r="O61" s="7" t="inlineStr">
         <is>
-          <t>62.4%</t>
+          <t>63.3%</t>
         </is>
       </c>
       <c r="P61" s="7" t="inlineStr">
         <is>
-          <t>15.5%</t>
+          <t>14.9%</t>
         </is>
       </c>
       <c r="Q61" s="7" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>13.6%</t>
         </is>
       </c>
       <c r="R61" s="7" t="inlineStr">
         <is>
-          <t>69.6%</t>
+          <t>71.5%</t>
         </is>
       </c>
     </row>
@@ -6087,47 +6087,47 @@
       </c>
       <c r="J62" s="7" t="inlineStr">
         <is>
-          <t>2.68</t>
+          <t>2.70</t>
         </is>
       </c>
       <c r="K62" s="7" t="inlineStr">
         <is>
-          <t>3.48</t>
+          <t>3.54</t>
         </is>
       </c>
       <c r="L62" s="7" t="inlineStr">
         <is>
-          <t>2.44</t>
+          <t>2.42</t>
         </is>
       </c>
       <c r="M62" s="7" t="inlineStr">
         <is>
-          <t>34.9%</t>
+          <t>34.7%</t>
         </is>
       </c>
       <c r="N62" s="7" t="inlineStr">
         <is>
-          <t>26.8%</t>
+          <t>26.5%</t>
         </is>
       </c>
       <c r="O62" s="7" t="inlineStr">
         <is>
-          <t>38.3%</t>
+          <t>38.8%</t>
         </is>
       </c>
       <c r="P62" s="7" t="inlineStr">
         <is>
-          <t>58.5%</t>
+          <t>59.4%</t>
         </is>
       </c>
       <c r="Q62" s="7" t="inlineStr">
         <is>
-          <t>14.2%</t>
+          <t>13.4%</t>
         </is>
       </c>
       <c r="R62" s="7" t="inlineStr">
         <is>
-          <t>27.3%</t>
+          <t>27.2%</t>
         </is>
       </c>
     </row>
@@ -6177,17 +6177,17 @@
       </c>
       <c r="J63" s="7" t="inlineStr">
         <is>
-          <t>2.11</t>
+          <t>2.13</t>
         </is>
       </c>
       <c r="K63" s="7" t="inlineStr">
         <is>
-          <t>3.21</t>
+          <t>3.23</t>
         </is>
       </c>
       <c r="L63" s="7" t="inlineStr">
         <is>
-          <t>3.46</t>
+          <t>3.50</t>
         </is>
       </c>
       <c r="M63" s="7" t="inlineStr">
@@ -6197,27 +6197,27 @@
       </c>
       <c r="N63" s="7" t="inlineStr">
         <is>
-          <t>29.0%</t>
+          <t>29.1%</t>
         </is>
       </c>
       <c r="O63" s="7" t="inlineStr">
         <is>
-          <t>26.9%</t>
+          <t>26.8%</t>
         </is>
       </c>
       <c r="P63" s="7" t="inlineStr">
         <is>
-          <t>37.9%</t>
+          <t>37.6%</t>
         </is>
       </c>
       <c r="Q63" s="7" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>18.4%</t>
         </is>
       </c>
       <c r="R63" s="7" t="inlineStr">
         <is>
-          <t>45.0%</t>
+          <t>44.1%</t>
         </is>
       </c>
     </row>
@@ -6267,17 +6267,17 @@
       </c>
       <c r="J64" s="7" t="inlineStr">
         <is>
-          <t>4.20</t>
+          <t>4.23</t>
         </is>
       </c>
       <c r="K64" s="7" t="inlineStr">
         <is>
-          <t>3.56</t>
+          <t>3.55</t>
         </is>
       </c>
       <c r="L64" s="7" t="inlineStr">
         <is>
-          <t>1.81</t>
+          <t>1.83</t>
         </is>
       </c>
       <c r="M64" s="7" t="inlineStr">
@@ -6287,27 +6287,27 @@
       </c>
       <c r="N64" s="7" t="inlineStr">
         <is>
-          <t>26.2%</t>
+          <t>26.5%</t>
         </is>
       </c>
       <c r="O64" s="7" t="inlineStr">
         <is>
-          <t>51.6%</t>
+          <t>51.3%</t>
         </is>
       </c>
       <c r="P64" s="7" t="inlineStr">
         <is>
-          <t>20.8%</t>
+          <t>18.7%</t>
         </is>
       </c>
       <c r="Q64" s="7" t="inlineStr">
         <is>
-          <t>14.0%</t>
+          <t>12.7%</t>
         </is>
       </c>
       <c r="R64" s="7" t="inlineStr">
         <is>
-          <t>65.2%</t>
+          <t>68.5%</t>
         </is>
       </c>
     </row>
@@ -6357,47 +6357,47 @@
       </c>
       <c r="J65" s="7" t="inlineStr">
         <is>
-          <t>1.41</t>
+          <t>1.39</t>
         </is>
       </c>
       <c r="K65" s="7" t="inlineStr">
         <is>
-          <t>4.48</t>
+          <t>4.54</t>
         </is>
       </c>
       <c r="L65" s="7" t="inlineStr">
         <is>
-          <t>7.44</t>
+          <t>7.95</t>
         </is>
       </c>
       <c r="M65" s="7" t="inlineStr">
         <is>
-          <t>66.5%</t>
+          <t>67.5%</t>
         </is>
       </c>
       <c r="N65" s="7" t="inlineStr">
         <is>
-          <t>20.9%</t>
+          <t>20.7%</t>
         </is>
       </c>
       <c r="O65" s="7" t="inlineStr">
         <is>
-          <t>12.6%</t>
+          <t>11.8%</t>
         </is>
       </c>
       <c r="P65" s="7" t="inlineStr">
         <is>
-          <t>64.6%</t>
+          <t>63.7%</t>
         </is>
       </c>
       <c r="Q65" s="7" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>15.0%</t>
         </is>
       </c>
       <c r="R65" s="7" t="inlineStr">
         <is>
-          <t>21.0%</t>
+          <t>21.3%</t>
         </is>
       </c>
     </row>
@@ -6447,47 +6447,47 @@
       </c>
       <c r="J66" s="7" t="inlineStr">
         <is>
-          <t>2.45</t>
+          <t>2.44</t>
         </is>
       </c>
       <c r="K66" s="7" t="inlineStr">
         <is>
-          <t>3.54</t>
+          <t>3.74</t>
         </is>
       </c>
       <c r="L66" s="7" t="inlineStr">
         <is>
-          <t>2.63</t>
+          <t>2.60</t>
         </is>
       </c>
       <c r="M66" s="7" t="inlineStr">
         <is>
-          <t>38.1%</t>
+          <t>38.6%</t>
         </is>
       </c>
       <c r="N66" s="7" t="inlineStr">
         <is>
-          <t>26.4%</t>
+          <t>25.2%</t>
         </is>
       </c>
       <c r="O66" s="7" t="inlineStr">
         <is>
-          <t>35.5%</t>
+          <t>36.2%</t>
         </is>
       </c>
       <c r="P66" s="7" t="inlineStr">
         <is>
-          <t>26.8%</t>
+          <t>26.2%</t>
         </is>
       </c>
       <c r="Q66" s="7" t="inlineStr">
         <is>
-          <t>19.4%</t>
+          <t>19.9%</t>
         </is>
       </c>
       <c r="R66" s="7" t="inlineStr">
         <is>
-          <t>53.8%</t>
+          <t>54.0%</t>
         </is>
       </c>
     </row>
@@ -6537,7 +6537,7 @@
       </c>
       <c r="J67" s="7" t="inlineStr">
         <is>
-          <t>5.16</t>
+          <t>5.15</t>
         </is>
       </c>
       <c r="K67" s="7" t="inlineStr">
@@ -6547,7 +6547,7 @@
       </c>
       <c r="L67" s="7" t="inlineStr">
         <is>
-          <t>1.62</t>
+          <t>1.63</t>
         </is>
       </c>
       <c r="M67" s="7" t="inlineStr">
@@ -6557,27 +6557,27 @@
       </c>
       <c r="N67" s="7" t="inlineStr">
         <is>
-          <t>24.0%</t>
+          <t>24.1%</t>
         </is>
       </c>
       <c r="O67" s="7" t="inlineStr">
         <is>
-          <t>57.8%</t>
+          <t>57.7%</t>
         </is>
       </c>
       <c r="P67" s="7" t="inlineStr">
         <is>
-          <t>15.1%</t>
+          <t>15.0%</t>
         </is>
       </c>
       <c r="Q67" s="7" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>15.9%</t>
         </is>
       </c>
       <c r="R67" s="7" t="inlineStr">
         <is>
-          <t>67.8%</t>
+          <t>69.1%</t>
         </is>
       </c>
     </row>
@@ -6627,42 +6627,42 @@
       </c>
       <c r="J68" s="7" t="inlineStr">
         <is>
-          <t>2.21</t>
+          <t>2.23</t>
         </is>
       </c>
       <c r="K68" s="7" t="inlineStr">
         <is>
-          <t>3.02</t>
+          <t>2.99</t>
         </is>
       </c>
       <c r="L68" s="7" t="inlineStr">
         <is>
-          <t>3.49</t>
+          <t>3.56</t>
         </is>
       </c>
       <c r="M68" s="7" t="inlineStr">
         <is>
-          <t>42.3%</t>
+          <t>42.2%</t>
         </is>
       </c>
       <c r="N68" s="7" t="inlineStr">
         <is>
-          <t>30.9%</t>
+          <t>31.4%</t>
         </is>
       </c>
       <c r="O68" s="7" t="inlineStr">
         <is>
-          <t>26.8%</t>
+          <t>26.4%</t>
         </is>
       </c>
       <c r="P68" s="7" t="inlineStr">
         <is>
-          <t>30.8%</t>
+          <t>30.4%</t>
         </is>
       </c>
       <c r="Q68" s="7" t="inlineStr">
         <is>
-          <t>16.9%</t>
+          <t>17.3%</t>
         </is>
       </c>
       <c r="R68" s="7" t="inlineStr">
@@ -6717,47 +6717,47 @@
       </c>
       <c r="J69" s="7" t="inlineStr">
         <is>
-          <t>9.25</t>
+          <t>9.71</t>
         </is>
       </c>
       <c r="K69" s="7" t="inlineStr">
         <is>
-          <t>5.46</t>
+          <t>5.49</t>
         </is>
       </c>
       <c r="L69" s="7" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t>1.28</t>
         </is>
       </c>
       <c r="M69" s="7" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>9.7%</t>
         </is>
       </c>
       <c r="N69" s="7" t="inlineStr">
         <is>
-          <t>17.2%</t>
+          <t>17.1%</t>
         </is>
       </c>
       <c r="O69" s="7" t="inlineStr">
         <is>
-          <t>72.7%</t>
+          <t>73.3%</t>
         </is>
       </c>
       <c r="P69" s="7" t="inlineStr">
         <is>
-          <t>11.3%</t>
+          <t>12.4%</t>
         </is>
       </c>
       <c r="Q69" s="7" t="inlineStr">
         <is>
-          <t>10.6%</t>
+          <t>12.2%</t>
         </is>
       </c>
       <c r="R69" s="7" t="inlineStr">
         <is>
-          <t>78.1%</t>
+          <t>75.4%</t>
         </is>
       </c>
     </row>
@@ -6807,12 +6807,12 @@
       </c>
       <c r="J70" s="7" t="inlineStr">
         <is>
-          <t>9.13</t>
+          <t>9.10</t>
         </is>
       </c>
       <c r="K70" s="7" t="inlineStr">
         <is>
-          <t>5.88</t>
+          <t>6.05</t>
         </is>
       </c>
       <c r="L70" s="7" t="inlineStr">
@@ -6827,27 +6827,27 @@
       </c>
       <c r="N70" s="7" t="inlineStr">
         <is>
-          <t>15.9%</t>
+          <t>15.6%</t>
         </is>
       </c>
       <c r="O70" s="7" t="inlineStr">
         <is>
-          <t>73.8%</t>
+          <t>74.1%</t>
         </is>
       </c>
       <c r="P70" s="7" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>11.4%</t>
         </is>
       </c>
       <c r="Q70" s="7" t="inlineStr">
         <is>
-          <t>17.2%</t>
+          <t>16.6%</t>
         </is>
       </c>
       <c r="R70" s="7" t="inlineStr">
         <is>
-          <t>71.6%</t>
+          <t>72.0%</t>
         </is>
       </c>
     </row>
@@ -6897,42 +6897,42 @@
       </c>
       <c r="J71" s="7" t="inlineStr">
         <is>
-          <t>1.63</t>
+          <t>1.62</t>
         </is>
       </c>
       <c r="K71" s="7" t="inlineStr">
         <is>
-          <t>3.74</t>
+          <t>3.76</t>
         </is>
       </c>
       <c r="L71" s="7" t="inlineStr">
         <is>
-          <t>5.35</t>
+          <t>5.44</t>
         </is>
       </c>
       <c r="M71" s="7" t="inlineStr">
         <is>
-          <t>57.5%</t>
+          <t>57.8%</t>
         </is>
       </c>
       <c r="N71" s="7" t="inlineStr">
         <is>
-          <t>25.0%</t>
+          <t>24.9%</t>
         </is>
       </c>
       <c r="O71" s="7" t="inlineStr">
         <is>
-          <t>17.5%</t>
+          <t>17.2%</t>
         </is>
       </c>
       <c r="P71" s="7" t="inlineStr">
         <is>
-          <t>80.6%</t>
+          <t>80.2%</t>
         </is>
       </c>
       <c r="Q71" s="7" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>10.7%</t>
         </is>
       </c>
       <c r="R71" s="7" t="inlineStr">
@@ -6987,47 +6987,47 @@
       </c>
       <c r="J72" s="7" t="inlineStr">
         <is>
-          <t>3.44</t>
+          <t>3.50</t>
         </is>
       </c>
       <c r="K72" s="7" t="inlineStr">
         <is>
-          <t>3.30</t>
+          <t>3.28</t>
         </is>
       </c>
       <c r="L72" s="7" t="inlineStr">
         <is>
-          <t>2.08</t>
+          <t>2.12</t>
         </is>
       </c>
       <c r="M72" s="7" t="inlineStr">
         <is>
-          <t>27.1%</t>
+          <t>26.9%</t>
         </is>
       </c>
       <c r="N72" s="7" t="inlineStr">
         <is>
-          <t>28.2%</t>
+          <t>28.7%</t>
         </is>
       </c>
       <c r="O72" s="7" t="inlineStr">
         <is>
-          <t>44.7%</t>
+          <t>44.4%</t>
         </is>
       </c>
       <c r="P72" s="7" t="inlineStr">
         <is>
-          <t>37.7%</t>
+          <t>40.2%</t>
         </is>
       </c>
       <c r="Q72" s="7" t="inlineStr">
         <is>
-          <t>17.9%</t>
+          <t>17.6%</t>
         </is>
       </c>
       <c r="R72" s="7" t="inlineStr">
         <is>
-          <t>44.4%</t>
+          <t>42.1%</t>
         </is>
       </c>
     </row>
@@ -7077,47 +7077,47 @@
       </c>
       <c r="J73" s="7" t="inlineStr">
         <is>
-          <t>2.31</t>
+          <t>2.30</t>
         </is>
       </c>
       <c r="K73" s="7" t="inlineStr">
         <is>
-          <t>3.24</t>
+          <t>3.30</t>
         </is>
       </c>
       <c r="L73" s="7" t="inlineStr">
         <is>
-          <t>3.04</t>
+          <t>3.05</t>
         </is>
       </c>
       <c r="M73" s="7" t="inlineStr">
         <is>
-          <t>40.4%</t>
+          <t>40.8%</t>
         </is>
       </c>
       <c r="N73" s="7" t="inlineStr">
         <is>
-          <t>28.8%</t>
+          <t>28.4%</t>
         </is>
       </c>
       <c r="O73" s="7" t="inlineStr">
         <is>
-          <t>30.7%</t>
+          <t>30.8%</t>
         </is>
       </c>
       <c r="P73" s="7" t="inlineStr">
         <is>
-          <t>32.6%</t>
+          <t>34.2%</t>
         </is>
       </c>
       <c r="Q73" s="7" t="inlineStr">
         <is>
-          <t>16.4%</t>
+          <t>17.5%</t>
         </is>
       </c>
       <c r="R73" s="7" t="inlineStr">
         <is>
-          <t>51.0%</t>
+          <t>48.3%</t>
         </is>
       </c>
     </row>
@@ -7167,12 +7167,12 @@
       </c>
       <c r="J74" s="7" t="inlineStr">
         <is>
-          <t>3.49</t>
+          <t>3.62</t>
         </is>
       </c>
       <c r="K74" s="7" t="inlineStr">
         <is>
-          <t>3.15</t>
+          <t>3.08</t>
         </is>
       </c>
       <c r="L74" s="7" t="inlineStr">
@@ -7182,32 +7182,32 @@
       </c>
       <c r="M74" s="7" t="inlineStr">
         <is>
-          <t>26.8%</t>
+          <t>25.9%</t>
         </is>
       </c>
       <c r="N74" s="7" t="inlineStr">
         <is>
-          <t>29.7%</t>
+          <t>30.5%</t>
         </is>
       </c>
       <c r="O74" s="7" t="inlineStr">
         <is>
-          <t>43.5%</t>
+          <t>43.6%</t>
         </is>
       </c>
       <c r="P74" s="7" t="inlineStr">
         <is>
-          <t>36.6%</t>
+          <t>37.0%</t>
         </is>
       </c>
       <c r="Q74" s="7" t="inlineStr">
         <is>
-          <t>20.1%</t>
+          <t>20.0%</t>
         </is>
       </c>
       <c r="R74" s="7" t="inlineStr">
         <is>
-          <t>43.4%</t>
+          <t>43.0%</t>
         </is>
       </c>
     </row>
@@ -7257,12 +7257,12 @@
       </c>
       <c r="J75" s="7" t="inlineStr">
         <is>
-          <t>13.25</t>
+          <t>13.77</t>
         </is>
       </c>
       <c r="K75" s="7" t="inlineStr">
         <is>
-          <t>6.88</t>
+          <t>7.04</t>
         </is>
       </c>
       <c r="L75" s="7" t="inlineStr">
@@ -7272,32 +7272,32 @@
       </c>
       <c r="M75" s="7" t="inlineStr">
         <is>
-          <t>7.1%</t>
+          <t>6.8%</t>
         </is>
       </c>
       <c r="N75" s="7" t="inlineStr">
         <is>
-          <t>13.6%</t>
+          <t>13.4%</t>
         </is>
       </c>
       <c r="O75" s="7" t="inlineStr">
         <is>
-          <t>79.3%</t>
+          <t>79.8%</t>
         </is>
       </c>
       <c r="P75" s="7" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>10.7%</t>
         </is>
       </c>
       <c r="Q75" s="7" t="inlineStr">
         <is>
-          <t>12.6%</t>
+          <t>10.9%</t>
         </is>
       </c>
       <c r="R75" s="7" t="inlineStr">
         <is>
-          <t>76.4%</t>
+          <t>78.3%</t>
         </is>
       </c>
     </row>
@@ -7323,7 +7323,7 @@
       </c>
       <c r="F76" s="13" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="G76" s="12" t="inlineStr">
@@ -7373,7 +7373,7 @@
       </c>
       <c r="P76" s="11" t="inlineStr">
         <is>
-          <t>39.7%</t>
+          <t>49.8%</t>
         </is>
       </c>
       <c r="Q76" s="11" t="inlineStr">
@@ -7383,7 +7383,7 @@
       </c>
       <c r="R76" s="11" t="inlineStr">
         <is>
-          <t>60.3%</t>
+          <t>50.2%</t>
         </is>
       </c>
     </row>
@@ -7459,7 +7459,7 @@
       </c>
       <c r="P77" s="11" t="inlineStr">
         <is>
-          <t>62.1%</t>
+          <t>62.0%</t>
         </is>
       </c>
       <c r="Q77" s="11" t="inlineStr">
@@ -7469,7 +7469,7 @@
       </c>
       <c r="R77" s="11" t="inlineStr">
         <is>
-          <t>37.9%</t>
+          <t>38.0%</t>
         </is>
       </c>
     </row>
@@ -7803,7 +7803,7 @@
       </c>
       <c r="P81" s="11" t="inlineStr">
         <is>
-          <t>84.8%</t>
+          <t>85.0%</t>
         </is>
       </c>
       <c r="Q81" s="11" t="inlineStr">
@@ -7813,7 +7813,7 @@
       </c>
       <c r="R81" s="11" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>15.0%</t>
         </is>
       </c>
     </row>
@@ -7889,7 +7889,7 @@
       </c>
       <c r="P82" s="11" t="inlineStr">
         <is>
-          <t>81.0%</t>
+          <t>80.9%</t>
         </is>
       </c>
       <c r="Q82" s="11" t="inlineStr">
@@ -7899,7 +7899,7 @@
       </c>
       <c r="R82" s="11" t="inlineStr">
         <is>
-          <t>19.0%</t>
+          <t>19.1%</t>
         </is>
       </c>
     </row>
@@ -7975,7 +7975,7 @@
       </c>
       <c r="P83" s="11" t="inlineStr">
         <is>
-          <t>74.1%</t>
+          <t>74.0%</t>
         </is>
       </c>
       <c r="Q83" s="11" t="inlineStr">
@@ -7985,7 +7985,7 @@
       </c>
       <c r="R83" s="11" t="inlineStr">
         <is>
-          <t>25.9%</t>
+          <t>26.0%</t>
         </is>
       </c>
     </row>
@@ -8097,7 +8097,7 @@
       </c>
       <c r="F85" s="12" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Bosnia and Herzegovina</t>
         </is>
       </c>
       <c r="G85" s="12" t="inlineStr">
@@ -8147,7 +8147,7 @@
       </c>
       <c r="P85" s="11" t="inlineStr">
         <is>
-          <t>67.4%</t>
+          <t>77.0%</t>
         </is>
       </c>
       <c r="Q85" s="11" t="inlineStr">
@@ -8157,7 +8157,7 @@
       </c>
       <c r="R85" s="11" t="inlineStr">
         <is>
-          <t>32.6%</t>
+          <t>23.0%</t>
         </is>
       </c>
     </row>
@@ -8350,12 +8350,12 @@
       <c r="D88" s="11" t="inlineStr"/>
       <c r="E88" s="13" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="F88" s="12" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="G88" s="12" t="inlineStr">
@@ -8405,7 +8405,7 @@
       </c>
       <c r="P88" s="11" t="inlineStr">
         <is>
-          <t>67.0%</t>
+          <t>74.5%</t>
         </is>
       </c>
       <c r="Q88" s="11" t="inlineStr">
@@ -8415,7 +8415,7 @@
       </c>
       <c r="R88" s="11" t="inlineStr">
         <is>
-          <t>33.0%</t>
+          <t>25.5%</t>
         </is>
       </c>
     </row>
@@ -8613,7 +8613,7 @@
       </c>
       <c r="F91" s="12" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="G91" s="12" t="inlineStr">
@@ -8663,7 +8663,7 @@
       </c>
       <c r="P91" s="11" t="inlineStr">
         <is>
-          <t>81.0%</t>
+          <t>78.2%</t>
         </is>
       </c>
       <c r="Q91" s="11" t="inlineStr">
@@ -8673,7 +8673,7 @@
       </c>
       <c r="R91" s="11" t="inlineStr">
         <is>
-          <t>19.0%</t>
+          <t>21.8%</t>
         </is>
       </c>
     </row>
@@ -8694,7 +8694,7 @@
       <c r="D92" s="15" t="inlineStr"/>
       <c r="E92" s="16" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F92" s="17" t="inlineStr">
@@ -8709,12 +8709,12 @@
       </c>
       <c r="H92" s="18" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="I92" s="18" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J92" s="15" t="inlineStr">
@@ -8749,7 +8749,7 @@
       </c>
       <c r="P92" s="15" t="inlineStr">
         <is>
-          <t>41.2%</t>
+          <t>28.8%</t>
         </is>
       </c>
       <c r="Q92" s="15" t="inlineStr">
@@ -8759,7 +8759,7 @@
       </c>
       <c r="R92" s="15" t="inlineStr">
         <is>
-          <t>58.8%</t>
+          <t>71.2%</t>
         </is>
       </c>
     </row>
@@ -9007,7 +9007,7 @@
       </c>
       <c r="P95" s="15" t="inlineStr">
         <is>
-          <t>37.7%</t>
+          <t>37.6%</t>
         </is>
       </c>
       <c r="Q95" s="15" t="inlineStr">
@@ -9017,7 +9017,7 @@
       </c>
       <c r="R95" s="15" t="inlineStr">
         <is>
-          <t>62.3%</t>
+          <t>62.4%</t>
         </is>
       </c>
     </row>
@@ -9296,7 +9296,7 @@
       <c r="D99" s="15" t="inlineStr"/>
       <c r="E99" s="16" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="F99" s="17" t="inlineStr">
@@ -9351,7 +9351,7 @@
       </c>
       <c r="P99" s="15" t="inlineStr">
         <is>
-          <t>22.3%</t>
+          <t>22.5%</t>
         </is>
       </c>
       <c r="Q99" s="15" t="inlineStr">
@@ -9361,7 +9361,7 @@
       </c>
       <c r="R99" s="15" t="inlineStr">
         <is>
-          <t>77.7%</t>
+          <t>77.5%</t>
         </is>
       </c>
     </row>
@@ -9609,7 +9609,7 @@
       </c>
       <c r="P102" s="19" t="inlineStr">
         <is>
-          <t>55.6%</t>
+          <t>55.7%</t>
         </is>
       </c>
       <c r="Q102" s="19" t="inlineStr">
@@ -9619,7 +9619,7 @@
       </c>
       <c r="R102" s="19" t="inlineStr">
         <is>
-          <t>44.4%</t>
+          <t>44.3%</t>
         </is>
       </c>
     </row>
@@ -9867,7 +9867,7 @@
       </c>
       <c r="P105" s="23" t="inlineStr">
         <is>
-          <t>45.1%</t>
+          <t>45.2%</t>
         </is>
       </c>
       <c r="Q105" s="23" t="inlineStr">
@@ -9877,7 +9877,7 @@
       </c>
       <c r="R105" s="23" t="inlineStr">
         <is>
-          <t>54.9%</t>
+          <t>54.8%</t>
         </is>
       </c>
     </row>
@@ -9953,7 +9953,7 @@
       </c>
       <c r="P106" s="27" t="inlineStr">
         <is>
-          <t>37.6%</t>
+          <t>37.5%</t>
         </is>
       </c>
       <c r="Q106" s="27" t="inlineStr">
@@ -9963,7 +9963,7 @@
       </c>
       <c r="R106" s="27" t="inlineStr">
         <is>
-          <t>62.4%</t>
+          <t>62.5%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add xG display and manual score updates
</commit_message>
<xml_diff>
--- a/github_vercel_app/public/files/Scorito_scores_met_kansen_latest.xlsx
+++ b/github_vercel_app/public/files/Scorito_scores_met_kansen_latest.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="WK 2026 voorspellingen" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WK 2026 voorspellingen" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -178,9 +178,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ScoritoScoresMetKansen" displayName="ScoritoScoresMetKansen" ref="A2:P106" headerRowCount="1">
-  <autoFilter ref="A2:P106"/>
-  <tableColumns count="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ScoritoScoresMetKansen" displayName="ScoritoScoresMetKansen" ref="A2:R106" headerRowCount="1">
+  <autoFilter ref="A2:R106"/>
+  <tableColumns count="18">
     <tableColumn id="1" name="Nr"/>
     <tableColumn id="2" name="Datum"/>
     <tableColumn id="3" name="Ronde"/>
@@ -193,10 +193,12 @@
     <tableColumn id="10" name="Kans thuis"/>
     <tableColumn id="11" name="Kans gelijk"/>
     <tableColumn id="12" name="Kans uit"/>
-    <tableColumn id="13" name="Voorspelde winnaar"/>
-    <tableColumn id="14" name="Door bij gelijk"/>
-    <tableColumn id="15" name="Status"/>
-    <tableColumn id="16" name="Uitslag"/>
+    <tableColumn id="13" name="xG thuis"/>
+    <tableColumn id="14" name="xG uit"/>
+    <tableColumn id="15" name="Voorspelde winnaar"/>
+    <tableColumn id="16" name="Door bij gelijk"/>
+    <tableColumn id="17" name="Status"/>
+    <tableColumn id="18" name="Uitslag"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -491,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P106"/>
+  <dimension ref="A1:R106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -506,10 +508,12 @@
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="22" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="13" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -582,20 +586,30 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
+          <t>xG thuis</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>xG uit</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
           <t>Voorspelde winnaar</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>Door bij gelijk</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="Q2" s="2" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="R2" s="2" t="inlineStr">
         <is>
           <t>Uitslag</t>
         </is>
@@ -638,18 +652,20 @@
       <c r="J3" s="6" t="inlineStr"/>
       <c r="K3" s="6" t="inlineStr"/>
       <c r="L3" s="6" t="inlineStr"/>
-      <c r="M3" s="3" t="inlineStr">
-        <is>
-          <t>Mexico</t>
-        </is>
-      </c>
+      <c r="M3" s="3" t="inlineStr"/>
       <c r="N3" s="3" t="inlineStr"/>
       <c r="O3" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P3" s="3" t="inlineStr">
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="inlineStr"/>
+      <c r="Q3" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R3" s="3" t="inlineStr">
         <is>
           <t>2-0</t>
         </is>
@@ -692,18 +708,20 @@
       <c r="J4" s="6" t="inlineStr"/>
       <c r="K4" s="6" t="inlineStr"/>
       <c r="L4" s="6" t="inlineStr"/>
-      <c r="M4" s="3" t="inlineStr">
-        <is>
-          <t>Draw</t>
-        </is>
-      </c>
+      <c r="M4" s="3" t="inlineStr"/>
       <c r="N4" s="3" t="inlineStr"/>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P4" s="3" t="inlineStr">
+          <t>Draw</t>
+        </is>
+      </c>
+      <c r="P4" s="3" t="inlineStr"/>
+      <c r="Q4" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R4" s="3" t="inlineStr">
         <is>
           <t>2-1</t>
         </is>
@@ -746,18 +764,20 @@
       <c r="J5" s="6" t="inlineStr"/>
       <c r="K5" s="6" t="inlineStr"/>
       <c r="L5" s="6" t="inlineStr"/>
-      <c r="M5" s="3" t="inlineStr">
-        <is>
-          <t>Canada</t>
-        </is>
-      </c>
+      <c r="M5" s="3" t="inlineStr"/>
       <c r="N5" s="3" t="inlineStr"/>
       <c r="O5" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P5" s="3" t="inlineStr">
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="P5" s="3" t="inlineStr"/>
+      <c r="Q5" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R5" s="3" t="inlineStr">
         <is>
           <t>1-1</t>
         </is>
@@ -800,18 +820,20 @@
       <c r="J6" s="6" t="inlineStr"/>
       <c r="K6" s="6" t="inlineStr"/>
       <c r="L6" s="6" t="inlineStr"/>
-      <c r="M6" s="3" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
+      <c r="M6" s="3" t="inlineStr"/>
       <c r="N6" s="3" t="inlineStr"/>
       <c r="O6" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P6" s="3" t="inlineStr">
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="P6" s="3" t="inlineStr"/>
+      <c r="Q6" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R6" s="3" t="inlineStr">
         <is>
           <t>4-1</t>
         </is>
@@ -854,18 +876,20 @@
       <c r="J7" s="6" t="inlineStr"/>
       <c r="K7" s="6" t="inlineStr"/>
       <c r="L7" s="6" t="inlineStr"/>
-      <c r="M7" s="3" t="inlineStr">
-        <is>
-          <t>Switzerland</t>
-        </is>
-      </c>
+      <c r="M7" s="3" t="inlineStr"/>
       <c r="N7" s="3" t="inlineStr"/>
       <c r="O7" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P7" s="3" t="inlineStr">
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="P7" s="3" t="inlineStr"/>
+      <c r="Q7" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R7" s="3" t="inlineStr">
         <is>
           <t>1-1</t>
         </is>
@@ -908,18 +932,20 @@
       <c r="J8" s="6" t="inlineStr"/>
       <c r="K8" s="6" t="inlineStr"/>
       <c r="L8" s="6" t="inlineStr"/>
-      <c r="M8" s="3" t="inlineStr">
-        <is>
-          <t>Brazil</t>
-        </is>
-      </c>
+      <c r="M8" s="3" t="inlineStr"/>
       <c r="N8" s="3" t="inlineStr"/>
       <c r="O8" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P8" s="3" t="inlineStr">
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="P8" s="3" t="inlineStr"/>
+      <c r="Q8" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R8" s="3" t="inlineStr">
         <is>
           <t>1-1</t>
         </is>
@@ -962,18 +988,20 @@
       <c r="J9" s="6" t="inlineStr"/>
       <c r="K9" s="6" t="inlineStr"/>
       <c r="L9" s="6" t="inlineStr"/>
-      <c r="M9" s="3" t="inlineStr">
-        <is>
-          <t>Scotland</t>
-        </is>
-      </c>
+      <c r="M9" s="3" t="inlineStr"/>
       <c r="N9" s="3" t="inlineStr"/>
       <c r="O9" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P9" s="3" t="inlineStr">
+          <t>Scotland</t>
+        </is>
+      </c>
+      <c r="P9" s="3" t="inlineStr"/>
+      <c r="Q9" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R9" s="3" t="inlineStr">
         <is>
           <t>0-1</t>
         </is>
@@ -1016,18 +1044,20 @@
       <c r="J10" s="6" t="inlineStr"/>
       <c r="K10" s="6" t="inlineStr"/>
       <c r="L10" s="6" t="inlineStr"/>
-      <c r="M10" s="3" t="inlineStr">
-        <is>
-          <t>Turkey</t>
-        </is>
-      </c>
+      <c r="M10" s="3" t="inlineStr"/>
       <c r="N10" s="3" t="inlineStr"/>
       <c r="O10" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P10" s="3" t="inlineStr">
+          <t>Turkey</t>
+        </is>
+      </c>
+      <c r="P10" s="3" t="inlineStr"/>
+      <c r="Q10" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R10" s="3" t="inlineStr">
         <is>
           <t>2-0</t>
         </is>
@@ -1070,18 +1100,20 @@
       <c r="J11" s="6" t="inlineStr"/>
       <c r="K11" s="6" t="inlineStr"/>
       <c r="L11" s="6" t="inlineStr"/>
-      <c r="M11" s="3" t="inlineStr">
-        <is>
-          <t>Germany</t>
-        </is>
-      </c>
+      <c r="M11" s="3" t="inlineStr"/>
       <c r="N11" s="3" t="inlineStr"/>
       <c r="O11" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P11" s="3" t="inlineStr">
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="P11" s="3" t="inlineStr"/>
+      <c r="Q11" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R11" s="3" t="inlineStr">
         <is>
           <t>7-1</t>
         </is>
@@ -1124,18 +1156,20 @@
       <c r="J12" s="6" t="inlineStr"/>
       <c r="K12" s="6" t="inlineStr"/>
       <c r="L12" s="6" t="inlineStr"/>
-      <c r="M12" s="3" t="inlineStr">
-        <is>
-          <t>Netherlands</t>
-        </is>
-      </c>
+      <c r="M12" s="3" t="inlineStr"/>
       <c r="N12" s="3" t="inlineStr"/>
       <c r="O12" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P12" s="3" t="inlineStr">
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="P12" s="3" t="inlineStr"/>
+      <c r="Q12" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R12" s="3" t="inlineStr">
         <is>
           <t>2-2</t>
         </is>
@@ -1178,18 +1212,20 @@
       <c r="J13" s="6" t="inlineStr"/>
       <c r="K13" s="6" t="inlineStr"/>
       <c r="L13" s="6" t="inlineStr"/>
-      <c r="M13" s="3" t="inlineStr">
-        <is>
-          <t>Ecuador</t>
-        </is>
-      </c>
+      <c r="M13" s="3" t="inlineStr"/>
       <c r="N13" s="3" t="inlineStr"/>
       <c r="O13" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P13" s="3" t="inlineStr">
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="P13" s="3" t="inlineStr"/>
+      <c r="Q13" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R13" s="3" t="inlineStr">
         <is>
           <t>1-0</t>
         </is>
@@ -1232,18 +1268,20 @@
       <c r="J14" s="6" t="inlineStr"/>
       <c r="K14" s="6" t="inlineStr"/>
       <c r="L14" s="6" t="inlineStr"/>
-      <c r="M14" s="3" t="inlineStr">
-        <is>
-          <t>Sweden</t>
-        </is>
-      </c>
+      <c r="M14" s="3" t="inlineStr"/>
       <c r="N14" s="3" t="inlineStr"/>
       <c r="O14" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P14" s="3" t="inlineStr">
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="P14" s="3" t="inlineStr"/>
+      <c r="Q14" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R14" s="3" t="inlineStr">
         <is>
           <t>5-1</t>
         </is>
@@ -1286,18 +1324,20 @@
       <c r="J15" s="6" t="inlineStr"/>
       <c r="K15" s="6" t="inlineStr"/>
       <c r="L15" s="6" t="inlineStr"/>
-      <c r="M15" s="3" t="inlineStr">
-        <is>
-          <t>Spain</t>
-        </is>
-      </c>
+      <c r="M15" s="3" t="inlineStr"/>
       <c r="N15" s="3" t="inlineStr"/>
       <c r="O15" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P15" s="3" t="inlineStr">
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="P15" s="3" t="inlineStr"/>
+      <c r="Q15" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R15" s="3" t="inlineStr">
         <is>
           <t>0-0</t>
         </is>
@@ -1340,18 +1380,20 @@
       <c r="J16" s="6" t="inlineStr"/>
       <c r="K16" s="6" t="inlineStr"/>
       <c r="L16" s="6" t="inlineStr"/>
-      <c r="M16" s="3" t="inlineStr">
-        <is>
-          <t>Belgium</t>
-        </is>
-      </c>
+      <c r="M16" s="3" t="inlineStr"/>
       <c r="N16" s="3" t="inlineStr"/>
       <c r="O16" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P16" s="3" t="inlineStr">
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="P16" s="3" t="inlineStr"/>
+      <c r="Q16" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R16" s="3" t="inlineStr">
         <is>
           <t>1-1</t>
         </is>
@@ -1394,18 +1436,20 @@
       <c r="J17" s="6" t="inlineStr"/>
       <c r="K17" s="6" t="inlineStr"/>
       <c r="L17" s="6" t="inlineStr"/>
-      <c r="M17" s="3" t="inlineStr">
-        <is>
-          <t>Uruguay</t>
-        </is>
-      </c>
+      <c r="M17" s="3" t="inlineStr"/>
       <c r="N17" s="3" t="inlineStr"/>
       <c r="O17" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P17" s="3" t="inlineStr">
+          <t>Uruguay</t>
+        </is>
+      </c>
+      <c r="P17" s="3" t="inlineStr"/>
+      <c r="Q17" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R17" s="3" t="inlineStr">
         <is>
           <t>1-1</t>
         </is>
@@ -1448,18 +1492,20 @@
       <c r="J18" s="6" t="inlineStr"/>
       <c r="K18" s="6" t="inlineStr"/>
       <c r="L18" s="6" t="inlineStr"/>
-      <c r="M18" s="3" t="inlineStr">
-        <is>
-          <t>Iran</t>
-        </is>
-      </c>
+      <c r="M18" s="3" t="inlineStr"/>
       <c r="N18" s="3" t="inlineStr"/>
       <c r="O18" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P18" s="3" t="inlineStr">
+          <t>Iran</t>
+        </is>
+      </c>
+      <c r="P18" s="3" t="inlineStr"/>
+      <c r="Q18" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R18" s="3" t="inlineStr">
         <is>
           <t>2-2</t>
         </is>
@@ -1502,18 +1548,20 @@
       <c r="J19" s="6" t="inlineStr"/>
       <c r="K19" s="6" t="inlineStr"/>
       <c r="L19" s="6" t="inlineStr"/>
-      <c r="M19" s="3" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
+      <c r="M19" s="3" t="inlineStr"/>
       <c r="N19" s="3" t="inlineStr"/>
       <c r="O19" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P19" s="3" t="inlineStr">
+          <t>France</t>
+        </is>
+      </c>
+      <c r="P19" s="3" t="inlineStr"/>
+      <c r="Q19" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R19" s="3" t="inlineStr">
         <is>
           <t>3-1</t>
         </is>
@@ -1556,18 +1604,20 @@
       <c r="J20" s="6" t="inlineStr"/>
       <c r="K20" s="6" t="inlineStr"/>
       <c r="L20" s="6" t="inlineStr"/>
-      <c r="M20" s="3" t="inlineStr">
-        <is>
-          <t>Norway</t>
-        </is>
-      </c>
+      <c r="M20" s="3" t="inlineStr"/>
       <c r="N20" s="3" t="inlineStr"/>
       <c r="O20" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P20" s="3" t="inlineStr">
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="P20" s="3" t="inlineStr"/>
+      <c r="Q20" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R20" s="3" t="inlineStr">
         <is>
           <t>1-4</t>
         </is>
@@ -1610,18 +1660,20 @@
       <c r="J21" s="6" t="inlineStr"/>
       <c r="K21" s="6" t="inlineStr"/>
       <c r="L21" s="6" t="inlineStr"/>
-      <c r="M21" s="3" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
+      <c r="M21" s="3" t="inlineStr"/>
       <c r="N21" s="3" t="inlineStr"/>
       <c r="O21" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P21" s="3" t="inlineStr">
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="P21" s="3" t="inlineStr"/>
+      <c r="Q21" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R21" s="3" t="inlineStr">
         <is>
           <t>3-0</t>
         </is>
@@ -1664,18 +1716,20 @@
       <c r="J22" s="6" t="inlineStr"/>
       <c r="K22" s="6" t="inlineStr"/>
       <c r="L22" s="6" t="inlineStr"/>
-      <c r="M22" s="3" t="inlineStr">
-        <is>
-          <t>Austria</t>
-        </is>
-      </c>
+      <c r="M22" s="3" t="inlineStr"/>
       <c r="N22" s="3" t="inlineStr"/>
       <c r="O22" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P22" s="3" t="inlineStr">
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="P22" s="3" t="inlineStr"/>
+      <c r="Q22" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R22" s="3" t="inlineStr">
         <is>
           <t>3-1</t>
         </is>
@@ -1718,18 +1772,20 @@
       <c r="J23" s="6" t="inlineStr"/>
       <c r="K23" s="6" t="inlineStr"/>
       <c r="L23" s="6" t="inlineStr"/>
-      <c r="M23" s="3" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
+      <c r="M23" s="3" t="inlineStr"/>
       <c r="N23" s="3" t="inlineStr"/>
       <c r="O23" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P23" s="3" t="inlineStr">
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="P23" s="3" t="inlineStr"/>
+      <c r="Q23" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R23" s="3" t="inlineStr">
         <is>
           <t>1-1</t>
         </is>
@@ -1772,18 +1828,20 @@
       <c r="J24" s="6" t="inlineStr"/>
       <c r="K24" s="6" t="inlineStr"/>
       <c r="L24" s="6" t="inlineStr"/>
-      <c r="M24" s="3" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
+      <c r="M24" s="3" t="inlineStr"/>
       <c r="N24" s="3" t="inlineStr"/>
       <c r="O24" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P24" s="3" t="inlineStr">
+          <t>England</t>
+        </is>
+      </c>
+      <c r="P24" s="3" t="inlineStr"/>
+      <c r="Q24" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R24" s="3" t="inlineStr">
         <is>
           <t>4-2</t>
         </is>
@@ -1826,18 +1884,20 @@
       <c r="J25" s="6" t="inlineStr"/>
       <c r="K25" s="6" t="inlineStr"/>
       <c r="L25" s="6" t="inlineStr"/>
-      <c r="M25" s="3" t="inlineStr">
-        <is>
-          <t>Ghana</t>
-        </is>
-      </c>
+      <c r="M25" s="3" t="inlineStr"/>
       <c r="N25" s="3" t="inlineStr"/>
       <c r="O25" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P25" s="3" t="inlineStr">
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="P25" s="3" t="inlineStr"/>
+      <c r="Q25" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R25" s="3" t="inlineStr">
         <is>
           <t>1-0</t>
         </is>
@@ -1880,18 +1940,20 @@
       <c r="J26" s="6" t="inlineStr"/>
       <c r="K26" s="6" t="inlineStr"/>
       <c r="L26" s="6" t="inlineStr"/>
-      <c r="M26" s="3" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
+      <c r="M26" s="3" t="inlineStr"/>
       <c r="N26" s="3" t="inlineStr"/>
       <c r="O26" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P26" s="3" t="inlineStr">
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="P26" s="3" t="inlineStr"/>
+      <c r="Q26" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R26" s="3" t="inlineStr">
         <is>
           <t>1-3</t>
         </is>
@@ -1934,18 +1996,20 @@
       <c r="J27" s="6" t="inlineStr"/>
       <c r="K27" s="6" t="inlineStr"/>
       <c r="L27" s="6" t="inlineStr"/>
-      <c r="M27" s="3" t="inlineStr">
-        <is>
-          <t>Czech Republic</t>
-        </is>
-      </c>
+      <c r="M27" s="3" t="inlineStr"/>
       <c r="N27" s="3" t="inlineStr"/>
       <c r="O27" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P27" s="3" t="inlineStr">
+          <t>Czech Republic</t>
+        </is>
+      </c>
+      <c r="P27" s="3" t="inlineStr"/>
+      <c r="Q27" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R27" s="3" t="inlineStr">
         <is>
           <t>1-1</t>
         </is>
@@ -1988,18 +2052,20 @@
       <c r="J28" s="6" t="inlineStr"/>
       <c r="K28" s="6" t="inlineStr"/>
       <c r="L28" s="6" t="inlineStr"/>
-      <c r="M28" s="3" t="inlineStr">
-        <is>
-          <t>Switzerland</t>
-        </is>
-      </c>
+      <c r="M28" s="3" t="inlineStr"/>
       <c r="N28" s="3" t="inlineStr"/>
       <c r="O28" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P28" s="3" t="inlineStr">
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="P28" s="3" t="inlineStr"/>
+      <c r="Q28" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R28" s="3" t="inlineStr">
         <is>
           <t>4-1</t>
         </is>
@@ -2042,18 +2108,20 @@
       <c r="J29" s="6" t="inlineStr"/>
       <c r="K29" s="6" t="inlineStr"/>
       <c r="L29" s="6" t="inlineStr"/>
-      <c r="M29" s="3" t="inlineStr">
-        <is>
-          <t>Canada</t>
-        </is>
-      </c>
+      <c r="M29" s="3" t="inlineStr"/>
       <c r="N29" s="3" t="inlineStr"/>
       <c r="O29" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P29" s="3" t="inlineStr">
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="P29" s="3" t="inlineStr"/>
+      <c r="Q29" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R29" s="3" t="inlineStr">
         <is>
           <t>6-0</t>
         </is>
@@ -2096,18 +2164,20 @@
       <c r="J30" s="6" t="inlineStr"/>
       <c r="K30" s="6" t="inlineStr"/>
       <c r="L30" s="6" t="inlineStr"/>
-      <c r="M30" s="3" t="inlineStr">
-        <is>
-          <t>Mexico</t>
-        </is>
-      </c>
+      <c r="M30" s="3" t="inlineStr"/>
       <c r="N30" s="3" t="inlineStr"/>
       <c r="O30" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P30" s="3" t="inlineStr">
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="P30" s="3" t="inlineStr"/>
+      <c r="Q30" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R30" s="3" t="inlineStr">
         <is>
           <t>1-0</t>
         </is>
@@ -2150,18 +2220,20 @@
       <c r="J31" s="6" t="inlineStr"/>
       <c r="K31" s="6" t="inlineStr"/>
       <c r="L31" s="6" t="inlineStr"/>
-      <c r="M31" s="3" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
+      <c r="M31" s="3" t="inlineStr"/>
       <c r="N31" s="3" t="inlineStr"/>
       <c r="O31" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P31" s="3" t="inlineStr">
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="P31" s="3" t="inlineStr"/>
+      <c r="Q31" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R31" s="3" t="inlineStr">
         <is>
           <t>2-0</t>
         </is>
@@ -2204,18 +2276,20 @@
       <c r="J32" s="6" t="inlineStr"/>
       <c r="K32" s="6" t="inlineStr"/>
       <c r="L32" s="6" t="inlineStr"/>
-      <c r="M32" s="3" t="inlineStr">
-        <is>
-          <t>Morocco</t>
-        </is>
-      </c>
+      <c r="M32" s="3" t="inlineStr"/>
       <c r="N32" s="3" t="inlineStr"/>
       <c r="O32" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P32" s="3" t="inlineStr">
+          <t>Morocco</t>
+        </is>
+      </c>
+      <c r="P32" s="3" t="inlineStr"/>
+      <c r="Q32" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R32" s="3" t="inlineStr">
         <is>
           <t>0-1</t>
         </is>
@@ -2258,18 +2332,20 @@
       <c r="J33" s="6" t="inlineStr"/>
       <c r="K33" s="6" t="inlineStr"/>
       <c r="L33" s="6" t="inlineStr"/>
-      <c r="M33" s="3" t="inlineStr">
-        <is>
-          <t>Brazil</t>
-        </is>
-      </c>
+      <c r="M33" s="3" t="inlineStr"/>
       <c r="N33" s="3" t="inlineStr"/>
       <c r="O33" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P33" s="3" t="inlineStr">
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="P33" s="3" t="inlineStr"/>
+      <c r="Q33" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R33" s="3" t="inlineStr">
         <is>
           <t>3-0</t>
         </is>
@@ -2312,18 +2388,20 @@
       <c r="J34" s="6" t="inlineStr"/>
       <c r="K34" s="6" t="inlineStr"/>
       <c r="L34" s="6" t="inlineStr"/>
-      <c r="M34" s="3" t="inlineStr">
-        <is>
-          <t>Turkey</t>
-        </is>
-      </c>
+      <c r="M34" s="3" t="inlineStr"/>
       <c r="N34" s="3" t="inlineStr"/>
       <c r="O34" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P34" s="3" t="inlineStr">
+          <t>Turkey</t>
+        </is>
+      </c>
+      <c r="P34" s="3" t="inlineStr"/>
+      <c r="Q34" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R34" s="3" t="inlineStr">
         <is>
           <t>0-1</t>
         </is>
@@ -2366,18 +2444,20 @@
       <c r="J35" s="6" t="inlineStr"/>
       <c r="K35" s="6" t="inlineStr"/>
       <c r="L35" s="6" t="inlineStr"/>
-      <c r="M35" s="3" t="inlineStr">
-        <is>
-          <t>Netherlands</t>
-        </is>
-      </c>
+      <c r="M35" s="3" t="inlineStr"/>
       <c r="N35" s="3" t="inlineStr"/>
       <c r="O35" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P35" s="3" t="inlineStr">
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="P35" s="3" t="inlineStr"/>
+      <c r="Q35" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R35" s="3" t="inlineStr">
         <is>
           <t>5-1</t>
         </is>
@@ -2420,18 +2500,20 @@
       <c r="J36" s="6" t="inlineStr"/>
       <c r="K36" s="6" t="inlineStr"/>
       <c r="L36" s="6" t="inlineStr"/>
-      <c r="M36" s="3" t="inlineStr">
-        <is>
-          <t>Germany</t>
-        </is>
-      </c>
+      <c r="M36" s="3" t="inlineStr"/>
       <c r="N36" s="3" t="inlineStr"/>
       <c r="O36" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P36" s="3" t="inlineStr">
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="P36" s="3" t="inlineStr"/>
+      <c r="Q36" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R36" s="3" t="inlineStr">
         <is>
           <t>2-1</t>
         </is>
@@ -2474,18 +2556,20 @@
       <c r="J37" s="6" t="inlineStr"/>
       <c r="K37" s="6" t="inlineStr"/>
       <c r="L37" s="6" t="inlineStr"/>
-      <c r="M37" s="3" t="inlineStr">
-        <is>
-          <t>Ecuador</t>
-        </is>
-      </c>
+      <c r="M37" s="3" t="inlineStr"/>
       <c r="N37" s="3" t="inlineStr"/>
       <c r="O37" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P37" s="3" t="inlineStr">
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="P37" s="3" t="inlineStr"/>
+      <c r="Q37" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R37" s="3" t="inlineStr">
         <is>
           <t>0-0</t>
         </is>
@@ -2528,18 +2612,20 @@
       <c r="J38" s="6" t="inlineStr"/>
       <c r="K38" s="6" t="inlineStr"/>
       <c r="L38" s="6" t="inlineStr"/>
-      <c r="M38" s="3" t="inlineStr">
-        <is>
-          <t>Japan</t>
-        </is>
-      </c>
+      <c r="M38" s="3" t="inlineStr"/>
       <c r="N38" s="3" t="inlineStr"/>
       <c r="O38" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P38" s="3" t="inlineStr">
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="P38" s="3" t="inlineStr"/>
+      <c r="Q38" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R38" s="3" t="inlineStr">
         <is>
           <t>0-4</t>
         </is>
@@ -2582,18 +2668,20 @@
       <c r="J39" s="6" t="inlineStr"/>
       <c r="K39" s="6" t="inlineStr"/>
       <c r="L39" s="6" t="inlineStr"/>
-      <c r="M39" s="3" t="inlineStr">
-        <is>
-          <t>Spain</t>
-        </is>
-      </c>
+      <c r="M39" s="3" t="inlineStr"/>
       <c r="N39" s="3" t="inlineStr"/>
       <c r="O39" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P39" s="3" t="inlineStr">
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="P39" s="3" t="inlineStr"/>
+      <c r="Q39" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R39" s="3" t="inlineStr">
         <is>
           <t>4-0</t>
         </is>
@@ -2636,18 +2724,20 @@
       <c r="J40" s="6" t="inlineStr"/>
       <c r="K40" s="6" t="inlineStr"/>
       <c r="L40" s="6" t="inlineStr"/>
-      <c r="M40" s="3" t="inlineStr">
-        <is>
-          <t>Belgium</t>
-        </is>
-      </c>
+      <c r="M40" s="3" t="inlineStr"/>
       <c r="N40" s="3" t="inlineStr"/>
       <c r="O40" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P40" s="3" t="inlineStr">
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="P40" s="3" t="inlineStr"/>
+      <c r="Q40" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R40" s="3" t="inlineStr">
         <is>
           <t>0-0</t>
         </is>
@@ -2690,18 +2780,20 @@
       <c r="J41" s="6" t="inlineStr"/>
       <c r="K41" s="6" t="inlineStr"/>
       <c r="L41" s="6" t="inlineStr"/>
-      <c r="M41" s="3" t="inlineStr">
-        <is>
-          <t>Uruguay</t>
-        </is>
-      </c>
+      <c r="M41" s="3" t="inlineStr"/>
       <c r="N41" s="3" t="inlineStr"/>
       <c r="O41" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P41" s="3" t="inlineStr">
+          <t>Uruguay</t>
+        </is>
+      </c>
+      <c r="P41" s="3" t="inlineStr"/>
+      <c r="Q41" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R41" s="3" t="inlineStr">
         <is>
           <t>2-2</t>
         </is>
@@ -2744,18 +2836,20 @@
       <c r="J42" s="6" t="inlineStr"/>
       <c r="K42" s="6" t="inlineStr"/>
       <c r="L42" s="6" t="inlineStr"/>
-      <c r="M42" s="3" t="inlineStr">
-        <is>
-          <t>Egypt</t>
-        </is>
-      </c>
+      <c r="M42" s="3" t="inlineStr"/>
       <c r="N42" s="3" t="inlineStr"/>
       <c r="O42" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P42" s="3" t="inlineStr">
+          <t>Egypt</t>
+        </is>
+      </c>
+      <c r="P42" s="3" t="inlineStr"/>
+      <c r="Q42" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R42" s="3" t="inlineStr">
         <is>
           <t>1-3</t>
         </is>
@@ -2798,18 +2892,20 @@
       <c r="J43" s="6" t="inlineStr"/>
       <c r="K43" s="6" t="inlineStr"/>
       <c r="L43" s="6" t="inlineStr"/>
-      <c r="M43" s="3" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
+      <c r="M43" s="3" t="inlineStr"/>
       <c r="N43" s="3" t="inlineStr"/>
       <c r="O43" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P43" s="3" t="inlineStr">
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="P43" s="3" t="inlineStr"/>
+      <c r="Q43" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R43" s="3" t="inlineStr">
         <is>
           <t>2-0</t>
         </is>
@@ -2852,18 +2948,20 @@
       <c r="J44" s="6" t="inlineStr"/>
       <c r="K44" s="6" t="inlineStr"/>
       <c r="L44" s="6" t="inlineStr"/>
-      <c r="M44" s="3" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
+      <c r="M44" s="3" t="inlineStr"/>
       <c r="N44" s="3" t="inlineStr"/>
       <c r="O44" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P44" s="3" t="inlineStr">
+          <t>France</t>
+        </is>
+      </c>
+      <c r="P44" s="3" t="inlineStr"/>
+      <c r="Q44" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R44" s="3" t="inlineStr">
         <is>
           <t>3-0</t>
         </is>
@@ -2906,18 +3004,20 @@
       <c r="J45" s="6" t="inlineStr"/>
       <c r="K45" s="6" t="inlineStr"/>
       <c r="L45" s="6" t="inlineStr"/>
-      <c r="M45" s="3" t="inlineStr">
-        <is>
-          <t>Norway</t>
-        </is>
-      </c>
+      <c r="M45" s="3" t="inlineStr"/>
       <c r="N45" s="3" t="inlineStr"/>
       <c r="O45" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P45" s="3" t="inlineStr">
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="P45" s="3" t="inlineStr"/>
+      <c r="Q45" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R45" s="3" t="inlineStr">
         <is>
           <t>3-2</t>
         </is>
@@ -2960,18 +3060,20 @@
       <c r="J46" s="6" t="inlineStr"/>
       <c r="K46" s="6" t="inlineStr"/>
       <c r="L46" s="6" t="inlineStr"/>
-      <c r="M46" s="3" t="inlineStr">
-        <is>
-          <t>Algeria</t>
-        </is>
-      </c>
+      <c r="M46" s="3" t="inlineStr"/>
       <c r="N46" s="3" t="inlineStr"/>
       <c r="O46" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P46" s="3" t="inlineStr">
+          <t>Algeria</t>
+        </is>
+      </c>
+      <c r="P46" s="3" t="inlineStr"/>
+      <c r="Q46" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R46" s="3" t="inlineStr">
         <is>
           <t>1-2</t>
         </is>
@@ -3014,18 +3116,20 @@
       <c r="J47" s="6" t="inlineStr"/>
       <c r="K47" s="6" t="inlineStr"/>
       <c r="L47" s="6" t="inlineStr"/>
-      <c r="M47" s="3" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
+      <c r="M47" s="3" t="inlineStr"/>
       <c r="N47" s="3" t="inlineStr"/>
       <c r="O47" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P47" s="3" t="inlineStr">
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="P47" s="3" t="inlineStr"/>
+      <c r="Q47" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R47" s="3" t="inlineStr">
         <is>
           <t>5-0</t>
         </is>
@@ -3068,18 +3172,20 @@
       <c r="J48" s="6" t="inlineStr"/>
       <c r="K48" s="6" t="inlineStr"/>
       <c r="L48" s="6" t="inlineStr"/>
-      <c r="M48" s="3" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
+      <c r="M48" s="3" t="inlineStr"/>
       <c r="N48" s="3" t="inlineStr"/>
       <c r="O48" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P48" s="3" t="inlineStr">
+          <t>England</t>
+        </is>
+      </c>
+      <c r="P48" s="3" t="inlineStr"/>
+      <c r="Q48" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R48" s="3" t="inlineStr">
         <is>
           <t>0-0</t>
         </is>
@@ -3122,18 +3228,20 @@
       <c r="J49" s="6" t="inlineStr"/>
       <c r="K49" s="6" t="inlineStr"/>
       <c r="L49" s="6" t="inlineStr"/>
-      <c r="M49" s="3" t="inlineStr">
-        <is>
-          <t>Croatia</t>
-        </is>
-      </c>
+      <c r="M49" s="3" t="inlineStr"/>
       <c r="N49" s="3" t="inlineStr"/>
       <c r="O49" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P49" s="3" t="inlineStr">
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="P49" s="3" t="inlineStr"/>
+      <c r="Q49" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R49" s="3" t="inlineStr">
         <is>
           <t>0-1</t>
         </is>
@@ -3176,18 +3284,20 @@
       <c r="J50" s="6" t="inlineStr"/>
       <c r="K50" s="6" t="inlineStr"/>
       <c r="L50" s="6" t="inlineStr"/>
-      <c r="M50" s="3" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
+      <c r="M50" s="3" t="inlineStr"/>
       <c r="N50" s="3" t="inlineStr"/>
       <c r="O50" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P50" s="3" t="inlineStr">
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="P50" s="3" t="inlineStr"/>
+      <c r="Q50" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R50" s="3" t="inlineStr">
         <is>
           <t>1-0</t>
         </is>
@@ -3230,18 +3340,20 @@
       <c r="J51" s="6" t="inlineStr"/>
       <c r="K51" s="6" t="inlineStr"/>
       <c r="L51" s="6" t="inlineStr"/>
-      <c r="M51" s="3" t="inlineStr">
-        <is>
-          <t>Bosnia and Herzegovina</t>
-        </is>
-      </c>
+      <c r="M51" s="3" t="inlineStr"/>
       <c r="N51" s="3" t="inlineStr"/>
       <c r="O51" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P51" s="3" t="inlineStr">
+          <t>Bosnia and Herzegovina</t>
+        </is>
+      </c>
+      <c r="P51" s="3" t="inlineStr"/>
+      <c r="Q51" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R51" s="3" t="inlineStr">
         <is>
           <t>3-1</t>
         </is>
@@ -3284,18 +3396,20 @@
       <c r="J52" s="6" t="inlineStr"/>
       <c r="K52" s="6" t="inlineStr"/>
       <c r="L52" s="6" t="inlineStr"/>
-      <c r="M52" s="3" t="inlineStr">
-        <is>
-          <t>Switzerland</t>
-        </is>
-      </c>
+      <c r="M52" s="3" t="inlineStr"/>
       <c r="N52" s="3" t="inlineStr"/>
       <c r="O52" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P52" s="3" t="inlineStr">
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="P52" s="3" t="inlineStr"/>
+      <c r="Q52" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R52" s="3" t="inlineStr">
         <is>
           <t>2-1</t>
         </is>
@@ -3338,18 +3452,20 @@
       <c r="J53" s="6" t="inlineStr"/>
       <c r="K53" s="6" t="inlineStr"/>
       <c r="L53" s="6" t="inlineStr"/>
-      <c r="M53" s="3" t="inlineStr">
-        <is>
-          <t>Morocco</t>
-        </is>
-      </c>
+      <c r="M53" s="3" t="inlineStr"/>
       <c r="N53" s="3" t="inlineStr"/>
       <c r="O53" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P53" s="3" t="inlineStr">
+          <t>Morocco</t>
+        </is>
+      </c>
+      <c r="P53" s="3" t="inlineStr"/>
+      <c r="Q53" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R53" s="3" t="inlineStr">
         <is>
           <t>4-2</t>
         </is>
@@ -3392,18 +3508,20 @@
       <c r="J54" s="6" t="inlineStr"/>
       <c r="K54" s="6" t="inlineStr"/>
       <c r="L54" s="6" t="inlineStr"/>
-      <c r="M54" s="3" t="inlineStr">
-        <is>
-          <t>Brazil</t>
-        </is>
-      </c>
+      <c r="M54" s="3" t="inlineStr"/>
       <c r="N54" s="3" t="inlineStr"/>
       <c r="O54" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P54" s="3" t="inlineStr">
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="P54" s="3" t="inlineStr"/>
+      <c r="Q54" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R54" s="3" t="inlineStr">
         <is>
           <t>0-3</t>
         </is>
@@ -3446,18 +3564,20 @@
       <c r="J55" s="6" t="inlineStr"/>
       <c r="K55" s="6" t="inlineStr"/>
       <c r="L55" s="6" t="inlineStr"/>
-      <c r="M55" s="3" t="inlineStr">
-        <is>
-          <t>Mexico</t>
-        </is>
-      </c>
+      <c r="M55" s="3" t="inlineStr"/>
       <c r="N55" s="3" t="inlineStr"/>
       <c r="O55" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P55" s="3" t="inlineStr">
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="P55" s="3" t="inlineStr"/>
+      <c r="Q55" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R55" s="3" t="inlineStr">
         <is>
           <t>0-3</t>
         </is>
@@ -3500,18 +3620,20 @@
       <c r="J56" s="6" t="inlineStr"/>
       <c r="K56" s="6" t="inlineStr"/>
       <c r="L56" s="6" t="inlineStr"/>
-      <c r="M56" s="3" t="inlineStr">
-        <is>
-          <t>South Korea</t>
-        </is>
-      </c>
+      <c r="M56" s="3" t="inlineStr"/>
       <c r="N56" s="3" t="inlineStr"/>
       <c r="O56" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P56" s="3" t="inlineStr">
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="P56" s="3" t="inlineStr"/>
+      <c r="Q56" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R56" s="3" t="inlineStr">
         <is>
           <t>1-0</t>
         </is>
@@ -3554,18 +3676,20 @@
       <c r="J57" s="6" t="inlineStr"/>
       <c r="K57" s="6" t="inlineStr"/>
       <c r="L57" s="6" t="inlineStr"/>
-      <c r="M57" s="3" t="inlineStr">
-        <is>
-          <t>Ivory Coast</t>
-        </is>
-      </c>
+      <c r="M57" s="3" t="inlineStr"/>
       <c r="N57" s="3" t="inlineStr"/>
       <c r="O57" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P57" s="3" t="inlineStr">
+          <t>Ivory Coast</t>
+        </is>
+      </c>
+      <c r="P57" s="3" t="inlineStr"/>
+      <c r="Q57" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R57" s="3" t="inlineStr">
         <is>
           <t>0-2</t>
         </is>
@@ -3608,18 +3732,20 @@
       <c r="J58" s="6" t="inlineStr"/>
       <c r="K58" s="6" t="inlineStr"/>
       <c r="L58" s="6" t="inlineStr"/>
-      <c r="M58" s="3" t="inlineStr">
-        <is>
-          <t>Germany</t>
-        </is>
-      </c>
+      <c r="M58" s="3" t="inlineStr"/>
       <c r="N58" s="3" t="inlineStr"/>
       <c r="O58" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P58" s="3" t="inlineStr">
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="P58" s="3" t="inlineStr"/>
+      <c r="Q58" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R58" s="3" t="inlineStr">
         <is>
           <t>2-1</t>
         </is>
@@ -3662,18 +3788,20 @@
       <c r="J59" s="6" t="inlineStr"/>
       <c r="K59" s="6" t="inlineStr"/>
       <c r="L59" s="6" t="inlineStr"/>
-      <c r="M59" s="3" t="inlineStr">
-        <is>
-          <t>Japan</t>
-        </is>
-      </c>
+      <c r="M59" s="3" t="inlineStr"/>
       <c r="N59" s="3" t="inlineStr"/>
       <c r="O59" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P59" s="3" t="inlineStr">
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="P59" s="3" t="inlineStr"/>
+      <c r="Q59" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R59" s="3" t="inlineStr">
         <is>
           <t>1-1</t>
         </is>
@@ -3716,18 +3844,20 @@
       <c r="J60" s="6" t="inlineStr"/>
       <c r="K60" s="6" t="inlineStr"/>
       <c r="L60" s="6" t="inlineStr"/>
-      <c r="M60" s="3" t="inlineStr">
-        <is>
-          <t>Netherlands</t>
-        </is>
-      </c>
+      <c r="M60" s="3" t="inlineStr"/>
       <c r="N60" s="3" t="inlineStr"/>
       <c r="O60" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P60" s="3" t="inlineStr">
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="P60" s="3" t="inlineStr"/>
+      <c r="Q60" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R60" s="3" t="inlineStr">
         <is>
           <t>1-3</t>
         </is>
@@ -3770,18 +3900,20 @@
       <c r="J61" s="6" t="inlineStr"/>
       <c r="K61" s="6" t="inlineStr"/>
       <c r="L61" s="6" t="inlineStr"/>
-      <c r="M61" s="3" t="inlineStr">
-        <is>
-          <t>Paraguay</t>
-        </is>
-      </c>
+      <c r="M61" s="3" t="inlineStr"/>
       <c r="N61" s="3" t="inlineStr"/>
       <c r="O61" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P61" s="3" t="inlineStr">
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="P61" s="3" t="inlineStr"/>
+      <c r="Q61" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R61" s="3" t="inlineStr">
         <is>
           <t>0-0</t>
         </is>
@@ -3824,18 +3956,20 @@
       <c r="J62" s="6" t="inlineStr"/>
       <c r="K62" s="6" t="inlineStr"/>
       <c r="L62" s="6" t="inlineStr"/>
-      <c r="M62" s="3" t="inlineStr">
-        <is>
-          <t>Turkey</t>
-        </is>
-      </c>
+      <c r="M62" s="3" t="inlineStr"/>
       <c r="N62" s="3" t="inlineStr"/>
       <c r="O62" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P62" s="3" t="inlineStr">
+          <t>Turkey</t>
+        </is>
+      </c>
+      <c r="P62" s="3" t="inlineStr"/>
+      <c r="Q62" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R62" s="3" t="inlineStr">
         <is>
           <t>3-2</t>
         </is>
@@ -3878,18 +4012,20 @@
       <c r="J63" s="6" t="inlineStr"/>
       <c r="K63" s="6" t="inlineStr"/>
       <c r="L63" s="6" t="inlineStr"/>
-      <c r="M63" s="3" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
+      <c r="M63" s="3" t="inlineStr"/>
       <c r="N63" s="3" t="inlineStr"/>
       <c r="O63" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P63" s="3" t="inlineStr">
+          <t>France</t>
+        </is>
+      </c>
+      <c r="P63" s="3" t="inlineStr"/>
+      <c r="Q63" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R63" s="3" t="inlineStr">
         <is>
           <t>1-4</t>
         </is>
@@ -3932,18 +4068,20 @@
       <c r="J64" s="6" t="inlineStr"/>
       <c r="K64" s="6" t="inlineStr"/>
       <c r="L64" s="6" t="inlineStr"/>
-      <c r="M64" s="3" t="inlineStr">
-        <is>
-          <t>Senegal</t>
-        </is>
-      </c>
+      <c r="M64" s="3" t="inlineStr"/>
       <c r="N64" s="3" t="inlineStr"/>
       <c r="O64" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P64" s="3" t="inlineStr">
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="P64" s="3" t="inlineStr"/>
+      <c r="Q64" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R64" s="3" t="inlineStr">
         <is>
           <t>5-0</t>
         </is>
@@ -3986,18 +4124,20 @@
       <c r="J65" s="6" t="inlineStr"/>
       <c r="K65" s="6" t="inlineStr"/>
       <c r="L65" s="6" t="inlineStr"/>
-      <c r="M65" s="3" t="inlineStr">
-        <is>
-          <t>Draw</t>
-        </is>
-      </c>
+      <c r="M65" s="3" t="inlineStr"/>
       <c r="N65" s="3" t="inlineStr"/>
       <c r="O65" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P65" s="3" t="inlineStr">
+          <t>Draw</t>
+        </is>
+      </c>
+      <c r="P65" s="3" t="inlineStr"/>
+      <c r="Q65" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R65" s="3" t="inlineStr">
         <is>
           <t>0-0</t>
         </is>
@@ -4040,18 +4180,20 @@
       <c r="J66" s="6" t="inlineStr"/>
       <c r="K66" s="6" t="inlineStr"/>
       <c r="L66" s="6" t="inlineStr"/>
-      <c r="M66" s="3" t="inlineStr">
-        <is>
-          <t>Spain</t>
-        </is>
-      </c>
+      <c r="M66" s="3" t="inlineStr"/>
       <c r="N66" s="3" t="inlineStr"/>
       <c r="O66" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P66" s="3" t="inlineStr">
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="P66" s="3" t="inlineStr"/>
+      <c r="Q66" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R66" s="3" t="inlineStr">
         <is>
           <t>0-1</t>
         </is>
@@ -4094,18 +4236,20 @@
       <c r="J67" s="6" t="inlineStr"/>
       <c r="K67" s="6" t="inlineStr"/>
       <c r="L67" s="6" t="inlineStr"/>
-      <c r="M67" s="3" t="inlineStr">
-        <is>
-          <t>Draw</t>
-        </is>
-      </c>
+      <c r="M67" s="3" t="inlineStr"/>
       <c r="N67" s="3" t="inlineStr"/>
       <c r="O67" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P67" s="3" t="inlineStr">
+          <t>Draw</t>
+        </is>
+      </c>
+      <c r="P67" s="3" t="inlineStr"/>
+      <c r="Q67" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R67" s="3" t="inlineStr">
         <is>
           <t>1-1</t>
         </is>
@@ -4148,18 +4292,20 @@
       <c r="J68" s="6" t="inlineStr"/>
       <c r="K68" s="6" t="inlineStr"/>
       <c r="L68" s="6" t="inlineStr"/>
-      <c r="M68" s="3" t="inlineStr">
-        <is>
-          <t>Belgium</t>
-        </is>
-      </c>
+      <c r="M68" s="3" t="inlineStr"/>
       <c r="N68" s="3" t="inlineStr"/>
       <c r="O68" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P68" s="3" t="inlineStr">
+          <t>Belgium</t>
+        </is>
+      </c>
+      <c r="P68" s="3" t="inlineStr"/>
+      <c r="Q68" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R68" s="3" t="inlineStr">
         <is>
           <t>1-5</t>
         </is>
@@ -4202,18 +4348,20 @@
       <c r="J69" s="6" t="inlineStr"/>
       <c r="K69" s="6" t="inlineStr"/>
       <c r="L69" s="6" t="inlineStr"/>
-      <c r="M69" s="3" t="inlineStr">
-        <is>
-          <t>Croatia</t>
-        </is>
-      </c>
+      <c r="M69" s="3" t="inlineStr"/>
       <c r="N69" s="3" t="inlineStr"/>
       <c r="O69" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P69" s="3" t="inlineStr">
+          <t>Croatia</t>
+        </is>
+      </c>
+      <c r="P69" s="3" t="inlineStr"/>
+      <c r="Q69" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R69" s="3" t="inlineStr">
         <is>
           <t>2-1</t>
         </is>
@@ -4256,18 +4404,20 @@
       <c r="J70" s="6" t="inlineStr"/>
       <c r="K70" s="6" t="inlineStr"/>
       <c r="L70" s="6" t="inlineStr"/>
-      <c r="M70" s="3" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
+      <c r="M70" s="3" t="inlineStr"/>
       <c r="N70" s="3" t="inlineStr"/>
       <c r="O70" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P70" s="3" t="inlineStr">
+          <t>England</t>
+        </is>
+      </c>
+      <c r="P70" s="3" t="inlineStr"/>
+      <c r="Q70" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R70" s="3" t="inlineStr">
         <is>
           <t>0-2</t>
         </is>
@@ -4310,18 +4460,20 @@
       <c r="J71" s="6" t="inlineStr"/>
       <c r="K71" s="6" t="inlineStr"/>
       <c r="L71" s="6" t="inlineStr"/>
-      <c r="M71" s="3" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
+      <c r="M71" s="3" t="inlineStr"/>
       <c r="N71" s="3" t="inlineStr"/>
       <c r="O71" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P71" s="3" t="inlineStr">
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="P71" s="3" t="inlineStr"/>
+      <c r="Q71" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R71" s="3" t="inlineStr">
         <is>
           <t>0-0</t>
         </is>
@@ -4364,18 +4516,20 @@
       <c r="J72" s="6" t="inlineStr"/>
       <c r="K72" s="6" t="inlineStr"/>
       <c r="L72" s="6" t="inlineStr"/>
-      <c r="M72" s="3" t="inlineStr">
-        <is>
-          <t>DR Congo</t>
-        </is>
-      </c>
+      <c r="M72" s="3" t="inlineStr"/>
       <c r="N72" s="3" t="inlineStr"/>
       <c r="O72" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P72" s="3" t="inlineStr">
+          <t>DR Congo</t>
+        </is>
+      </c>
+      <c r="P72" s="3" t="inlineStr"/>
+      <c r="Q72" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R72" s="3" t="inlineStr">
         <is>
           <t>3-1</t>
         </is>
@@ -4418,18 +4572,20 @@
       <c r="J73" s="6" t="inlineStr"/>
       <c r="K73" s="6" t="inlineStr"/>
       <c r="L73" s="6" t="inlineStr"/>
-      <c r="M73" s="3" t="inlineStr">
-        <is>
-          <t>Draw</t>
-        </is>
-      </c>
+      <c r="M73" s="3" t="inlineStr"/>
       <c r="N73" s="3" t="inlineStr"/>
       <c r="O73" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P73" s="3" t="inlineStr">
+          <t>Draw</t>
+        </is>
+      </c>
+      <c r="P73" s="3" t="inlineStr"/>
+      <c r="Q73" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R73" s="3" t="inlineStr">
         <is>
           <t>3-3</t>
         </is>
@@ -4472,18 +4628,20 @@
       <c r="J74" s="6" t="inlineStr"/>
       <c r="K74" s="6" t="inlineStr"/>
       <c r="L74" s="6" t="inlineStr"/>
-      <c r="M74" s="3" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
+      <c r="M74" s="3" t="inlineStr"/>
       <c r="N74" s="3" t="inlineStr"/>
       <c r="O74" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P74" s="3" t="inlineStr">
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="P74" s="3" t="inlineStr"/>
+      <c r="Q74" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R74" s="3" t="inlineStr">
         <is>
           <t>1-3</t>
         </is>
@@ -4522,18 +4680,20 @@
       <c r="J75" s="6" t="inlineStr"/>
       <c r="K75" s="6" t="inlineStr"/>
       <c r="L75" s="6" t="inlineStr"/>
-      <c r="M75" s="3" t="inlineStr">
-        <is>
-          <t>Canada</t>
-        </is>
-      </c>
+      <c r="M75" s="3" t="inlineStr"/>
       <c r="N75" s="3" t="inlineStr"/>
       <c r="O75" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P75" s="3" t="inlineStr">
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="P75" s="3" t="inlineStr"/>
+      <c r="Q75" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R75" s="3" t="inlineStr">
         <is>
           <t>0-1</t>
         </is>
@@ -4572,18 +4732,20 @@
       <c r="J76" s="6" t="inlineStr"/>
       <c r="K76" s="6" t="inlineStr"/>
       <c r="L76" s="6" t="inlineStr"/>
-      <c r="M76" s="3" t="inlineStr">
-        <is>
-          <t>Brazil</t>
-        </is>
-      </c>
+      <c r="M76" s="3" t="inlineStr"/>
       <c r="N76" s="3" t="inlineStr"/>
       <c r="O76" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P76" s="3" t="inlineStr">
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="P76" s="3" t="inlineStr"/>
+      <c r="Q76" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R76" s="3" t="inlineStr">
         <is>
           <t>2-1</t>
         </is>
@@ -4622,18 +4784,20 @@
       <c r="J77" s="6" t="inlineStr"/>
       <c r="K77" s="6" t="inlineStr"/>
       <c r="L77" s="6" t="inlineStr"/>
-      <c r="M77" s="3" t="inlineStr">
-        <is>
-          <t>Germany</t>
-        </is>
-      </c>
+      <c r="M77" s="3" t="inlineStr"/>
       <c r="N77" s="3" t="inlineStr"/>
       <c r="O77" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P77" s="3" t="inlineStr">
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="P77" s="3" t="inlineStr"/>
+      <c r="Q77" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R77" s="3" t="inlineStr">
         <is>
           <t>1-1</t>
         </is>
@@ -4672,18 +4836,20 @@
       <c r="J78" s="6" t="inlineStr"/>
       <c r="K78" s="6" t="inlineStr"/>
       <c r="L78" s="6" t="inlineStr"/>
-      <c r="M78" s="3" t="inlineStr">
-        <is>
-          <t>Netherlands</t>
-        </is>
-      </c>
+      <c r="M78" s="3" t="inlineStr"/>
       <c r="N78" s="3" t="inlineStr"/>
       <c r="O78" s="3" t="inlineStr">
         <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P78" s="3" t="inlineStr">
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="P78" s="3" t="inlineStr"/>
+      <c r="Q78" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R78" s="3" t="inlineStr">
         <is>
           <t>1-1</t>
         </is>
@@ -4719,31 +4885,41 @@
       </c>
       <c r="H79" s="3" t="inlineStr">
         <is>
-          <t>1-2</t>
-        </is>
-      </c>
-      <c r="I79" s="3" t="inlineStr"/>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="I79" s="3" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
       <c r="J79" s="6" t="n">
-        <v>0.2593967154053816</v>
+        <v>0.2395221762283596</v>
       </c>
       <c r="K79" s="6" t="n">
-        <v>0.2409137615394984</v>
+        <v>0.2507856341556973</v>
       </c>
       <c r="L79" s="6" t="n">
-        <v>0.4996895230551199</v>
-      </c>
-      <c r="M79" s="3" t="inlineStr">
+        <v>0.5096921896159431</v>
+      </c>
+      <c r="M79" s="3" t="n">
+        <v>0.95431834</v>
+      </c>
+      <c r="N79" s="3" t="n">
+        <v>1.4211165</v>
+      </c>
+      <c r="O79" s="3" t="inlineStr">
         <is>
           <t>Norway</t>
         </is>
       </c>
-      <c r="N79" s="3" t="inlineStr"/>
-      <c r="O79" s="3" t="inlineStr">
-        <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
       <c r="P79" s="3" t="inlineStr"/>
+      <c r="Q79" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R79" s="3" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="3" t="n">
@@ -4780,26 +4956,32 @@
       </c>
       <c r="I80" s="3" t="inlineStr"/>
       <c r="J80" s="6" t="n">
-        <v>0.7618028528427053</v>
+        <v>0.7403545998732053</v>
       </c>
       <c r="K80" s="6" t="n">
-        <v>0.1367267415503548</v>
+        <v>0.1463523031009907</v>
       </c>
       <c r="L80" s="6" t="n">
-        <v>0.1014704056069399</v>
-      </c>
-      <c r="M80" s="3" t="inlineStr">
+        <v>0.113293097025804</v>
+      </c>
+      <c r="M80" s="3" t="n">
+        <v>2.2604704</v>
+      </c>
+      <c r="N80" s="3" t="n">
+        <v>0.6237355999999999</v>
+      </c>
+      <c r="O80" s="3" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="N80" s="3" t="inlineStr"/>
-      <c r="O80" s="3" t="inlineStr">
-        <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
       <c r="P80" s="3" t="inlineStr"/>
+      <c r="Q80" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R80" s="3" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="3" t="n">
@@ -4836,30 +5018,36 @@
       </c>
       <c r="I81" s="3" t="inlineStr"/>
       <c r="J81" s="6" t="n">
-        <v>0.3374151661390585</v>
+        <v>0.3339299329194478</v>
       </c>
       <c r="K81" s="6" t="n">
-        <v>0.3386565480414149</v>
+        <v>0.3486974454470022</v>
       </c>
       <c r="L81" s="6" t="n">
-        <v>0.3239282858195267</v>
-      </c>
-      <c r="M81" s="3" t="inlineStr">
+        <v>0.3173726216335499</v>
+      </c>
+      <c r="M81" s="3" t="n">
+        <v>1.237195</v>
+      </c>
+      <c r="N81" s="3" t="n">
+        <v>1.0279981</v>
+      </c>
+      <c r="O81" s="3" t="inlineStr">
         <is>
           <t>Draw</t>
         </is>
       </c>
-      <c r="N81" s="3" t="inlineStr">
+      <c r="P81" s="3" t="inlineStr">
         <is>
           <t>Mexico</t>
         </is>
       </c>
-      <c r="O81" s="3" t="inlineStr">
-        <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P81" s="3" t="inlineStr"/>
+      <c r="Q81" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R81" s="3" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="3" t="n">
@@ -4896,26 +5084,32 @@
       </c>
       <c r="I82" s="3" t="inlineStr"/>
       <c r="J82" s="6" t="n">
-        <v>0.7454126266494137</v>
+        <v>0.7538609557229126</v>
       </c>
       <c r="K82" s="6" t="n">
-        <v>0.1807887595121333</v>
+        <v>0.1734156820091866</v>
       </c>
       <c r="L82" s="6" t="n">
-        <v>0.073798613838453</v>
-      </c>
-      <c r="M82" s="3" t="inlineStr">
+        <v>0.07272336226790092</v>
+      </c>
+      <c r="M82" s="3" t="n">
+        <v>2.0189307</v>
+      </c>
+      <c r="N82" s="3" t="n">
+        <v>0.6254953</v>
+      </c>
+      <c r="O82" s="3" t="inlineStr">
         <is>
           <t>England</t>
         </is>
       </c>
-      <c r="N82" s="3" t="inlineStr"/>
-      <c r="O82" s="3" t="inlineStr">
-        <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
       <c r="P82" s="3" t="inlineStr"/>
+      <c r="Q82" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R82" s="3" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="3" t="n">
@@ -4952,26 +5146,32 @@
       </c>
       <c r="I83" s="3" t="inlineStr"/>
       <c r="J83" s="6" t="n">
-        <v>0.5208908705084515</v>
+        <v>0.5156179691882963</v>
       </c>
       <c r="K83" s="6" t="n">
-        <v>0.2510906889620449</v>
+        <v>0.2705727658083974</v>
       </c>
       <c r="L83" s="6" t="n">
-        <v>0.2280184405295036</v>
-      </c>
-      <c r="M83" s="3" t="inlineStr">
+        <v>0.2138092650033063</v>
+      </c>
+      <c r="M83" s="3" t="n">
+        <v>1.6579897</v>
+      </c>
+      <c r="N83" s="3" t="n">
+        <v>1.0114748</v>
+      </c>
+      <c r="O83" s="3" t="inlineStr">
         <is>
           <t>Belgium</t>
         </is>
       </c>
-      <c r="N83" s="3" t="inlineStr"/>
-      <c r="O83" s="3" t="inlineStr">
-        <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
       <c r="P83" s="3" t="inlineStr"/>
+      <c r="Q83" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R83" s="3" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="3" t="n">
@@ -5003,31 +5203,41 @@
       </c>
       <c r="H84" s="3" t="inlineStr">
         <is>
-          <t>1-0</t>
-        </is>
-      </c>
-      <c r="I84" s="3" t="inlineStr"/>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="I84" s="3" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
       <c r="J84" s="6" t="n">
-        <v>0.6262432418337703</v>
+        <v>0.6347002622796442</v>
       </c>
       <c r="K84" s="6" t="n">
-        <v>0.2148057194698543</v>
+        <v>0.2010998563708226</v>
       </c>
       <c r="L84" s="6" t="n">
-        <v>0.1589510386963754</v>
-      </c>
-      <c r="M84" s="3" t="inlineStr">
+        <v>0.1641998813495332</v>
+      </c>
+      <c r="M84" s="3" t="n">
+        <v>1.655824</v>
+      </c>
+      <c r="N84" s="3" t="n">
+        <v>0.80044484</v>
+      </c>
+      <c r="O84" s="3" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="N84" s="3" t="inlineStr"/>
-      <c r="O84" s="3" t="inlineStr">
-        <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
       <c r="P84" s="3" t="inlineStr"/>
+      <c r="Q84" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R84" s="3" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="3" t="n">
@@ -5064,26 +5274,32 @@
       </c>
       <c r="I85" s="3" t="inlineStr"/>
       <c r="J85" s="6" t="n">
-        <v>0.6613598361949842</v>
+        <v>0.6422269916189836</v>
       </c>
       <c r="K85" s="6" t="n">
-        <v>0.1938613353415957</v>
+        <v>0.2073484195192632</v>
       </c>
       <c r="L85" s="6" t="n">
-        <v>0.1447788284634201</v>
-      </c>
-      <c r="M85" s="3" t="inlineStr">
+        <v>0.1504245888617533</v>
+      </c>
+      <c r="M85" s="3" t="n">
+        <v>1.9921775</v>
+      </c>
+      <c r="N85" s="3" t="n">
+        <v>0.73966795</v>
+      </c>
+      <c r="O85" s="3" t="inlineStr">
         <is>
           <t>Spain</t>
         </is>
       </c>
-      <c r="N85" s="3" t="inlineStr"/>
-      <c r="O85" s="3" t="inlineStr">
-        <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
       <c r="P85" s="3" t="inlineStr"/>
+      <c r="Q85" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R85" s="3" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="3" t="n">
@@ -5124,26 +5340,32 @@
         </is>
       </c>
       <c r="J86" s="6" t="n">
-        <v>0.45722519151763</v>
+        <v>0.4474320504796094</v>
       </c>
       <c r="K86" s="6" t="n">
-        <v>0.3107820790401717</v>
+        <v>0.3179839516475488</v>
       </c>
       <c r="L86" s="6" t="n">
-        <v>0.2319927294421983</v>
-      </c>
-      <c r="M86" s="3" t="inlineStr">
+        <v>0.2345839978728418</v>
+      </c>
+      <c r="M86" s="3" t="n">
+        <v>1.564798</v>
+      </c>
+      <c r="N86" s="3" t="n">
+        <v>1.0314984</v>
+      </c>
+      <c r="O86" s="3" t="inlineStr">
         <is>
           <t>Portugal</t>
         </is>
       </c>
-      <c r="N86" s="3" t="inlineStr"/>
-      <c r="O86" s="3" t="inlineStr">
-        <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
       <c r="P86" s="3" t="inlineStr"/>
+      <c r="Q86" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R86" s="3" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="3" t="n">
@@ -5180,26 +5402,32 @@
       </c>
       <c r="I87" s="3" t="inlineStr"/>
       <c r="J87" s="6" t="n">
-        <v>0.5038607556724858</v>
+        <v>0.5006338299381323</v>
       </c>
       <c r="K87" s="6" t="n">
-        <v>0.2618429167603477</v>
+        <v>0.2741811495090014</v>
       </c>
       <c r="L87" s="6" t="n">
-        <v>0.2342963275671667</v>
-      </c>
-      <c r="M87" s="3" t="inlineStr">
+        <v>0.2251850205528662</v>
+      </c>
+      <c r="M87" s="3" t="n">
+        <v>1.6694916</v>
+      </c>
+      <c r="N87" s="3" t="n">
+        <v>1.0056431</v>
+      </c>
+      <c r="O87" s="3" t="inlineStr">
         <is>
           <t>Switzerland</t>
         </is>
       </c>
-      <c r="N87" s="3" t="inlineStr"/>
-      <c r="O87" s="3" t="inlineStr">
-        <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
       <c r="P87" s="3" t="inlineStr"/>
+      <c r="Q87" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R87" s="3" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="3" t="n">
@@ -5236,30 +5464,36 @@
       </c>
       <c r="I88" s="3" t="inlineStr"/>
       <c r="J88" s="6" t="n">
-        <v>0.3769989957865302</v>
+        <v>0.3737968374754114</v>
       </c>
       <c r="K88" s="6" t="n">
-        <v>0.3472613362034865</v>
+        <v>0.3559628001066526</v>
       </c>
       <c r="L88" s="6" t="n">
-        <v>0.2757396680099833</v>
-      </c>
-      <c r="M88" s="3" t="inlineStr">
+        <v>0.270240362417936</v>
+      </c>
+      <c r="M88" s="3" t="n">
+        <v>1.361172</v>
+      </c>
+      <c r="N88" s="3" t="n">
+        <v>1.0059781</v>
+      </c>
+      <c r="O88" s="3" t="inlineStr">
         <is>
           <t>Draw</t>
         </is>
       </c>
-      <c r="N88" s="3" t="inlineStr">
+      <c r="P88" s="3" t="inlineStr">
         <is>
           <t>Australia</t>
         </is>
       </c>
-      <c r="O88" s="3" t="inlineStr">
-        <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
-      <c r="P88" s="3" t="inlineStr"/>
+      <c r="Q88" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R88" s="3" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="3" t="n">
@@ -5296,26 +5530,32 @@
       </c>
       <c r="I89" s="3" t="inlineStr"/>
       <c r="J89" s="6" t="n">
-        <v>0.8689324622694531</v>
+        <v>0.8676248172327331</v>
       </c>
       <c r="K89" s="6" t="n">
-        <v>0.1029321098153271</v>
+        <v>0.1052467273557611</v>
       </c>
       <c r="L89" s="6" t="n">
-        <v>0.0281354279152198</v>
-      </c>
-      <c r="M89" s="3" t="inlineStr">
+        <v>0.0271284554115058</v>
+      </c>
+      <c r="M89" s="3" t="n">
+        <v>2.6222327</v>
+      </c>
+      <c r="N89" s="3" t="n">
+        <v>0.47000164</v>
+      </c>
+      <c r="O89" s="3" t="inlineStr">
         <is>
           <t>Argentina</t>
         </is>
       </c>
-      <c r="N89" s="3" t="inlineStr"/>
-      <c r="O89" s="3" t="inlineStr">
-        <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
       <c r="P89" s="3" t="inlineStr"/>
+      <c r="Q89" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R89" s="3" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="3" t="n">
@@ -5347,35 +5587,37 @@
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
-          <t>2-1</t>
-        </is>
-      </c>
-      <c r="I90" s="3" t="inlineStr">
-        <is>
-          <t>2-1</t>
-        </is>
-      </c>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="I90" s="3" t="inlineStr"/>
       <c r="J90" s="6" t="n">
-        <v>0.7902869818560336</v>
+        <v>0.7751377191591644</v>
       </c>
       <c r="K90" s="6" t="n">
-        <v>0.1500108535962172</v>
+        <v>0.1625831142098152</v>
       </c>
       <c r="L90" s="6" t="n">
-        <v>0.05970216454774921</v>
-      </c>
-      <c r="M90" s="3" t="inlineStr">
+        <v>0.0622791666310204</v>
+      </c>
+      <c r="M90" s="3" t="n">
+        <v>2.4145937</v>
+      </c>
+      <c r="N90" s="3" t="n">
+        <v>0.5740192</v>
+      </c>
+      <c r="O90" s="3" t="inlineStr">
         <is>
           <t>Colombia</t>
         </is>
       </c>
-      <c r="N90" s="3" t="inlineStr"/>
-      <c r="O90" s="3" t="inlineStr">
-        <is>
-          <t>Vastgezet</t>
-        </is>
-      </c>
       <c r="P90" s="3" t="inlineStr"/>
+      <c r="Q90" s="3" t="inlineStr">
+        <is>
+          <t>Vastgezet</t>
+        </is>
+      </c>
+      <c r="R90" s="3" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="3" t="n">
@@ -5412,30 +5654,36 @@
       </c>
       <c r="I91" s="3" t="inlineStr"/>
       <c r="J91" s="6" t="n">
-        <v>0.2017571205557528</v>
+        <v>0.200556911770865</v>
       </c>
       <c r="K91" s="6" t="n">
-        <v>0.378715077605386</v>
+        <v>0.3897062130509938</v>
       </c>
       <c r="L91" s="6" t="n">
-        <v>0.4195278018388612</v>
-      </c>
-      <c r="M91" s="3" t="inlineStr">
+        <v>0.409736875178141</v>
+      </c>
+      <c r="M91" s="3" t="n">
+        <v>0.9239122</v>
+      </c>
+      <c r="N91" s="3" t="n">
+        <v>1.4140741</v>
+      </c>
+      <c r="O91" s="3" t="inlineStr">
         <is>
           <t>Draw</t>
         </is>
       </c>
-      <c r="N91" s="3" t="inlineStr">
+      <c r="P91" s="3" t="inlineStr">
         <is>
           <t>Morocco</t>
         </is>
       </c>
-      <c r="O91" s="3" t="inlineStr">
+      <c r="Q91" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="P91" s="3" t="inlineStr"/>
+      <c r="R91" s="3" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="3" t="n">
@@ -5452,7 +5700,7 @@
       <c r="D92" s="3" t="inlineStr"/>
       <c r="E92" s="3" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Paraguay</t>
         </is>
       </c>
       <c r="F92" s="3" t="inlineStr">
@@ -5480,18 +5728,24 @@
       <c r="L92" s="6" t="n">
         <v>0.344</v>
       </c>
-      <c r="M92" s="3" t="inlineStr">
-        <is>
-          <t>Brazil</t>
-        </is>
-      </c>
-      <c r="N92" s="3" t="inlineStr"/>
+      <c r="M92" s="3" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="N92" s="3" t="n">
+        <v>1.02</v>
+      </c>
       <c r="O92" s="3" t="inlineStr">
         <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="P92" s="3" t="inlineStr"/>
+      <c r="Q92" s="3" t="inlineStr">
+        <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="P92" s="3" t="inlineStr"/>
+      <c r="R92" s="3" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="3" t="n">
@@ -5508,7 +5762,7 @@
       <c r="D93" s="3" t="inlineStr"/>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="F93" s="3" t="inlineStr">
@@ -5518,36 +5772,42 @@
       </c>
       <c r="G93" s="5" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>0-2</t>
         </is>
       </c>
       <c r="H93" s="3" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>0-2</t>
         </is>
       </c>
       <c r="I93" s="3" t="inlineStr"/>
       <c r="J93" s="6" t="n">
-        <v>0.3129999999999999</v>
+        <v>0.175</v>
       </c>
       <c r="K93" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L93" s="6" t="n">
-        <v>0.6870000000000001</v>
-      </c>
-      <c r="M93" s="3" t="inlineStr">
+        <v>0.825</v>
+      </c>
+      <c r="M93" s="3" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="N93" s="3" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="O93" s="3" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="N93" s="3" t="inlineStr"/>
-      <c r="O93" s="3" t="inlineStr">
+      <c r="P93" s="3" t="inlineStr"/>
+      <c r="Q93" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="P93" s="3" t="inlineStr"/>
+      <c r="R93" s="3" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="3" t="n">
@@ -5592,18 +5852,24 @@
       <c r="L94" s="6" t="n">
         <v>0.551</v>
       </c>
-      <c r="M94" s="3" t="inlineStr">
+      <c r="M94" s="3" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="N94" s="3" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="O94" s="3" t="inlineStr">
         <is>
           <t>England</t>
         </is>
       </c>
-      <c r="N94" s="3" t="inlineStr"/>
-      <c r="O94" s="3" t="inlineStr">
+      <c r="P94" s="3" t="inlineStr"/>
+      <c r="Q94" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="P94" s="3" t="inlineStr"/>
+      <c r="R94" s="3" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="3" t="n">
@@ -5648,18 +5914,24 @@
       <c r="L95" s="6" t="n">
         <v>0.28</v>
       </c>
-      <c r="M95" s="3" t="inlineStr">
+      <c r="M95" s="3" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="N95" s="3" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="O95" s="3" t="inlineStr">
         <is>
           <t>Spain</t>
         </is>
       </c>
-      <c r="N95" s="3" t="inlineStr"/>
-      <c r="O95" s="3" t="inlineStr">
+      <c r="P95" s="3" t="inlineStr"/>
+      <c r="Q95" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="P95" s="3" t="inlineStr"/>
+      <c r="R95" s="3" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="3" t="n">
@@ -5704,18 +5976,24 @@
       <c r="L96" s="6" t="n">
         <v>0.423</v>
       </c>
-      <c r="M96" s="3" t="inlineStr">
+      <c r="M96" s="3" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="N96" s="3" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="O96" s="3" t="inlineStr">
         <is>
           <t>Belgium</t>
         </is>
       </c>
-      <c r="N96" s="3" t="inlineStr"/>
-      <c r="O96" s="3" t="inlineStr">
+      <c r="P96" s="3" t="inlineStr"/>
+      <c r="Q96" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="P96" s="3" t="inlineStr"/>
+      <c r="R96" s="3" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="3" t="n">
@@ -5760,18 +6038,24 @@
       <c r="L97" s="6" t="n">
         <v>0.773</v>
       </c>
-      <c r="M97" s="3" t="inlineStr">
+      <c r="M97" s="3" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="N97" s="3" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="O97" s="3" t="inlineStr">
         <is>
           <t>Colombia</t>
         </is>
       </c>
-      <c r="N97" s="3" t="inlineStr"/>
-      <c r="O97" s="3" t="inlineStr">
+      <c r="P97" s="3" t="inlineStr"/>
+      <c r="Q97" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="P97" s="3" t="inlineStr"/>
+      <c r="R97" s="3" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="3" t="n">
@@ -5816,18 +6100,24 @@
       <c r="L98" s="6" t="n">
         <v>0.783</v>
       </c>
-      <c r="M98" s="3" t="inlineStr">
+      <c r="M98" s="3" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="N98" s="3" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="O98" s="3" t="inlineStr">
         <is>
           <t>Argentina</t>
         </is>
       </c>
-      <c r="N98" s="3" t="inlineStr"/>
-      <c r="O98" s="3" t="inlineStr">
+      <c r="P98" s="3" t="inlineStr"/>
+      <c r="Q98" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="P98" s="3" t="inlineStr"/>
+      <c r="R98" s="3" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="3" t="n">
@@ -5849,7 +6139,7 @@
       </c>
       <c r="F99" s="3" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Paraguay</t>
         </is>
       </c>
       <c r="G99" s="5" t="inlineStr">
@@ -5872,18 +6162,24 @@
       <c r="L99" s="6" t="n">
         <v>0.703</v>
       </c>
-      <c r="M99" s="3" t="inlineStr">
-        <is>
-          <t>Brazil</t>
-        </is>
-      </c>
-      <c r="N99" s="3" t="inlineStr"/>
+      <c r="M99" s="3" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="N99" s="3" t="n">
+        <v>1.7</v>
+      </c>
       <c r="O99" s="3" t="inlineStr">
         <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="P99" s="3" t="inlineStr"/>
+      <c r="Q99" s="3" t="inlineStr">
+        <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="P99" s="3" t="inlineStr"/>
+      <c r="R99" s="3" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="3" t="n">
@@ -5928,18 +6224,24 @@
       <c r="L100" s="6" t="n">
         <v>0.181</v>
       </c>
-      <c r="M100" s="3" t="inlineStr">
+      <c r="M100" s="3" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="N100" s="3" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="O100" s="3" t="inlineStr">
         <is>
           <t>Spain</t>
         </is>
       </c>
-      <c r="N100" s="3" t="inlineStr"/>
-      <c r="O100" s="3" t="inlineStr">
+      <c r="P100" s="3" t="inlineStr"/>
+      <c r="Q100" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="P100" s="3" t="inlineStr"/>
+      <c r="R100" s="3" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="3" t="n">
@@ -5984,18 +6286,24 @@
       <c r="L101" s="6" t="n">
         <v>0.347</v>
       </c>
-      <c r="M101" s="3" t="inlineStr">
+      <c r="M101" s="3" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="N101" s="3" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="O101" s="3" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="N101" s="3" t="inlineStr"/>
-      <c r="O101" s="3" t="inlineStr">
+      <c r="P101" s="3" t="inlineStr"/>
+      <c r="Q101" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="P101" s="3" t="inlineStr"/>
+      <c r="R101" s="3" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="3" t="n">
@@ -6040,18 +6348,24 @@
       <c r="L102" s="6" t="n">
         <v>0.724</v>
       </c>
-      <c r="M102" s="3" t="inlineStr">
+      <c r="M102" s="3" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="N102" s="3" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="O102" s="3" t="inlineStr">
         <is>
           <t>Argentina</t>
         </is>
       </c>
-      <c r="N102" s="3" t="inlineStr"/>
-      <c r="O102" s="3" t="inlineStr">
+      <c r="P102" s="3" t="inlineStr"/>
+      <c r="Q102" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="P102" s="3" t="inlineStr"/>
+      <c r="R102" s="3" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="3" t="n">
@@ -6068,7 +6382,7 @@
       <c r="D103" s="3" t="inlineStr"/>
       <c r="E103" s="3" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Paraguay</t>
         </is>
       </c>
       <c r="F103" s="3" t="inlineStr">
@@ -6096,18 +6410,24 @@
       <c r="L103" s="6" t="n">
         <v>0.676</v>
       </c>
-      <c r="M103" s="3" t="inlineStr">
+      <c r="M103" s="3" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="N103" s="3" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="O103" s="3" t="inlineStr">
         <is>
           <t>Spain</t>
         </is>
       </c>
-      <c r="N103" s="3" t="inlineStr"/>
-      <c r="O103" s="3" t="inlineStr">
+      <c r="P103" s="3" t="inlineStr"/>
+      <c r="Q103" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="P103" s="3" t="inlineStr"/>
+      <c r="R103" s="3" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="3" t="n">
@@ -6152,18 +6472,24 @@
       <c r="L104" s="6" t="n">
         <v>0.521</v>
       </c>
-      <c r="M104" s="3" t="inlineStr">
+      <c r="M104" s="3" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="N104" s="3" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="O104" s="3" t="inlineStr">
         <is>
           <t>Argentina</t>
         </is>
       </c>
-      <c r="N104" s="3" t="inlineStr"/>
-      <c r="O104" s="3" t="inlineStr">
+      <c r="P104" s="3" t="inlineStr"/>
+      <c r="Q104" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="P104" s="3" t="inlineStr"/>
+      <c r="R104" s="3" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="3" t="n">
@@ -6180,7 +6506,7 @@
       <c r="D105" s="3" t="inlineStr"/>
       <c r="E105" s="3" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Paraguay</t>
         </is>
       </c>
       <c r="F105" s="3" t="inlineStr">
@@ -6208,18 +6534,24 @@
       <c r="L105" s="6" t="n">
         <v>0.665</v>
       </c>
-      <c r="M105" s="3" t="inlineStr">
+      <c r="M105" s="3" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="N105" s="3" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="O105" s="3" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="N105" s="3" t="inlineStr"/>
-      <c r="O105" s="3" t="inlineStr">
+      <c r="P105" s="3" t="inlineStr"/>
+      <c r="Q105" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="P105" s="3" t="inlineStr"/>
+      <c r="R105" s="3" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="3" t="n">
@@ -6264,22 +6596,28 @@
       <c r="L106" s="6" t="n">
         <v>0.509</v>
       </c>
-      <c r="M106" s="3" t="inlineStr">
+      <c r="M106" s="3" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="N106" s="3" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="O106" s="3" t="inlineStr">
         <is>
           <t>Argentina</t>
         </is>
       </c>
-      <c r="N106" s="3" t="inlineStr"/>
-      <c r="O106" s="3" t="inlineStr">
+      <c r="P106" s="3" t="inlineStr"/>
+      <c r="Q106" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="P106" s="3" t="inlineStr"/>
+      <c r="R106" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A1:R1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>